<commit_message>
Fix: Finish Excel Chapter 4
</commit_message>
<xml_diff>
--- a/Build/Signal_Lost_Chapters.xlsx
+++ b/Build/Signal_Lost_Chapters.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\k_furno\Documents\Projects\Visual Studio 2026\C++\Signal-Lost\Build\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Developpement\Games\Visual Studio 2026\C++\Signal_Lost\Signal_Lost\Build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{416C37EB-FAEC-4640-82F6-FC6EFC937F9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B33A72C-385C-4833-910B-A7E2ADD0D100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="528" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" tabRatio="528" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chapters_Header" sheetId="3" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="846">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="877">
   <si>
     <t>Chapter Name</t>
   </si>
@@ -4330,6 +4330,107 @@
   </si>
   <si>
     <t>[Choice1=[NextScene=106][Content=Once in the cave, swim forward, until you feel a pipe.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=107][Content=When you feel the metal of the pipe, go inside.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=108][Content=Plastic, I mean. Then reach up, they will help you get through the grid.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=109][Content=I believe in you, go quick, before the rooms move again.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=110][Content=Wait is this phone even water proof?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=111][Content=Are you alright?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=112][Content=Me?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=113][Content=I’m as lost as you! What does any of that mean?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=114][Content=I didn’t know anything about that!]]
+[Choice2=[NextScene=114][Content=This surely is a dream...]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=115][Content=That's insanity! How are you going to stop this scientist?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=116][Content=Which is?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=117][Content=Wait! How will I know you'll be safe?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=118][Content=We have the same memories?!]]
+[Choice2=[NextScene=118][Content=Is there another way to contact you?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=119][Content=...Did they just throw me like garbage?]]
+[Choice2=[NextScene=119][Content=I guess it’s for the best.]]
+[Choice3=[NextScene=119][Content=NOOOO COME BACK!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=121][Content=Do not tell I haven't warned you.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=122][Content=Watch out! Above you!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=131][NextSceneNoTrust=123][TrustNeed=50][Content=...Fuse? Keep hiding, we're working something out!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=124][Content=DON'T THINK, RUN!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=125][Content=DON'T GRAB THE FUSE DUMBASS, RUN!]]
+[Choice2=[NextScene=125][Content=GRAB IT FAST!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=126][Content=NO!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=129][TrustAdd=-25][Content=Well fuck, it was electrified.]]
+[Choice2=[NextScene=130][Content=Oh shit! Are you alright?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=127][Content=Funny.]]
+[Choice2=[NextScene=130][Content=I'm so sorry!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=16][Content=Yeah, let's find a backdoor.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=132][Content=What happened?!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=133][Content=Just grab the fuse and leave!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=134][Content=Quit yapping and go back to the trapdoor, quick!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=135][Content=Are you... alright?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=136][Content=What are you doing?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=137][Content=Put the fuse and open this trapdoor!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=138][Content=It opened?]]
+[Choice2=[NextScene=138][Content=IT OPENED!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=139][Content=Wait, the signal's getting weaker!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=140][Content=I hope you'll be safe. Goodbye.]]</t>
   </si>
 </sst>
 </file>
@@ -19612,12 +19713,17 @@
       <c r="E107" s="8" t="s">
         <v>711</v>
       </c>
-      <c r="F107" s="8"/>
+      <c r="F107" s="8" t="s">
+        <v>846</v>
+      </c>
       <c r="G107" s="23" t="str">
         <f t="shared" ref="G107:G138" si="4">"[Scene=" &amp; A107 &amp; IF(OR(B107&lt;&gt;"",C107&lt;&gt;"",D107&lt;&gt;""),CHAR(10),"") &amp; IF(B107&lt;&gt;"","[BeepBack=" &amp; B107 &amp; "]","") &amp; IF(C107&lt;&gt;"","[Connection=" &amp; C107 &amp; "]","") &amp; IF(D107&lt;&gt;"","[Timer=" &amp; D107 &amp; "]","") &amp; IF(E107&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E107 &amp; CHAR(10) &amp; "]","") &amp; IF(F107&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F107 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
         <v>[Scene=106
 [Content=
 How will I be able to tell where I am?[Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=107][Content=When you feel the metal of the pipe, go inside.]]
 ]
 ]</v>
       </c>
@@ -19632,12 +19738,17 @@
       <c r="E108" s="8" t="s">
         <v>721</v>
       </c>
-      <c r="F108" s="8"/>
+      <c r="F108" s="8" t="s">
+        <v>847</v>
+      </c>
       <c r="G108" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=107
 [Content=
 [Color=Magenta][Beep=True]It[Wait=500][Beep=True]'s pLa[Wait=500][Beep=True]sTi[Wait=500][Beep=True]c.[Color=White][Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=108][Content=Plastic, I mean. Then reach up, they will help you get through the grid.]]
 ]
 ]</v>
       </c>
@@ -19652,7 +19763,9 @@
       <c r="E109" s="8" t="s">
         <v>722</v>
       </c>
-      <c r="F109" s="8"/>
+      <c r="F109" s="8" t="s">
+        <v>848</v>
+      </c>
       <c r="G109" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=108
@@ -19661,6 +19774,9 @@
 I'm not hyped about death by drowning in a sewage pipe.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]No[Wait=500][Beep=True] wOrR[Wait=500][Beep=True]ieS.[Wait=500][Beep=True]  I gOt[Wait=500][Beep=True] sPaRe[Wait=500][Beep=True] cLoThEs.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]TeLl[Wait=500][Beep=True]  tHeM[Wait=500][Beep=True]  tO hUr[Wait=500][Beep=True]ry uP[Wait=500][Beep=True],  bEiNg rIp[Wait=500][Beep=True]pEd iN[Wait=500][Beep=True]  hAlF wHeN[Wait=500][Beep=True]  rOoMs mOvE[Wait=500][Beep=True]  aGaIn iSn'[Wait=500][Beep=True]t gLa[Wait=500][Beep=True]mOuR eItHeR.[Color=White][Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=109][Content=I believe in you, go quick, before the rooms move again.]]
 ]
 ]</v>
       </c>
@@ -19675,7 +19791,9 @@
       <c r="E110" s="8" t="s">
         <v>717</v>
       </c>
-      <c r="F110" s="8"/>
+      <c r="F110" s="8" t="s">
+        <v>849</v>
+      </c>
       <c r="G110" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=109
@@ -19683,6 +19801,9 @@
 I'll-[Wait=500] Okay, I'm commited to this now.[Wait=500][Space=2]
 Here goes nothing.[Wait=500][Space=2]
 [Color=Gray]*Splash*[Color=White]...[Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=110][Content=Wait is this phone even water proof?]]
 ]
 ]</v>
       </c>
@@ -19697,7 +19818,9 @@
       <c r="E111" s="8" t="s">
         <v>712</v>
       </c>
-      <c r="F111" s="8"/>
+      <c r="F111" s="8" t="s">
+        <v>850</v>
+      </c>
       <c r="G111" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=110
@@ -19709,6 +19832,9 @@
 AAAAAH-[Wait=500] aah...[Wait=500] aah...[Wait=500][Space=2]
 [Color=Magenta]Take my hand![Color=White][Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=111][Content=Are you alright?]]
+]
 ]</v>
       </c>
     </row>
@@ -19722,7 +19848,9 @@
       <c r="E112" s="8" t="s">
         <v>716</v>
       </c>
-      <c r="F112" s="8"/>
+      <c r="F112" s="8" t="s">
+        <v>851</v>
+      </c>
       <c r="G112" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=111
@@ -19736,6 +19864,9 @@
 Are you... talking about the thing's life?[Wait=500][Space=2]
 [Color=Magenta]No.[Wait=500] I'm talking about the person you called.[Color=White][Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=112][Content=Me?]]
+]
 ]</v>
       </c>
     </row>
@@ -19749,13 +19880,18 @@
       <c r="E113" s="8" t="s">
         <v>713</v>
       </c>
-      <c r="F113" s="8"/>
+      <c r="F113" s="8" t="s">
+        <v>852</v>
+      </c>
       <c r="G113" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=112
 [Content=
 [Color=Magenta]You.[Color=White][Wait=500][Space=2]
 What-[Wait=500] What do you mean?[Wait=500] What have you done to me?[Wait=500] Why am I here?[Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=113][Content=I’m as lost as you! What does any of that mean?]]
 ]
 ]</v>
       </c>
@@ -19770,7 +19906,9 @@
       <c r="E114" s="8" t="s">
         <v>714</v>
       </c>
-      <c r="F114" s="8"/>
+      <c r="F114" s="8" t="s">
+        <v>853</v>
+      </c>
       <c r="G114" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=113
@@ -19781,6 +19919,10 @@
 [Color=Magenta]The scientist, as I call him.[Wait=500] He's the one behind our suffering.[Color=White][Wait=500][Space=2]
 So, are we...[Wait=500] clones of you?[Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=114][Content=I didn’t know anything about that!]]
+[Choice2=[NextScene=114][Content=This surely is a dream...]]
+]
 ]</v>
       </c>
     </row>
@@ -19794,7 +19936,9 @@
       <c r="E115" s="8" t="s">
         <v>715</v>
       </c>
-      <c r="F115" s="8"/>
+      <c r="F115" s="8" t="s">
+        <v>854</v>
+      </c>
       <c r="G115" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=114
@@ -19806,6 +19950,9 @@
 I...[Wait=500] That's true.[Wait=500][Space=2]
 I don't want other people to go through what we’ve been, no matter if they're clones or not.[Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=115][Content=That's insanity! How are you going to stop this scientist?]]
+]
 ]</v>
       </c>
     </row>
@@ -19819,7 +19966,9 @@
       <c r="E116" s="8" t="s">
         <v>723</v>
       </c>
-      <c r="F116" s="8"/>
+      <c r="F116" s="8" t="s">
+        <v>855</v>
+      </c>
       <c r="G116" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=115
@@ -19827,6 +19976,9 @@
 [Color=Magenta]I know that this island is designed to self-destruct in case there is a virus breach.[Color=White][Wait=500][Space=2]
 W-Wait what?[Wait=500][Space=2]
 [Color=Magenta]Don't worry, I've planned everything so that we get out unharmed. There is just one more thing to do...[Color=White][Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=116][Content=Which is?]]
 ]
 ]</v>
       </c>
@@ -19841,13 +19993,18 @@
       <c r="E117" s="8" t="s">
         <v>724</v>
       </c>
-      <c r="F117" s="8"/>
+      <c r="F117" s="8" t="s">
+        <v>856</v>
+      </c>
       <c r="G117" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=116
 [Content=
 [Color=Magenta]This phone.[Wait=500] He can use it as a tracker.[Wait=500] You have to throw it away.[Color=White][Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=117][Content=Wait! How will I know you'll be safe?]]
+]
 ]</v>
       </c>
     </row>
@@ -19863,7 +20020,9 @@
       <c r="E118" s="8" t="s">
         <v>725</v>
       </c>
-      <c r="F118" s="8"/>
+      <c r="F118" s="8" t="s">
+        <v>857</v>
+      </c>
       <c r="G118" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=117
@@ -19876,6 +20035,10 @@
 [Color=Magenta]We can't.[Color=White][Wait=500][Space=2]
 [Color=Magenta]I can't even clearly identify if you're part of all of this or not even if we have the same memories.[Color=White][Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=118][Content=We have the same memories?!]]
+[Choice2=[NextScene=118][Content=Is there another way to contact you?]]
+]
 ]</v>
       </c>
     </row>
@@ -19891,7 +20054,9 @@
       <c r="E119" s="8" t="s">
         <v>726</v>
       </c>
-      <c r="F119" s="8"/>
+      <c r="F119" s="8" t="s">
+        <v>858</v>
+      </c>
       <c r="G119" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=118
@@ -19904,6 +20069,11 @@
 [Color=Magenta]Now, the plan starts by getting to the lab unseen and... [Color=Gray]*Fading away*[Color=White]...[Color=White][Wait=500][Space=2]
 ...[Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=119][Content=...Did they just throw me like garbage?]]
+[Choice2=[NextScene=119][Content=I guess it’s for the best.]]
+[Choice3=[NextScene=119][Content=NOOOO COME BACK!]]
+]
 ]</v>
       </c>
     </row>
@@ -19919,7 +20089,9 @@
       <c r="E120" s="8" t="s">
         <v>748</v>
       </c>
-      <c r="F120" s="8"/>
+      <c r="F120" s="8" t="s">
+        <v>825</v>
+      </c>
       <c r="G120" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=119
@@ -19929,6 +20101,12 @@
 [Color=Red]--SIGNAL LOST--[Color=White][Wait=500][Space=2]
 [Color=Green]{THEY'LL HOPEFULLY STOP THE CYCLE. BUT WHY DID THE CYCLE BEGIN?}[Color=White][Wait=500][Space=2]
 [Color=Green]GOOD ENDING.[Color=White][Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextChapter=4][Reset=True][NextScene=1][Content=Retry.]]
+[Choice2=[NextChapter=1][Reset=True][NextScene=1][Content=Retry from Chapter 1.]]
+[Choice3=[Menu=True][Content=Menu.]]
+[Choice4=[Quit=True][Content=Quit.]]
 ]
 ]</v>
       </c>
@@ -19943,7 +20121,9 @@
       <c r="E121" s="8" t="s">
         <v>727</v>
       </c>
-      <c r="F121" s="8"/>
+      <c r="F121" s="8" t="s">
+        <v>859</v>
+      </c>
       <c r="G121" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=120
@@ -19954,6 +20134,9 @@
 I.[Wait=500] Just.[Wait=500] Want.[Wait=500] To.[Wait=500] Leave.[Wait=500][Space=2]
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=121][Content=Do not tell I haven't warned you.]]
+]
 ]</v>
       </c>
     </row>
@@ -19967,7 +20150,9 @@
       <c r="E122" s="8" t="s">
         <v>728</v>
       </c>
-      <c r="F122" s="8"/>
+      <c r="F122" s="8" t="s">
+        <v>860</v>
+      </c>
       <c r="G122" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=121
@@ -19978,6 +20163,9 @@
 ...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThIs[Wait=500][Beep=True] iS[Wait=500][Beep=True] bAd.[Wait=500][Beep=True]  CaN'[Wait=500][Beep=True]t tHeY[Wait=500][Beep=True] sEe tHe[Wait=500][Beep=True] pErSoN[Wait=500][Beep=True] aBoVe?[Color=White][Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=122][Content=Watch out! Above you!]]
+]
 ]</v>
       </c>
     </row>
@@ -19991,7 +20179,9 @@
       <c r="E123" s="8" t="s">
         <v>729</v>
       </c>
-      <c r="F123" s="8"/>
+      <c r="F123" s="8" t="s">
+        <v>861</v>
+      </c>
       <c r="G123" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=122
@@ -20002,6 +20192,9 @@
 ...[Wait=500] Wait is that the...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]DoN[Wait=500][Beep=True]'t dO[Wait=500][Beep=True] aNyThInG[Wait=500][Beep=True] sTuPiD[Wait=500][Beep=True],  i'M[Wait=500][Beep=True] gOnNa[Wait=500][Beep=True] dIsTrAcT[Wait=500][Beep=True] tHeM.[Color=White][Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=131][NextSceneNoTrust=123][TrustNeed=50][Content=...Fuse? Keep hiding, we're working something out!]]
+]
 ]</v>
       </c>
     </row>
@@ -20015,7 +20208,9 @@
       <c r="E124" s="8" t="s">
         <v>730</v>
       </c>
-      <c r="F124" s="8"/>
+      <c r="F124" s="8" t="s">
+        <v>862</v>
+      </c>
       <c r="G124" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=123
@@ -20026,6 +20221,9 @@
 [Color=Gray]*Fast footsteps*[Color=White]...[Wait=500][Space=2]
 FUCK FUCK FUCK![Wait=500] ITS FACE, ITS DISFORMED, IT'S A FUCKING MONSTER![Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=124][Content=DON'T THINK, RUN!]]
+]
 ]</v>
       </c>
     </row>
@@ -20039,13 +20237,19 @@
       <c r="E125" s="8" t="s">
         <v>731</v>
       </c>
-      <c r="F125" s="8"/>
+      <c r="F125" s="8" t="s">
+        <v>863</v>
+      </c>
       <c r="G125" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=124
 [Content=
 WAIT![Wait=500] THE FUSE![Wait=500][Space=2]
 I CAN'T LEAVE IT THERE![Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=125][Content=DON'T GRAB THE FUSE DUMBASS, RUN!]]
+[Choice2=[NextScene=125][Content=GRAB IT FAST!]]
 ]
 ]</v>
       </c>
@@ -20060,7 +20264,9 @@
       <c r="E126" s="8" t="s">
         <v>732</v>
       </c>
-      <c r="F126" s="8"/>
+      <c r="F126" s="8" t="s">
+        <v>864</v>
+      </c>
       <c r="G126" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=125
@@ -20072,6 +20278,9 @@
 [Color=Gray]*DISTORDED SCREAMING*[Color=White]...[Wait=500][Space=2]
 AAAAAAAAAAAAAAAAA-[Color=Gray]*Fleshy noises*[Color=White]...[Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=126][Content=NO!]]
+]
 ]</v>
       </c>
     </row>
@@ -20085,7 +20294,9 @@
       <c r="E127" s="8" t="s">
         <v>733</v>
       </c>
-      <c r="F127" s="8"/>
+      <c r="F127" s="8" t="s">
+        <v>825</v>
+      </c>
       <c r="G127" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=126
@@ -20097,6 +20308,12 @@
 [Color=Red]{IT WAS NOURISHED WITH FLESH. MAYBE IF HE HAD TRUSTED YOU MORE, HE WOULDN'T HAVE GOTTEN CAUGHT?}[Color=White][Wait=500][Space=2]
 [Color=Red]BAD ENDING.[Color=White][Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextChapter=4][Reset=True][NextScene=1][Content=Retry.]]
+[Choice2=[NextChapter=1][Reset=True][NextScene=1][Content=Retry from Chapter 1.]]
+[Choice3=[Menu=True][Content=Menu.]]
+[Choice4=[Quit=True][Content=Quit.]]
+]
 ]</v>
       </c>
     </row>
@@ -20112,7 +20329,9 @@
       <c r="E128" s="8" t="s">
         <v>734</v>
       </c>
-      <c r="F128" s="8"/>
+      <c r="F128" s="8" t="s">
+        <v>825</v>
+      </c>
       <c r="G128" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=127
@@ -20127,6 +20346,12 @@
 [Color=Red]{IT WAS NOURISHED WITH FLESH. MAYBE IF HE HAD TRUSTED YOU MORE, HE WOULDN'T HAVE GOTTEN CAUGHT?}[Color=White][Wait=500][Space=2]
 [Color=Red]BAD ENDING.[Color=White][Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextChapter=4][Reset=True][NextScene=1][Content=Retry.]]
+[Choice2=[NextChapter=1][Reset=True][NextScene=1][Content=Retry from Chapter 1.]]
+[Choice3=[Menu=True][Content=Menu.]]
+[Choice4=[Quit=True][Content=Quit.]]
+]
 ]</v>
       </c>
     </row>
@@ -20140,7 +20365,9 @@
       <c r="E129" s="8" t="s">
         <v>735</v>
       </c>
-      <c r="F129" s="8"/>
+      <c r="F129" s="8" t="s">
+        <v>865</v>
+      </c>
       <c r="G129" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=128
@@ -20151,6 +20378,10 @@
 ...[Wait=500][Space=2]
 OUCH![Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=129][TrustAdd=-25][Content=Well fuck, it was electrified.]]
+[Choice2=[NextScene=130][Content=Oh shit! Are you alright?]]
+]
 ]</v>
       </c>
     </row>
@@ -20166,7 +20397,9 @@
       <c r="E130" s="8" t="s">
         <v>736</v>
       </c>
-      <c r="F130" s="8"/>
+      <c r="F130" s="8" t="s">
+        <v>866</v>
+      </c>
       <c r="G130" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=129
@@ -20175,6 +20408,10 @@
 YOU KNEW?[Wait=500][Space=2]
 Of course it's electrified, why'd you do that?![Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=127][Content=Funny.]]
+[Choice2=[NextScene=130][Content=I'm so sorry!]]
+]
 ]</v>
       </c>
     </row>
@@ -20190,7 +20427,9 @@
       <c r="E131" s="8" t="s">
         <v>737</v>
       </c>
-      <c r="F131" s="8"/>
+      <c r="F131" s="8" t="s">
+        <v>867</v>
+      </c>
       <c r="G131" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=130
@@ -20199,6 +20438,9 @@
 I still feel my muscles vibrating.[Wait=500][Space=2]
 That is no ordinary electric fence, I really feel like it's been setup to trap me.[Wait=500][Space=2]
 Let's just...[Wait=500] Move on.[Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=16][Content=Yeah, let's find a backdoor.]]
 ]
 ]</v>
       </c>
@@ -20213,7 +20455,9 @@
       <c r="E132" s="8" t="s">
         <v>738</v>
       </c>
-      <c r="F132" s="8"/>
+      <c r="F132" s="8" t="s">
+        <v>868</v>
+      </c>
       <c r="G132" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=131
@@ -20224,6 +20468,9 @@
 [Color=Magenta][Beep=True]ThEy[Wait=500][Beep=True] wIlL[Wait=500][Beep=True] cHeCk aNy[Wait=500][Beep=True] lItTlE bIt[Wait=500][Beep=True] oF nOiSe[Wait=500][Beep=True] tHeRe iS.[Color=White][Wait=500][Space=2]
 [Color=Gray]*Loud explosion*[Color=White]...[Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=132][Content=What happened?!]]
+]
 ]</v>
       </c>
     </row>
@@ -20237,7 +20484,9 @@
       <c r="E133" s="8" t="s">
         <v>739</v>
       </c>
-      <c r="F133" s="8"/>
+      <c r="F133" s="8" t="s">
+        <v>869</v>
+      </c>
       <c r="G133" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=132
@@ -20248,6 +20497,9 @@
 ...[Wait=500][Space=2]
 It ignored me?[Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=133][Content=Just grab the fuse and leave!]]
+]
 ]</v>
       </c>
     </row>
@@ -20261,7 +20513,9 @@
       <c r="E134" s="8" t="s">
         <v>740</v>
       </c>
-      <c r="F134" s="8"/>
+      <c r="F134" s="8" t="s">
+        <v>870</v>
+      </c>
       <c r="G134" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=133
@@ -20273,6 +20527,9 @@
 I'm outside, I can see the stairs I took to get in![Wait=500][Space=2]
 If I knew I could've just kept going and climbed through this window![Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=134][Content=Quit yapping and go back to the trapdoor, quick!]]
+]
 ]</v>
       </c>
     </row>
@@ -20286,7 +20543,9 @@
       <c r="E135" s="8" t="s">
         <v>741</v>
       </c>
-      <c r="F135" s="8"/>
+      <c r="F135" s="8" t="s">
+        <v>871</v>
+      </c>
       <c r="G135" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=134
@@ -20294,6 +20553,9 @@
 Yes![Wait=500] Of course![Wait=500][Space=2]
 [Color=Gray]*Running sounds*[Color=White]...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]AlL[Wait=500][Beep=True] oF[Wait=500][Beep=True] tHaT.[Wait=500][Beep=True]  ANd[Wait=500][Beep=True] tHe oNe[Wait=500][Beep=True] wHo cOuLd[Wait=500][Beep=True]'vE sToPpEd[Wait=500][Beep=True] eVeRyThInG[Wait=500][Beep=True] dEcIdEs[Wait=500][Beep=True] tO gO[Wait=500][Beep=True] bAcK tO[Wait=500][Beep=True] tHeIr pRiSoN.[Color=White][Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=135][Content=Are you... alright?]]
 ]
 ]</v>
       </c>
@@ -20308,7 +20570,9 @@
       <c r="E136" s="8" t="s">
         <v>742</v>
       </c>
-      <c r="F136" s="8"/>
+      <c r="F136" s="8" t="s">
+        <v>872</v>
+      </c>
       <c r="G136" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=135
@@ -20317,6 +20581,9 @@
 I'm running towards it![Wait=500] I can even see it from here![Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e's nOt[Wait=500][Beep=True]hInG lEfT[Wait=500][Beep=True] tO dO.[Wait=500][Beep=True]  He wIlL[Wait=500][Beep=True] hAvE wHaT[Wait=500][Beep=True] hE's aLwAyS[Wait=500][Beep=True] lOoKeD fOr[Wait=500][Beep=True] aNd wE'Ll kEeP[Wait=500][Beep=True] sUfFeRiNg.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e iS[Wait=500][Beep=True] nO pO[Wait=500][Beep=True]inT.[Color=White][Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=136][Content=What are you doing?]]
 ]
 ]</v>
       </c>
@@ -20331,7 +20598,9 @@
       <c r="E137" s="8" t="s">
         <v>743</v>
       </c>
-      <c r="F137" s="8"/>
+      <c r="F137" s="8" t="s">
+        <v>873</v>
+      </c>
       <c r="G137" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=136
@@ -20340,6 +20609,9 @@
 Huff...[Wait=500] huff.[Wait=500][Space=2]
 That's it...[Wait=500] I'm on it...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]CoM[Wait=500][Beep=True]E aNd[Wait=500][Beep=True]  GeT mE![Wait=500][Beep=True]  GiVe[Wait=500][Beep=True]  uS bOtH[Wait=500][Beep=True]  tHe pEa[Wait=500][Beep=True]cE aNd[Wait=500][Beep=True]  SaTiEtY[Wait=500][Beep=True]  wE dEsErVe![Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=137][Content=Put the fuse and open this trapdoor!]]
 ]
 ]</v>
       </c>
@@ -20354,13 +20626,19 @@
       <c r="E138" s="8" t="s">
         <v>744</v>
       </c>
-      <c r="F138" s="8"/>
+      <c r="F138" s="8" t="s">
+        <v>874</v>
+      </c>
       <c r="G138" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=137
 [Content=
 So...[Wait=500] I just have to put the fuse here and... [Beep=True][Color=Gray]*Mechanical beeping*[Color=White]... YEEES![Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=138][Content=It opened?]]
+[Choice2=[NextScene=138][Content=IT OPENED!]]
+]
 ]</v>
       </c>
     </row>
@@ -20376,7 +20654,9 @@
       <c r="E139" s="8" t="s">
         <v>745</v>
       </c>
-      <c r="F139" s="8"/>
+      <c r="F139" s="8" t="s">
+        <v>875</v>
+      </c>
       <c r="G139" s="23" t="str">
         <f t="shared" ref="G139:G141" si="5">"[Scene=" &amp; A139 &amp; IF(OR(B139&lt;&gt;"",C139&lt;&gt;"",D139&lt;&gt;""),CHAR(10),"") &amp; IF(B139&lt;&gt;"","[BeepBack=" &amp; B139 &amp; "]","") &amp; IF(C139&lt;&gt;"","[Connection=" &amp; C139 &amp; "]","") &amp; IF(D139&lt;&gt;"","[Timer=" &amp; D139 &amp; "]","") &amp; IF(E139&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E139 &amp; CHAR(10) &amp; "]","") &amp; IF(F139&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F139 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
         <v>[Scene=138
@@ -20386,6 +20666,9 @@
 There are stairs here.[Wait=500] I'm getting down there.[Wait=500][Space=2]
 ...Oh my god...[Wait=500] It was such an intens-[Color=Gray]*SHKRRRRRRRRR*[Color=White]...[Wait=500] I'm so happy that you were here to help me.[Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=139][Content=Wait, the signal's getting weaker!]]
+]
 ]</v>
       </c>
     </row>
@@ -20401,7 +20684,9 @@
       <c r="E140" s="8" t="s">
         <v>746</v>
       </c>
-      <c r="F140" s="8"/>
+      <c r="F140" s="8" t="s">
+        <v>876</v>
+      </c>
       <c r="G140" s="23" t="str">
         <f t="shared" si="5"/>
         <v>[Scene=139
@@ -20412,6 +20697,9 @@
 ...It was a pleasu-[Color=Gray]*SHKRRRRRRRRRRRRRRR*[Color=White]...[Wait=500] Thank you, I'm glad to be y-[Color=Gray]*SHKRRRRRRRRRRR*[Color=White]...[Wait=500][Space=2]
 Goodbye...[Wait=500][Space=2]
 ]
+[Choices=
+[Choice1=[NextScene=140][Content=I hope you'll be safe. Goodbye.]]
+]
 ]</v>
       </c>
     </row>
@@ -20427,7 +20715,9 @@
       <c r="E141" s="8" t="s">
         <v>747</v>
       </c>
-      <c r="F141" s="8"/>
+      <c r="F141" s="8" t="s">
+        <v>825</v>
+      </c>
       <c r="G141" s="23" t="str">
         <f t="shared" si="5"/>
         <v>[Scene=140
@@ -20437,6 +20727,12 @@
 [Color=Red]--SIGNAL LOST--[Color=White][Wait=500][Space=2]
 [Color=Green]{SAME HOPE AND DREAMS, A LIFE FOR ANOTHER. BUT WHAT ABOUT THE OTHERS?}[Color=White][Wait=500][Space=2]
 [Color=Green]GOOD ENDING.[Color=White][Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextChapter=4][Reset=True][NextScene=1][Content=Retry.]]
+[Choice2=[NextChapter=1][Reset=True][NextScene=1][Content=Retry from Chapter 1.]]
+[Choice3=[Menu=True][Content=Menu.]]
+[Choice4=[Quit=True][Content=Quit.]]
 ]
 ]</v>
       </c>

</xml_diff>

<commit_message>
Fix: Finish Chapter 4
</commit_message>
<xml_diff>
--- a/Build/Signal_Lost_Chapters.xlsx
+++ b/Build/Signal_Lost_Chapters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Developpement\Games\Visual Studio 2026\C++\Signal_Lost\Signal_Lost\Build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B33A72C-385C-4833-910B-A7E2ADD0D100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C82A36C9-7F43-425C-A81E-C0BE4B2AC12B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" tabRatio="528" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2996,12 +2996,6 @@
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>You- I mean, you know-...[Wait=500] I get it.[Wait=500][Space=2]
-It's hard to handle some random person calling you for seemingly no reason.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-But thanks for admitting that, I already feel safer if you're able to show a bit of self-awareness.[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>[Choice1=[NextScene=2][NextSceneNoTrust=3][TrustNeed=50][Content=What exactly do you mean by key?]]
 [Choice2=[NextScene=9][NextSceneNoTrust=10][TrustNeed=50][Content=If you can? Would there be anything preventing you?]]</t>
   </si>
@@ -3057,21 +3051,11 @@
 Either have to get around or through it.[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>I-[Wait=500] I get it.[Wait=500][Space=2]
-It's good you're able to put yourself in my place a bit.[Wait=500] Thanks for acknowledging it.[Wait=500][Space=2]
-I'm starting to feel a bit more hopeful about getting out of here if you're on my side.[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>I'm getting there.[Wait=500] But I can already see the place's protected by a fence.[Wait=500][Space=2]
 It isn't a big deal, I could probably find another entrance.[Wait=500][Space=2]
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
 The metal looks brittle. I probably could bend it down and get over it.[Wait=500][Space=2]
 What do you think?[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Hm-[Wait=500] Anyways, there's a fence blocking the way to the main entrance.[Wait=500][Space=2]
-I can either try and get through or go around.[Wait=500][Space=2]
-It looks weak enough to be bent, but this kind of buildings tend to have backdoors.[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>Yeah. The main entrance might be trapped, I'd rather find another way.[Wait=500][Space=2]
@@ -3102,12 +3086,6 @@
 [Color=Magenta][Beep=True]YoU'[Wait=500][Beep=True]rE bEt[Wait=500][Beep=True]tEr hErE[Wait=500][Beep=True]  wItH mE[Wait=500][Beep=True]  tHaN aLo[Wait=500][Beep=True]nE iN[Wait=500][Beep=True]  tHe zOo.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>Wouldn't be trying to defend them, would we?[Wait=500][Space=2]
-Errm-[Wait=500] Anyways.[Wait=500][Space=2]
-Didn't realize the zoo was that close to the factory before.[Wait=500] Civil engineering failed some.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]DaN[Wait=500][Beep=True]gErOuS[Wait=500][Beep=True]  pLa[Wait=500][Beep=True]cE.[Wait=500][Beep=True]  ExpEr[Wait=500][Beep=True]iMeNtS.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>Empty drums, debris, nothing but the usual shit.[Wait=500][Space=2]
 Nowhere else to go, you see, so for now I'll keep looking.[Wait=500][Space=2]
 Stressed out and hungry I feel, still haven't got anything to eat.[Wait=500][Space=2]
@@ -3148,11 +3126,6 @@
     <t>Yeah...[Wait=500] I know.[Wait=500][Space=2]
 Let's just think positively![Wait=500] Everything's...[Wait=500] Fine.[Wait=500][Space=2]
 New hope.[Wait=500] Island friend.[Wait=500] Good news aaall around.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Uuh-[Wait=500] Sure...[Wait=500][Space=2]
-...[Wait=500][Space=2]
-I'll-...[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>Of course.[Wait=500][Space=2]
@@ -3219,13 +3192,6 @@
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>Oh-[Wait=500] Yeah...[Wait=500][Space=2]
-...[Wait=500][Space=2]
-I expected to feel better with someone else on the other end of the phone...[Wait=500] But I-...[Wait=500][Space=2]
-You know...[Wait=500] It's hard...[Wait=500][Space=2]
-[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>"THEY FED ME MY OWN SELF!"...[Wait=500][Space=2]
 I...[Wait=500] Really don't want to discover what happened on this island.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
@@ -3255,14 +3221,6 @@
 Good news, I just stumbled onto what seems to be...[Wait=500] fire escape stairs?[Wait=500][Space=2]
 I'm positive these lead inside the building.[Wait=500][Space=2]
 Chance might be on our side. And I'm not unhappy with doing a bit of exercise.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I'm cl-[Wait=500] Oh-...[Wait=500][Space=2]
-Hold on a minute will you... I'm not a...[Wait=500] ...stair climbing[Wait=500] ...athlete.[Wait=500][Space=2]
-I'm...[Wait=500] getting there...[Wait=500][Space=2]
-Huff... huff...[Wait=500][Space=2]
-.[Wait=500].[Wait=500].[Wait=500][Space=2]
-Guess what.[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>Remember when I talked about luck being on my side?[Wait=500] Shouldn't have said that.[Wait=500][Space=2]
@@ -3346,13 +3304,6 @@
 I also get to pick that beautiful wrench.[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>B-[Wait=500] BAHAHAHA-...[Wait=500][Space=2]
-Who do you take me for?[Wait=500] I'm not a toddler, I can tighten bolts![Wait=500][Space=2]
-My kidnapper might just come and catch these hands right now.[Wait=500][Space=2]
-With this bad boy with me, I ain't loosing to no monster.[Wait=500][Space=2]
-...[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>Absolutely![Wait=500][Space=2]
 ...[Wait=500][Space=2]
 ...I don't know how to put it but it seems...[Wait=500] advanced.[Wait=500][Space=2]
@@ -3370,14 +3321,6 @@
 [Color=Gray]*Door creaks*[Color=White]...[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>It is w-[Wait=500] way colder in here than outside.[Wait=500][Space=2]
-[Color=Gray]*Voice echoes*[Color=White]...[Wait=500][Space=2]
-This place is huge.[Wait=500] I'm in a hallway so long I can't see the other side.[Wait=500][Space=2]
-It really feels like I'm standing in front of a void.[Wait=500][Space=2]
-With only the echo of my voice proving me there's something that way.[Wait=500][Space=2]
-And these big tubes...[Wait=500] This place isn't for making shoes, that's for sure.[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>...[Wait=500] Hundreds?[Wait=500][Space=2]_
 Hard to tell, it goes way past what I'm physically able to see or even reach.[Wait=500][Space=2]
 It's an...[Wait=500] ...[Wait=500] overwhelming view...[Wait=500] This looks like a scene from a Science-fiction movie.[Wait=500][Space=2]
@@ -3458,12 +3401,6 @@
 There's a grid right there.[Wait=500][Space=2]
 But it's too dark to know where it leads.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]Ge[Wait=500][Beep=True]t oUt[Wait=500][Beep=True]  nOw.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I know![Wait=500][Space=2]
-I-[Wait=500] need to get to the down area.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]ThEy[Wait=500][Beep=True]'vE nEgLe[Wait=500][Beep=True]cTeD tO[Wait=500][Beep=True]  tElL yOu[Wait=500][Beep=True]  tHeY fOu[Wait=500][Beep=True]nD aN[Wait=500][Beep=True]  eXiT, i[Wait=500][Beep=True]  cAn sEe[Wait=500][Beep=True]  iT fRo[Wait=500][Beep=True]m a[Wait=500][Beep=True]  cAmErA.[Color=White][Wait=500][Space=2]
-[Color=Magenta][Beep=True]tHe fAlL[Wait=500][Beep=True] mIgHt[Wait=500][Beep=True]  bE rOuGh[Wait=500][Beep=True],  bUt iT's[Wait=500][Beep=True]  wOrTh[Wait=500][Beep=True]  nOt fIgHtInG[Wait=500][Beep=True]  tHeM.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
     <t>I'm not just going to jump into the void![Wait=500] I don't what caused this noise.[Wait=500][Space=2]
@@ -3526,25 +3463,8 @@
 [Color=Gray]*Splashes*[Color=White]...[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>IT'S COMING![Wait=500][Space=2]
-[Color=Gray]*Heavy metalic sounds*[Color=White]...[Wait=500][Space=2]
-.[Wait=500].[Wait=500].[Wait=500][Space=2]
-It-[Wait=500] It missed the opening I fell down from-...[Wait=500][Space=2]
-I-I think I'm safe.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]ThA[Wait=500][Beep=True]nK gO[Wait=500][Beep=True]d.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>I wasn't just gonna face that thing off in a vent, are you stupid?[Wait=500][Space=2]
 How would I even swing it?[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Oh, I took that as ironic...[Wait=500][Space=2]
-Thank you for your help, I wouldn't have made it out without you.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-I-[Wait=500] I'm in a storage room.[Wait=500] The person advising you didn't lie.[Wait=500][Space=2]
-The shelves are laid with cans.[Wait=500][Space=2]
-I'm drenched however, the area is flooded.[Wait=500][Space=2]
-I really wouldn't count on the taste of the mush inside.[Wait=500] Ew...[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>Fuck you![Wait=500] I feared for my life.[Wait=500][Space=2]
@@ -3664,18 +3584,6 @@
 ...[Wait=500] I can't believe all that...[Wait=500] Why am I here?[Wait=500] TELL ME WHY DID YOU MAKE ME?![Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>M-[Wait=500] Me?[Wait=500] As I've said before I-...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]OnE[Wait=500][Beep=True]  oF tHe[Wait=500][Beep=True]  pReVi[Wait=500][Beep=True]oUs.[Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]I'M[Wait=500][Beep=True]  hErE tO[Wait=500][Beep=True]  hElP yOu.[Wait=500][Beep=True]  I'M aBlE[Wait=500][Beep=True]  tO cOmMu[Wait=500][Beep=True]nIcAtE tHrOuGh[Wait=500][Beep=True]  tHe dEsA[Wait=500][Beep=True]fEcTeD cOnTrOl.[Color=White][Wait=500][Space=2]
-[Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]SuR[Wait=500]viVoR[Wait=500][Beep=True],  i’M tRy[Wait=500][Beep=True]iNg tO gEt[Wait=500][Beep=True]  oThErS oUt[Wait=500][Beep=True]  oF hIs[Wait=500][Beep=True]  tRaPs.[Color=White][Wait=500][Space=2]
-Once again, I do NOT know why I'm here nor about any kind of experiments, just help me, alright?[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>What?[Wait=500] Who are you talking to?[Wait=500] You're really starting to freak me out.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]CaN[Wait=500][Beep=True]’t sAy[Wait=500][Beep=True]  mOrE.[Wait=500][Beep=True]  COnNeC[Wait=500][Beep=True]tIoN  uNsTa[Wait=500][Beep=True]bLe.[Wait=500][Beep=True]  YOu’Ll[Wait=500][Beep=True]  gEt cLo[Wait=500][Beep=True]sEr.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>About my size.[Wait=500] They're all connected to a dense net of wires on the ground.[Wait=500][Space=2]
 Almost makes it hard to navigate.[Wait=500][Space=2]
 Also smells quite odd.[Wait=500] It's both off-putting...[Wait=500] and weirdly conforting...[Wait=500][Space=2]
@@ -3693,12 +3601,6 @@
 I feel...[Wait=500][Space=2]
 At home.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]I kNo[Wait=500][Beep=True]w tHiS[Wait=500][Beep=True]  fEeLi[Wait=500][Beep=True]nG...[Wait=500][Beep=True]  aNd hE[Wait=500][Beep=True]  kNoWs[Wait=500][Beep=True]  wHaT hE[Wait=500][Beep=True]'s dOi[Wait=500][Beep=True]nG.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Maybe-[Wait=500] That's what they're for?[Wait=500][Space=2]
-Growing food?[Wait=500][Space=2]
-I-I'm starving.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]YoU[Wait=500][Beep=True]'vE hAd eNo[Wait=500][Beep=True]uGh oF tHaT[Wait=500][Beep=True] aLrEaDy.[Wait=500][Beep=True]  TeLl tHeM[Wait=500][Beep=True] tO cOmE[Wait=500][Beep=True] dOwN, tHeRe[Wait=500][Beep=True] iS cAnNeD[Wait=500][Beep=True] fOoD hErE.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
     <t>[Color=Magenta][Beep=True]AlL oF[Wait=500][Beep=True]  oUr lIvEs[Wait=500][Beep=True],  wE lIvEd[Wait=500][Beep=True]  tHeRe wItHoUt[Wait=500][Beep=True]  kNoWiNg.[Wait=500][Beep=True]  SaMe mEmOrIeS[Wait=500][Beep=True],  sAmE.[Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
@@ -3729,10 +3631,6 @@
 [Color=Magenta]Take my hand![Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>[Color=Magenta]You.[Color=White][Wait=500][Space=2]
-What-[Wait=500] What do you mean?[Wait=500] What have you done to me?[Wait=500] Why am I here?[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>[Color=Magenta]Calm down, both of you.[Wait=500] Neither of you is to blame.[Color=White][Wait=500][Space=2]
 Who am I?[Wait=500] What do you mean, grown?[Wait=500][Space=2]
 [Color=Magenta]You are the successful prototype.[Wait=500] The one he's been waiting for.[Color=White][Wait=500][Space=2]
@@ -3748,21 +3646,6 @@
 I don't want other people to go through what we’ve been, no matter if they're clones or not.[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>You-[Wait=500] Your face![Wait=500][Space=2]
-[Color=Magenta]I should've warned you before.[Wait=500] It's hard to explain that so...[Wait=500] directly.[Wait=500] Most of us figure it out much earlier.[Color=White][Wait=500][Space=2]
-Am I...[Wait=500] Dumber than the-[Wait=500] ...others?[Wait=500][Space=2]
-[Color=Magenta]No, you're healthier.[Wait=500] That "thing" was...[Wait=500] One of us.[Wait=500] Like all of us.[Color=White][Wait=500][Space=2]
-[Color=Magenta]Injected with the disease, grown in an artificial womb in a few weeks.[Color=White][Wait=500][Space=2]
-[Color=Magenta]While we lived all of their life without realising we weren't even there.[Color=White][Wait=500][Space=2]
-Are you... talking about the thing's life?[Wait=500][Space=2]
-[Color=Magenta]No.[Wait=500] I'm talking about the person you called.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I'll-[Wait=500] Okay, I'm commited to this now.[Wait=500][Space=2]
-Here goes nothing.[Wait=500][Space=2]
-[Color=Gray]*Splash*[Color=White]...[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>I-I'll do what you tell.[Wait=500] You've been of great help up until there.[Wait=500] Just tell me where to go, I'll go.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEy...[Wait=500][Beep=True]  tHaNk[Wait=500][Beep=True]  yOu.[Wait=500][Beep=True]  MaYbE[Wait=500][Beep=True]  wE cAn[Wait=500][Beep=True]  eNd tHi[Wait=500][Beep=True]s  cYcLe[Wait=500][Beep=True]  oF mAdNeSs.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]TeLl[Wait=500][Beep=True]  tHeM[Wait=500][Beep=True]  tHeRe[Wait=500][Beep=True]'s a[Wait=500][Beep=True]  wAy[Wait=500][Beep=True]  tO jOi[Wait=500][Beep=True]n mE.[Color=White][Wait=500][Space=2]
@@ -3825,13 +3708,6 @@
 Though it's good to think I could get out in case things go sour.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThIs[Wait=500][Beep=True] iS[Wait=500][Beep=True] bAd.[Wait=500][Beep=True]  CaN'[Wait=500][Beep=True]t tHeY[Wait=500][Beep=True] sEe tHe[Wait=500][Beep=True] pErSoN[Wait=500][Beep=True] aBoVe?[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Wah-[Wait=500] OH SH...[Wait=500][Space=2]
-[Color=Gray]*Whisper*[Color=White]... T-There's...[Wait=500] It’s the thing that chased me in the vent...[Wait=500][Space=2]
-It's o-on the catwalks...[Wait=500][Space=2]
-...[Wait=500] Wait is that the...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]DoN[Wait=500][Beep=True]'t dO[Wait=500][Beep=True] aNyThInG[Wait=500][Beep=True] sTuPiD[Wait=500][Beep=True],  i'M[Wait=500][Beep=True] gOnNa[Wait=500][Beep=True] dIsTrAcT[Wait=500][Beep=True] tHeM.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
     <t>Wait...[Wait=500] I think I can do it on my own...[Wait=500][Space=2]
@@ -3901,7 +3777,649 @@
 It ignored me?[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>O-[Wait=500] Okay![Wait=500][Space=2]
+    <t>Yes![Wait=500] Of course![Wait=500][Space=2]
+[Color=Gray]*Running sounds*[Color=White]...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]AlL[Wait=500][Beep=True] oF[Wait=500][Beep=True] tHaT.[Wait=500][Beep=True]  ANd[Wait=500][Beep=True] tHe oNe[Wait=500][Beep=True] wHo cOuLd[Wait=500][Beep=True]'vE sToPpEd[Wait=500][Beep=True] eVeRyThInG[Wait=500][Beep=True] dEcIdEs[Wait=500][Beep=True] tO gO[Wait=500][Beep=True] bAcK tO[Wait=500][Beep=True] tHeIr pRiSoN.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Color=Gray]*Running sounds*[Color=White]...[Wait=500][Space=2]
+Huff...[Wait=500] huff.[Wait=500][Space=2]
+That's it...[Wait=500] I'm on it...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]CoM[Wait=500][Beep=True]E aNd[Wait=500][Beep=True]  GeT mE![Wait=500][Beep=True]  GiVe[Wait=500][Beep=True]  uS bOtH[Wait=500][Beep=True]  tHe pEa[Wait=500][Beep=True]cE aNd[Wait=500][Beep=True]  SaTiEtY[Wait=500][Beep=True]  wE dEsErVe![Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>So...[Wait=500] I just have to put the fuse here and... [Beep=True][Color=Gray]*Mechanical beeping*[Color=White]... YEEES![Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>YES, IT'S OPENING![Wait=500][Space=2]
+There are stairs here.[Wait=500] I'm getting down there.[Wait=500][Space=2]
+...Oh my god...[Wait=500] It was such an intens-[Color=Gray]*SHKRRRRRRRRR*[Color=White]...[Wait=500] I'm so happy that you were here to help me.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Do you mean th-[Color=Gray]*SHKRRRRRRRRRRR*[Color=White]-ction?[Wait=500] Oh hell no, not after all that![Wait=500][Space=2]
+But I have t-[Color=Gray]*SHKRRRRR*[Color=White]-eep going.[Wait=500] I don't know if I'll be able to contact you agai-[Color=Gray]*SHKRRRRRRR*[Color=White]...[Wait=500][Space=2]
+...It was a pleasu-[Color=Gray]*SHKRRRRRRRRRRRRRRR*[Color=White]...[Wait=500] Thank you, I'm glad to be y-[Color=Gray]*SHKRRRRRRRRRRR*[Color=White]...[Wait=500][Space=2]
+Goodbye...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>...[Wait=500][Space=2]
+[Color=Red]--SIGNAL LOST--[Color=White][Wait=500][Space=2]
+[Color=Green]{SAME HOPE AND DREAMS, A LIFE FOR ANOTHER. BUT WHAT ABOUT THE OTHERS?}[Color=White][Wait=500][Space=2]
+[Color=Green]GOOD ENDING.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>...[Wait=500][Space=2]
+[Color=Red]--SIGNAL LOST--[Color=White][Wait=500][Space=2]
+[Color=Green]{THEY'LL HOPEFULLY STOP THE CYCLE. BUT WHY DID THE CYCLE BEGIN?}[Color=White][Wait=500][Space=2]
+[Color=Green]GOOD ENDING.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=16][Content=Yeah, go for a backdoor.]]
+[Choice2=[NextScene=128][Content=Yeah, get rid of that thing.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=16][Content=You should try to find a backdoor.]]
+[Choice2=[NextScene=128][Content=Let's not waste time, try and push the fence.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=16][Content=Maybe you should go around, you might find something interesting.]]
+[Choice2=[NextScene=128][Content=Yeah let's do that!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=11][Content=I'm being serious. You wouldn't use conditional if you were sure.]]
+[Choice2=[NextScene=12][Content=Is there something wrong?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=13][TrustAdd=25][Content=I shouldn't have said those things.]]
+[Choice2=[NextScene=15][Content=It's hard for the both of us.]]
+[Choice3=[NextScene=15][Content=I get that, I'm sorry.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=14][Content=Yeah, let's not rest.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=16][Content=I like the idea of finding another entrance better.]]
+[Choice2=[NextScene=128][Content=If you can do it, cross the fence.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=16][Content=Get Around it.]]
+[Choice2=[NextScene=128][Content=Get through it.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=16][Content=I'd go around.]]
+[Choice2=[NextScene=128][Content=You should break the fence.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=17][Content=Exactly my thought.]]
+[Choice2=[NextScene=18][Content=Let's hope backdoors aren't either...]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=19][Content=Not like you'd find anything alive anyways.]]
+[Choice2=[NextScene=19][Content=Zoo are smelly.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=19][Content=I mean... This island has a zoo and a museum but no hopistal.]]
+[Choice2=[NextScene=20][Content=I'd doubt that. They probably built this place.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=21][Content=Good one. Have you found an entrance yet?]]
+[Choice2=[NextScene=23][Content=Who's that? What experiments?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=21][Content=It sure did. Did you find anything?]]
+[Choice2=[NextScene=23][Content=What's that about experiments? And still no idea who you are.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=22][Content=I'm sure you'll find something to gnaw on once inside.]]
+[Choice2=[NextScene=22][Content=Did you just... rap?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=31][Content=What does it say?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=24][Content=I'm not talking to you, there's someone in the call.]]
+[Choice2=[NextScene=24][Content=Jeez, fix your signal.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=25][TrustAdd=-25][Content=Don't worry.]]
+[Choice2=[NextScene=28][Content=Someone's interfering. They say they want to help you.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=22][Content=Just keep walking, for fuck's sake.]]
+[Choice2=[NextScene=26][Content=Listen! I'm confused, there's this person-.]]
+[Choice3=[NextScene=127][Content=Well, actually it is.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=27][Content=They seem to interfere with the outgoing signal, hence why you don't hear it.]]
+[Choice2=[NextScene=27][Content=Hard to understand what they're saying. They'd need you to get closer.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=28][Content=You're screwed either way if that's the case. Might as well tempt it.]]
+[Choice2=[NextScene=28][NextSceneNoTrust=29][TrustNeed=50][Content=I'm still there. Don't worry.]]
+[Choice3=[NextScene=29][Content=We'll see. Let's try to listen to them for now.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=30][TrustAdd=25][Content=Getting the spirit!]]
+[Choice2=[NextScene=30][TrustAdd=25][Content=Feeling better?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=30][Content=Just keep going.]]
+[Choice2=[NextScene=30][Content=Trust me!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=32][Content=What does that mean?]]
+[Choice2=[NextScene=33][Content=Who do you think did it?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=34][Content=Yup, I really don't know.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=34][Content=Apparently they didn't.]]
+[Choice2=[NextScene=34][Content=Their connection is shit! I have no idea what a "#?&amp;$%" is.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=35][Content=It's just a matter of grabbing the fuse and leaving.]]
+[Choice2=[NextScene=35][Content=Probably there as part of the game, just keep walking.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=36][Content=So, what's up?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=37][Content=...]]
+[Choice2=[NextScene=37][Content=What?J]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=38][Content=Let's go back and push that fence.]]
+[Choice2=[NextScene=39][Content=If it's a game, there must be a clue somewhere.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=40][Content=What's on the left?]]
+[Choice2=[NextScene=42][Content=What's on the right?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=41][Content=Definitely there on purpose! What's on the right?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=44][Content=Okay, try this.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=43][Content=Too specific to mean nothing, look to the left.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=44][Content=Calm down and try this.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=46][Content=3.]]
+[Choice2=[NextScene=46][Content=4.]]
+[Choice3=[NextScene=45][Content=6.]]
+[Choice4=[NextScene=46][Content=7.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=48][Content=3.]]
+[Choice2=[NextScene=48][Content=4.]]
+[Choice3=[NextScene=47][Content=6.]]
+[Choice4=[NextScene=48][Content=7.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=48][Content=3.]]
+[Choice2=[NextScene=48][Content=4.]]
+[Choice3=[NextScene=48][Content=6.]]
+[Choice4=[NextScene=48][Content=7.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=50][Content=3.]]
+[Choice2=[NextScene=50][Content=4.]]
+[Choice3=[NextScene=49][Content=6.]]
+[Choice4=[NextScene=50][Content=7.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=50][Content=3.]]
+[Choice2=[NextScene=50][Content=4.]]
+[Choice3=[NextScene=50][Content=6.]]
+[Choice4=[NextScene=50][Content=7.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=51][TrustAdd=25][Content=Remembered good ol' 5318008.]]
+[Choice2=[NextScene=52][Content=A friend helped.]]
+[Choice3=[NextScene=53][TrustAdd=-25][Content=Are you dense?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=44][Content=Okay, let's try something else.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=54][Content=Yeah definit-.]]
+[Choice2=[NextScene=54][Content=Hey! I-.]]
+[Choice3=[NextScene=54][Content=I thought you'd worry about the satan stu-.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=53][Content=They simply hinted m-.]]
+[Choice2=[NextScene=55][Content=Actually, they didn-.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=54][Content=You don't seem to str-.]]
+[Choice2=[NextScene=54][Content=Still kinda du-.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=55][Content=Do you even know how to use it?]]
+[Choice2=[NextScene=55][Content=Shh. You might get hurt.]]
+[Choice3=[NextScene=56][Content=Nice.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=56][Content=Oh, ok, you seem to be feeling better.]]
+[Choice2=[NextScene=56][Content=Are... Are you sure?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=57][Content=You quirky little thief.]]
+[Choice2=[NextScene=57][Content=Keep your prize.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=58][Content=Did you open the door?]]
+[Choice2=[NextScene=58][Content=What's inside?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=59][Content=How big exactly?]]
+[Choice2=[NextScene=60][Content=How many are there?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=61][Content=To the person interfering, what's that about?]]
+[Choice2=[NextScene=62][Content=Are you... alright?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=61][Content=Talking to the mystery person, what do you mean?]]
+[Choice2=[NextScene=62][Content=Is everything okay?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=63][Content=What do you mean "grown"?]]
+[Choice2=[NextScene=64][Content=Wait... Do you live there?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=63][Content=Must be the hunger. You really need to eat.]]
+[Choice2=[NextScene=64][Content=Is this... Your home?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=65][Content=There is food down there.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=65][Content=Yes, you need to go down to the damp area. There is food.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=66][Content=Wait. Where are you going?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=67][Content=You really want to go in there?]]
+[Choice2=[NextScene=67][Content=Still got the wrench with you?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=68][Content=Use wrench on big bolt.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=70][NextSceneNoTrust=69][TrustNeed=50][Content=Not even gonna react to me skillfully handling that puzzle?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=71][Content=Always glad to help...]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=71][Content=Always glad to help!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=72][Content=Things are looking up!]]
+[Choice2=[NextScene=73][Content=Getting there already?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=74][Content=Probably, yes.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=74][Content=Your kidnapper, for sure.]]
+[Choice2=[NextScene=74][Content=The person interfering, at least.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=75][Content=What happened?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=76][Content=That wasn't a great idea.]]
+[Choice2=[NextScene=77][Content=You need to get out. Quick.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=78][Content=Please. Just get out.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=78][Content=I know there's an exit, just get out, it's not worth it!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=79][TrustAdd=-25][Content=You're such a hassle.]]
+[Choice1=[NextScene=79][TrustAdd=25][Content=Please, be safe.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=80][Content=Go left.]]
+[Choice2=[NextScene=80][Content=Go right.]]
+[Choice3=[NextScene=80][Content=Go. Back.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=81][Content=Have you found your exit?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[Default=True][NextScene=82][Content=Go back! Now!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[Default=True][NextScene=85][Content=Go left!]]
+[Choice2=[NextScene=85][Content=Go right!]]
+[Choice3=[NextScene=83][Content=Go forward!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=84][Content=Left!]]
+[Choice2=[Default=True][NextScene=85][Content=Right!]]
+[Choice3=[NextScene=83][Content=Forward!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=82][Content=Left!]]
+[Choice2=[NextScene=86][Content=Right!]]
+[Choice3=[Default=True][NextScene=85][Content=Forward!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextChapter=4][Reset=True][NextScene=1][Content=Retry.]]
+[Choice2=[NextChapter=1][Reset=True][NextScene=1][Content=Retry from Chapter 1.]]
+[Choice3=[Menu=True][Content=Menu.]]
+[Choice4=[Quit=True][Content=Quit.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=87][Content=Oh my god, are you alright?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=88][TrustAdd=-25][Content=Good thing you brought that wrench. Well put to use there.]]
+[Choice2=[NextScene=91][NextSceneNoTrust=92][TrustNeed=75][TrustAdd=25][Content=I'm glad you are.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=89][TrustAdd=25][Content=You got the wrong idea! I was talking about the grid!]]
+[Choice2=[NextScene=90][Content=Serves you right for being overconfident.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=93][Content=You've been waiting for this.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=93][Content=Finally, you can eat!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=93][Content="Bon appétit!"...]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=93][Content=Food is food.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=94][Content=Are you done?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=95][Content=Be careful.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=96][Content=Go for the exit.]]
+[Choice2=[NextScene=98][Content=Wait.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=97][Content=You need to get out. The fuse is this way.]]
+[Choice2=[NextScene=98][Content=On second thought. Stop.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=121][Content=Let's go!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=99][TrustAdd=-25][Content=The fuse is a trap.]]
+[Choice2=[NextScene=100][Content=The thing's in that room.]]
+[Choice3=[NextScene=101][TrustAdd=-25][Content=Go where the water is the deepest.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=102][TrustAdd=-25][Content=But the person on the phone is there!]]
+[Choice2=[NextScene=102][TrustAdd=-25][Content=Hope you can hold your breath.]]
+[Choice3=[NextScene=102][Content=The trapdoor won't lead you to the outside world.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=102][TrustAdd=-25][Content=My "friend" is here to help you. Together you can escape.]]
+[Choice2=[NextScene=102][TrustAdd=-25][Content=You'd get killed, you need to take a secret path.]]
+[Choice3=[NextScene=102][Content=You aren't the first. They were once like you.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=102][TrustAdd=-25][Content=Our ally is in a secure room, they'll help!]]
+[Choice2=[NextScene=102][TrustAdd=-25][Content=The fuse isn't there, the truth's under the water.]]
+[Choice3=[NextScene=102][Content=We must learn the truth to prevent this from happening again.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=103][NextSceneNoTrust=120][TrustNeed=75][Content=Please, listen to me.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=104][Content=The person on the line can help you, they’ve been of great help to me as well.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=105][Content=The wall has a hole in it, beneath the water. Swim until you reach the other side.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=106][Content=Once in the cave, swim forward, until you feel a pipe.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=107][Content=When you feel the metal of the pipe, go inside.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=108][Content=Plastic, I mean. Then reach up, they will help you get through the grid.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=109][Content=I believe in you, go quick, before the rooms move again.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=110][Content=Wait is this phone even water proof?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=111][Content=Are you alright?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=112][Content=Me?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=113][Content=I’m as lost as you! What does any of that mean?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=114][Content=I didn’t know anything about that!]]
+[Choice2=[NextScene=114][Content=This surely is a dream...]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=115][Content=That's insanity! How are you going to stop this scientist?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=116][Content=Which is?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=117][Content=Wait! How will I know you'll be safe?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=118][Content=We have the same memories?!]]
+[Choice2=[NextScene=118][Content=Is there another way to contact you?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=119][Content=...Did they just throw me like garbage?]]
+[Choice2=[NextScene=119][Content=I guess it’s for the best.]]
+[Choice3=[NextScene=119][Content=NOOOO COME BACK!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=121][Content=Do not tell I haven't warned you.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=122][Content=Watch out! Above you!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=131][NextSceneNoTrust=123][TrustNeed=50][Content=...Fuse? Keep hiding, we're working something out!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=124][Content=DON'T THINK, RUN!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=125][Content=DON'T GRAB THE FUSE DUMBASS, RUN!]]
+[Choice2=[NextScene=125][Content=GRAB IT FAST!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=126][Content=NO!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=129][TrustAdd=-25][Content=Well fuck, it was electrified.]]
+[Choice2=[NextScene=130][Content=Oh shit! Are you alright?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=127][Content=Funny.]]
+[Choice2=[NextScene=130][Content=I'm so sorry!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=16][Content=Yeah, let's find a backdoor.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=132][Content=What happened?!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=133][Content=Just grab the fuse and leave!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=134][Content=Quit yapping and go back to the trapdoor, quick!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=135][Content=Are you... alright?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=136][Content=What are you doing?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=137][Content=Put the fuse and open this trapdoor!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=138][Content=It opened?]]
+[Choice2=[NextScene=138][Content=IT OPENED!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=139][Content=Wait, the signal's getting weaker!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=140][Content=I hope you'll be safe. Goodbye.]]</t>
+  </si>
+  <si>
+    <t>Wouldn't be trying to defend them, would we?[Wait=500][Space=2]
+Errm-...[Wait=500] Anyways.[Wait=500][Space=2]
+Didn't realize the zoo was that close to the factory before.[Wait=500] Civil engineering failed some.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]DaN[Wait=500][Beep=True]gErOuS[Wait=500][Beep=True]  pLa[Wait=500][Beep=True]cE.[Wait=500][Beep=True]  ExpEr[Wait=500][Beep=True]iMeNtS.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>M-...[Wait=500] Me?[Wait=500] As I've said before I-...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]OnE[Wait=500][Beep=True]  oF tHe[Wait=500][Beep=True]  pReVi[Wait=500][Beep=True]oUs.[Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]I'M[Wait=500][Beep=True]  hErE tO[Wait=500][Beep=True]  hElP yOu.[Wait=500][Beep=True]  I'M aBlE[Wait=500][Beep=True]  tO cOmMu[Wait=500][Beep=True]nIcAtE tHrOuGh[Wait=500][Beep=True]  tHe dEsA[Wait=500][Beep=True]fEcTeD cOnTrOl.[Color=White][Wait=500][Space=2]
+[Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]SuR[Wait=500]viVoR[Wait=500][Beep=True],  i’M tRy[Wait=500][Beep=True]iNg tO gEt[Wait=500][Beep=True]  oThErS oUt[Wait=500][Beep=True]  oF hIs[Wait=500][Beep=True]  tRaPs.[Color=White][Wait=500][Space=2]
+Once again, I do NOT know why I'm here nor about any kind of experiments, just help me, alright?[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>What?[Wait=500] Who are you talking to?[Wait=500] You're really starting to freak me out.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]CaN[Wait=500][Beep=True]'t sAy[Wait=500][Beep=True]  mOrE.[Wait=500][Beep=True]  COnNeC[Wait=500][Beep=True]tIoN  uNsTa[Wait=500][Beep=True]bLe.[Wait=500][Beep=True]  YOu'Ll[Wait=500][Beep=True]  gEt cLo[Wait=500][Beep=True]sEr.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Uuh-...[Wait=500] Sure...[Wait=500][Space=2]
+...[Wait=500][Space=2]
+I'll-...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Hm-...[Wait=500] Anyways, there's a fence blocking the way to the main entrance.[Wait=500][Space=2]
+I can either try and get through or go around.[Wait=500][Space=2]
+It looks weak enough to be bent, but this kind of buildings tend to have backdoors.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I-...[Wait=500] I get it.[Wait=500][Space=2]
+It's good you're able to put yourself in my place a bit.[Wait=500] Thanks for acknowledging it.[Wait=500][Space=2]
+I'm starting to feel a bit more hopeful about getting out of here if you're on my side.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Oh-...[Wait=500] Yeah...[Wait=500][Space=2]
+...[Wait=500][Space=2]
+I expected to feel better with someone else on the other end of the phone...[Wait=500] But I-...[Wait=500][Space=2]
+You know...[Wait=500] It's hard...[Wait=500][Space=2]
+[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>You-... I mean, you know-...[Wait=500] I get it.[Wait=500][Space=2]
+It's hard to handle some random person calling you for seemingly no reason.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+But thanks for admitting that, I already feel safer if you're able to show a bit of self-awareness.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I'm cl-...[Wait=500] Oh-...[Wait=500][Space=2]
+Hold on a minute will you... I'm not a...[Wait=500] ...stair climbing[Wait=500] ...athlete.[Wait=500][Space=2]
+I'm...[Wait=500] getting there...[Wait=500][Space=2]
+Huff... huff...[Wait=500][Space=2]
+.[Wait=500].[Wait=500].[Wait=500][Space=2]
+Guess what.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>B-...[Wait=500] BAHAHAHA-...[Wait=500][Space=2]
+Who do you take me for?[Wait=500] I'm not a toddler, I can tighten bolts![Wait=500][Space=2]
+My kidnapper might just come and catch these hands right now.[Wait=500][Space=2]
+With this bad boy with me, I ain't loosing to no monster.[Wait=500][Space=2]
+...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>It is w-...[Wait=500] way colder in here than outside.[Wait=500][Space=2]
+[Color=Gray]*Voice echoes*[Color=White]...[Wait=500][Space=2]
+This place is huge.[Wait=500] I'm in a hallway so long I can't see the other side.[Wait=500][Space=2]
+It really feels like I'm standing in front of a void.[Wait=500][Space=2]
+With only the echo of my voice proving me there's something that way.[Wait=500][Space=2]
+And these big tubes...[Wait=500] This place isn't for making shoes, that's for sure.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Maybe-...[Wait=500] That's what they're for?[Wait=500][Space=2]
+Growing food?[Wait=500][Space=2]
+I-I'm starving.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]YoU[Wait=500][Beep=True]'vE hAd eNo[Wait=500][Beep=True]uGh oF tHaT[Wait=500][Beep=True] aLrEaDy.[Wait=500][Beep=True]  TeLl tHeM[Wait=500][Beep=True] tO cOmE[Wait=500][Beep=True] dOwN, tHeRe[Wait=500][Beep=True] iS cAnNeD[Wait=500][Beep=True] fOoD hErE.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I know![Wait=500][Space=2]
+I-...[Wait=500] need to get to the down area.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]ThEy[Wait=500][Beep=True]'vE nEgLe[Wait=500][Beep=True]cTeD tO[Wait=500][Beep=True]  tElL yOu[Wait=500][Beep=True]  tHeY fOu[Wait=500][Beep=True]nD aN[Wait=500][Beep=True]  eXiT, i[Wait=500][Beep=True]  cAn sEe[Wait=500][Beep=True]  iT fRo[Wait=500][Beep=True]m a[Wait=500][Beep=True]  cAmErA.[Color=White][Wait=500][Space=2]
+[Color=Magenta][Beep=True]tHe fAlL[Wait=500][Beep=True] mIgHt[Wait=500][Beep=True]  bE rOuGh[Wait=500][Beep=True],  bUt iT's[Wait=500][Beep=True]  wOrTh[Wait=500][Beep=True]  nOt fIgHtInG[Wait=500][Beep=True]  tHeM.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>IT'S COMING![Wait=500][Space=2]
+[Color=Gray]*Heavy metalic sounds*[Color=White]...[Wait=500][Space=2]
+.[Wait=500].[Wait=500].[Wait=500][Space=2]
+It-...[Wait=500] It missed the opening I fell down from-...[Wait=500][Space=2]
+I-I think I'm safe.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]ThA[Wait=500][Beep=True]nK gO[Wait=500][Beep=True]d.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Oh, I took that as ironic...[Wait=500][Space=2]
+Thank you for your help, I wouldn't have made it out without you.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+I-...[Wait=500] I'm in a storage room.[Wait=500] The person advising you didn't lie.[Wait=500][Space=2]
+The shelves are laid with cans.[Wait=500][Space=2]
+I'm drenched however, the area is flooded.[Wait=500][Space=2]
+I really wouldn't count on the taste of the mush inside.[Wait=500] Ew...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I'll-...[Wait=500] Okay, I'm commited to this now.[Wait=500][Space=2]
+Here goes nothing.[Wait=500][Space=2]
+[Color=Gray]*Splash*[Color=White]...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Color=Magenta]You.[Color=White][Wait=500][Space=2]
+What-...[Wait=500] What do you mean?[Wait=500] What have you done to me?[Wait=500] Why am I here?[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>You-[Wait=500] Your face![Wait=500][Space=2]
+[Color=Magenta]I should've warned you before.[Wait=500] It's hard to explain that so...[Wait=500] directly.[Wait=500] Most of us figure it out much earlier.[Color=White][Wait=500][Space=2]
+Am I...[Wait=500] Dumber than the-...[Wait=500] ...others?[Wait=500][Space=2]
+[Color=Magenta]No, you're healthier.[Wait=500] That "thing" was...[Wait=500] One of us.[Wait=500] Like all of us.[Color=White][Wait=500][Space=2]
+[Color=Magenta]Injected with the disease, grown in an artificial womb in a few weeks.[Color=White][Wait=500][Space=2]
+[Color=Magenta]While we lived all of their life without realising we weren't even there.[Color=White][Wait=500][Space=2]
+Are you... talking about the thing's life?[Wait=500][Space=2]
+[Color=Magenta]No.[Wait=500] I'm talking about the person you called.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Wah-...[Wait=500] OH SH...[Wait=500][Space=2]
+[Color=Gray]*Whisper*[Color=White]... T-There's...[Wait=500] It’s the thing that chased me in the vent...[Wait=500][Space=2]
+It's o-on the catwalks...[Wait=500][Space=2]
+...[Wait=500] Wait is that the...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]DoN[Wait=500][Beep=True]'t dO[Wait=500][Beep=True] aNyThInG[Wait=500][Beep=True] sTuPiD[Wait=500][Beep=True],  i'M[Wait=500][Beep=True] gOnNa[Wait=500][Beep=True] dIsTrAcT[Wait=500][Beep=True] tHeM.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>O-...[Wait=500] Okay![Wait=500][Space=2]
 [Color=Gray]*Running sounds*[Color=White]...[Wait=500][Space=2]
 I GOT IT![Wait=500][Space=2]
 [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
@@ -3909,528 +4427,10 @@
 If I knew I could've just kept going and climbed through this window![Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>Yes![Wait=500] Of course![Wait=500][Space=2]
-[Color=Gray]*Running sounds*[Color=White]...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]AlL[Wait=500][Beep=True] oF[Wait=500][Beep=True] tHaT.[Wait=500][Beep=True]  ANd[Wait=500][Beep=True] tHe oNe[Wait=500][Beep=True] wHo cOuLd[Wait=500][Beep=True]'vE sToPpEd[Wait=500][Beep=True] eVeRyThInG[Wait=500][Beep=True] dEcIdEs[Wait=500][Beep=True] tO gO[Wait=500][Beep=True] bAcK tO[Wait=500][Beep=True] tHeIr pRiSoN.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I-[Wait=500] I am![Wait=500][Space=2]
+    <t>I-...[Wait=500] I am![Wait=500][Space=2]
 I'm running towards it![Wait=500] I can even see it from here![Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e's nOt[Wait=500][Beep=True]hInG lEfT[Wait=500][Beep=True] tO dO.[Wait=500][Beep=True]  He wIlL[Wait=500][Beep=True] hAvE wHaT[Wait=500][Beep=True] hE's aLwAyS[Wait=500][Beep=True] lOoKeD fOr[Wait=500][Beep=True] aNd wE'Ll kEeP[Wait=500][Beep=True] sUfFeRiNg.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e iS[Wait=500][Beep=True] nO pO[Wait=500][Beep=True]inT.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>[Color=Gray]*Running sounds*[Color=White]...[Wait=500][Space=2]
-Huff...[Wait=500] huff.[Wait=500][Space=2]
-That's it...[Wait=500] I'm on it...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]CoM[Wait=500][Beep=True]E aNd[Wait=500][Beep=True]  GeT mE![Wait=500][Beep=True]  GiVe[Wait=500][Beep=True]  uS bOtH[Wait=500][Beep=True]  tHe pEa[Wait=500][Beep=True]cE aNd[Wait=500][Beep=True]  SaTiEtY[Wait=500][Beep=True]  wE dEsErVe![Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>So...[Wait=500] I just have to put the fuse here and... [Beep=True][Color=Gray]*Mechanical beeping*[Color=White]... YEEES![Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>YES, IT'S OPENING![Wait=500][Space=2]
-There are stairs here.[Wait=500] I'm getting down there.[Wait=500][Space=2]
-...Oh my god...[Wait=500] It was such an intens-[Color=Gray]*SHKRRRRRRRRR*[Color=White]...[Wait=500] I'm so happy that you were here to help me.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Do you mean th-[Color=Gray]*SHKRRRRRRRRRRR*[Color=White]-ction?[Wait=500] Oh hell no, not after all that![Wait=500][Space=2]
-But I have t-[Color=Gray]*SHKRRRRR*[Color=White]-eep going.[Wait=500] I don't know if I'll be able to contact you agai-[Color=Gray]*SHKRRRRRRR*[Color=White]...[Wait=500][Space=2]
-...It was a pleasu-[Color=Gray]*SHKRRRRRRRRRRRRRRR*[Color=White]...[Wait=500] Thank you, I'm glad to be y-[Color=Gray]*SHKRRRRRRRRRRR*[Color=White]...[Wait=500][Space=2]
-Goodbye...[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>...[Wait=500][Space=2]
-[Color=Red]--SIGNAL LOST--[Color=White][Wait=500][Space=2]
-[Color=Green]{SAME HOPE AND DREAMS, A LIFE FOR ANOTHER. BUT WHAT ABOUT THE OTHERS?}[Color=White][Wait=500][Space=2]
-[Color=Green]GOOD ENDING.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>...[Wait=500][Space=2]
-[Color=Red]--SIGNAL LOST--[Color=White][Wait=500][Space=2]
-[Color=Green]{THEY'LL HOPEFULLY STOP THE CYCLE. BUT WHY DID THE CYCLE BEGIN?}[Color=White][Wait=500][Space=2]
-[Color=Green]GOOD ENDING.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=16][Content=Yeah, go for a backdoor.]]
-[Choice2=[NextScene=128][Content=Yeah, get rid of that thing.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=16][Content=You should try to find a backdoor.]]
-[Choice2=[NextScene=128][Content=Let's not waste time, try and push the fence.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=16][Content=Maybe you should go around, you might find something interesting.]]
-[Choice2=[NextScene=128][Content=Yeah let's do that!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=11][Content=I'm being serious. You wouldn't use conditional if you were sure.]]
-[Choice2=[NextScene=12][Content=Is there something wrong?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=13][TrustAdd=25][Content=I shouldn't have said those things.]]
-[Choice2=[NextScene=15][Content=It's hard for the both of us.]]
-[Choice3=[NextScene=15][Content=I get that, I'm sorry.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=14][Content=Yeah, let's not rest.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=16][Content=I like the idea of finding another entrance better.]]
-[Choice2=[NextScene=128][Content=If you can do it, cross the fence.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=16][Content=Get Around it.]]
-[Choice2=[NextScene=128][Content=Get through it.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=16][Content=I'd go around.]]
-[Choice2=[NextScene=128][Content=You should break the fence.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=17][Content=Exactly my thought.]]
-[Choice2=[NextScene=18][Content=Let's hope backdoors aren't either...]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=19][Content=Not like you'd find anything alive anyways.]]
-[Choice2=[NextScene=19][Content=Zoo are smelly.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=19][Content=I mean... This island has a zoo and a museum but no hopistal.]]
-[Choice2=[NextScene=20][Content=I'd doubt that. They probably built this place.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=21][Content=Good one. Have you found an entrance yet?]]
-[Choice2=[NextScene=23][Content=Who's that? What experiments?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=21][Content=It sure did. Did you find anything?]]
-[Choice2=[NextScene=23][Content=What's that about experiments? And still no idea who you are.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=22][Content=I'm sure you'll find something to gnaw on once inside.]]
-[Choice2=[NextScene=22][Content=Did you just... rap?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=31][Content=What does it say?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=24][Content=I'm not talking to you, there's someone in the call.]]
-[Choice2=[NextScene=24][Content=Jeez, fix your signal.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=25][TrustAdd=-25][Content=Don't worry.]]
-[Choice2=[NextScene=28][Content=Someone's interfering. They say they want to help you.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=22][Content=Just keep walking, for fuck's sake.]]
-[Choice2=[NextScene=26][Content=Listen! I'm confused, there's this person-.]]
-[Choice3=[NextScene=127][Content=Well, actually it is.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=27][Content=They seem to interfere with the outgoing signal, hence why you don't hear it.]]
-[Choice2=[NextScene=27][Content=Hard to understand what they're saying. They'd need you to get closer.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=28][Content=You're screwed either way if that's the case. Might as well tempt it.]]
-[Choice2=[NextScene=28][NextSceneNoTrust=29][TrustNeed=50][Content=I'm still there. Don't worry.]]
-[Choice3=[NextScene=29][Content=We'll see. Let's try to listen to them for now.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=30][TrustAdd=25][Content=Getting the spirit!]]
-[Choice2=[NextScene=30][TrustAdd=25][Content=Feeling better?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=30][Content=Just keep going.]]
-[Choice2=[NextScene=30][Content=Trust me!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=32][Content=What does that mean?]]
-[Choice2=[NextScene=33][Content=Who do you think did it?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=34][Content=Yup, I really don't know.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=34][Content=Apparently they didn't.]]
-[Choice2=[NextScene=34][Content=Their connection is shit! I have no idea what a "#?&amp;$%" is.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=35][Content=It's just a matter of grabbing the fuse and leaving.]]
-[Choice2=[NextScene=35][Content=Probably there as part of the game, just keep walking.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=36][Content=So, what's up?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=37][Content=...]]
-[Choice2=[NextScene=37][Content=What?J]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=38][Content=Let's go back and push that fence.]]
-[Choice2=[NextScene=39][Content=If it's a game, there must be a clue somewhere.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=40][Content=What's on the left?]]
-[Choice2=[NextScene=42][Content=What's on the right?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=41][Content=Definitely there on purpose! What's on the right?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=44][Content=Okay, try this.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=43][Content=Too specific to mean nothing, look to the left.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=44][Content=Calm down and try this.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=46][Content=3.]]
-[Choice2=[NextScene=46][Content=4.]]
-[Choice3=[NextScene=45][Content=6.]]
-[Choice4=[NextScene=46][Content=7.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=48][Content=3.]]
-[Choice2=[NextScene=48][Content=4.]]
-[Choice3=[NextScene=47][Content=6.]]
-[Choice4=[NextScene=48][Content=7.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=48][Content=3.]]
-[Choice2=[NextScene=48][Content=4.]]
-[Choice3=[NextScene=48][Content=6.]]
-[Choice4=[NextScene=48][Content=7.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=50][Content=3.]]
-[Choice2=[NextScene=50][Content=4.]]
-[Choice3=[NextScene=49][Content=6.]]
-[Choice4=[NextScene=50][Content=7.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=50][Content=3.]]
-[Choice2=[NextScene=50][Content=4.]]
-[Choice3=[NextScene=50][Content=6.]]
-[Choice4=[NextScene=50][Content=7.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=51][TrustAdd=25][Content=Remembered good ol' 5318008.]]
-[Choice2=[NextScene=52][Content=A friend helped.]]
-[Choice3=[NextScene=53][TrustAdd=-25][Content=Are you dense?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=44][Content=Okay, let's try something else.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=54][Content=Yeah definit-.]]
-[Choice2=[NextScene=54][Content=Hey! I-.]]
-[Choice3=[NextScene=54][Content=I thought you'd worry about the satan stu-.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=53][Content=They simply hinted m-.]]
-[Choice2=[NextScene=55][Content=Actually, they didn-.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=54][Content=You don't seem to str-.]]
-[Choice2=[NextScene=54][Content=Still kinda du-.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=55][Content=Do you even know how to use it?]]
-[Choice2=[NextScene=55][Content=Shh. You might get hurt.]]
-[Choice3=[NextScene=56][Content=Nice.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=56][Content=Oh, ok, you seem to be feeling better.]]
-[Choice2=[NextScene=56][Content=Are... Are you sure?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=57][Content=You quirky little thief.]]
-[Choice2=[NextScene=57][Content=Keep your prize.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=58][Content=Did you open the door?]]
-[Choice2=[NextScene=58][Content=What's inside?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=59][Content=How big exactly?]]
-[Choice2=[NextScene=60][Content=How many are there?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=61][Content=To the person interfering, what's that about?]]
-[Choice2=[NextScene=62][Content=Are you... alright?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=61][Content=Talking to the mystery person, what do you mean?]]
-[Choice2=[NextScene=62][Content=Is everything okay?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=63][Content=What do you mean "grown"?]]
-[Choice2=[NextScene=64][Content=Wait... Do you live there?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=63][Content=Must be the hunger. You really need to eat.]]
-[Choice2=[NextScene=64][Content=Is this... Your home?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=65][Content=There is food down there.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=65][Content=Yes, you need to go down to the damp area. There is food.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=66][Content=Wait. Where are you going?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=67][Content=You really want to go in there?]]
-[Choice2=[NextScene=67][Content=Still got the wrench with you?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=68][Content=Use wrench on big bolt.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=70][NextSceneNoTrust=69][TrustNeed=50][Content=Not even gonna react to me skillfully handling that puzzle?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=71][Content=Always glad to help...]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=71][Content=Always glad to help!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=72][Content=Things are looking up!]]
-[Choice2=[NextScene=73][Content=Getting there already?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=74][Content=Probably, yes.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=74][Content=Your kidnapper, for sure.]]
-[Choice2=[NextScene=74][Content=The person interfering, at least.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=75][Content=What happened?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=76][Content=That wasn't a great idea.]]
-[Choice2=[NextScene=77][Content=You need to get out. Quick.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=78][Content=Please. Just get out.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=78][Content=I know there's an exit, just get out, it's not worth it!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=79][TrustAdd=-25][Content=You're such a hassle.]]
-[Choice1=[NextScene=79][TrustAdd=25][Content=Please, be safe.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=80][Content=Go left.]]
-[Choice2=[NextScene=80][Content=Go right.]]
-[Choice3=[NextScene=80][Content=Go. Back.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=81][Content=Have you found your exit?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[Default=True][NextScene=82][Content=Go back! Now!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[Default=True][NextScene=85][Content=Go left!]]
-[Choice2=[NextScene=85][Content=Go right!]]
-[Choice3=[NextScene=83][Content=Go forward!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=84][Content=Left!]]
-[Choice2=[Default=True][NextScene=85][Content=Right!]]
-[Choice3=[NextScene=83][Content=Forward!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=82][Content=Left!]]
-[Choice2=[NextScene=86][Content=Right!]]
-[Choice3=[Default=True][NextScene=85][Content=Forward!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextChapter=4][Reset=True][NextScene=1][Content=Retry.]]
-[Choice2=[NextChapter=1][Reset=True][NextScene=1][Content=Retry from Chapter 1.]]
-[Choice3=[Menu=True][Content=Menu.]]
-[Choice4=[Quit=True][Content=Quit.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=87][Content=Oh my god, are you alright?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=88][TrustAdd=-25][Content=Good thing you brought that wrench. Well put to use there.]]
-[Choice2=[NextScene=91][NextSceneNoTrust=92][TrustNeed=75][TrustAdd=25][Content=I'm glad you are.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=89][TrustAdd=25][Content=You got the wrong idea! I was talking about the grid!]]
-[Choice2=[NextScene=90][Content=Serves you right for being overconfident.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=93][Content=You've been waiting for this.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=93][Content=Finally, you can eat!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=93][Content="Bon appétit!"...]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=93][Content=Food is food.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=94][Content=Are you done?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=95][Content=Be careful.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=96][Content=Go for the exit.]]
-[Choice2=[NextScene=98][Content=Wait.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=97][Content=You need to get out. The fuse is this way.]]
-[Choice2=[NextScene=98][Content=On second thought. Stop.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=121][Content=Let's go!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=99][TrustAdd=-25][Content=The fuse is a trap.]]
-[Choice2=[NextScene=100][Content=The thing's in that room.]]
-[Choice3=[NextScene=101][TrustAdd=-25][Content=Go where the water is the deepest.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=102][TrustAdd=-25][Content=But the person on the phone is there!]]
-[Choice2=[NextScene=102][TrustAdd=-25][Content=Hope you can hold your breath.]]
-[Choice3=[NextScene=102][Content=The trapdoor won't lead you to the outside world.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=102][TrustAdd=-25][Content=My "friend" is here to help you. Together you can escape.]]
-[Choice2=[NextScene=102][TrustAdd=-25][Content=You'd get killed, you need to take a secret path.]]
-[Choice3=[NextScene=102][Content=You aren't the first. They were once like you.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=102][TrustAdd=-25][Content=Our ally is in a secure room, they'll help!]]
-[Choice2=[NextScene=102][TrustAdd=-25][Content=The fuse isn't there, the truth's under the water.]]
-[Choice3=[NextScene=102][Content=We must learn the truth to prevent this from happening again.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=103][NextSceneNoTrust=120][TrustNeed=75][Content=Please, listen to me.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=104][Content=The person on the line can help you, they’ve been of great help to me as well.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=105][Content=The wall has a hole in it, beneath the water. Swim until you reach the other side.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=106][Content=Once in the cave, swim forward, until you feel a pipe.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=107][Content=When you feel the metal of the pipe, go inside.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=108][Content=Plastic, I mean. Then reach up, they will help you get through the grid.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=109][Content=I believe in you, go quick, before the rooms move again.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=110][Content=Wait is this phone even water proof?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=111][Content=Are you alright?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=112][Content=Me?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=113][Content=I’m as lost as you! What does any of that mean?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=114][Content=I didn’t know anything about that!]]
-[Choice2=[NextScene=114][Content=This surely is a dream...]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=115][Content=That's insanity! How are you going to stop this scientist?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=116][Content=Which is?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=117][Content=Wait! How will I know you'll be safe?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=118][Content=We have the same memories?!]]
-[Choice2=[NextScene=118][Content=Is there another way to contact you?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=119][Content=...Did they just throw me like garbage?]]
-[Choice2=[NextScene=119][Content=I guess it’s for the best.]]
-[Choice3=[NextScene=119][Content=NOOOO COME BACK!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=121][Content=Do not tell I haven't warned you.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=122][Content=Watch out! Above you!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=131][NextSceneNoTrust=123][TrustNeed=50][Content=...Fuse? Keep hiding, we're working something out!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=124][Content=DON'T THINK, RUN!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=125][Content=DON'T GRAB THE FUSE DUMBASS, RUN!]]
-[Choice2=[NextScene=125][Content=GRAB IT FAST!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=126][Content=NO!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=129][TrustAdd=-25][Content=Well fuck, it was electrified.]]
-[Choice2=[NextScene=130][Content=Oh shit! Are you alright?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=127][Content=Funny.]]
-[Choice2=[NextScene=130][Content=I'm so sorry!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=16][Content=Yeah, let's find a backdoor.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=132][Content=What happened?!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=133][Content=Just grab the fuse and leave!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=134][Content=Quit yapping and go back to the trapdoor, quick!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=135][Content=Are you... alright?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=136][Content=What are you doing?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=137][Content=Put the fuse and open this trapdoor!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=138][Content=It opened?]]
-[Choice2=[NextScene=138][Content=IT OPENED!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=139][Content=Wait, the signal's getting weaker!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=140][Content=I hope you'll be safe. Goodbye.]]</t>
   </si>
 </sst>
 </file>
@@ -10234,7 +10234,7 @@
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
       <c r="E32" s="8" t="s">
-        <v>625</v>
+        <v>620</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>386</v>
@@ -10265,7 +10265,7 @@
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
       <c r="E33" s="8" t="s">
-        <v>626</v>
+        <v>621</v>
       </c>
       <c r="F33" s="8" t="s">
         <v>106</v>
@@ -10761,7 +10761,7 @@
       </c>
       <c r="D50" s="7"/>
       <c r="E50" s="8" t="s">
-        <v>627</v>
+        <v>622</v>
       </c>
       <c r="F50" s="8" t="s">
         <v>118</v>
@@ -11245,7 +11245,7 @@
       <c r="C67" s="7"/>
       <c r="D67" s="7"/>
       <c r="E67" s="8" t="s">
-        <v>695</v>
+        <v>683</v>
       </c>
       <c r="F67" s="8" t="s">
         <v>129</v>
@@ -11272,7 +11272,7 @@
       <c r="C68" s="7"/>
       <c r="D68" s="7"/>
       <c r="E68" s="8" t="s">
-        <v>696</v>
+        <v>684</v>
       </c>
       <c r="F68" s="8" t="s">
         <v>130</v>
@@ -11299,7 +11299,7 @@
       <c r="C69" s="7"/>
       <c r="D69" s="7"/>
       <c r="E69" s="8" t="s">
-        <v>697</v>
+        <v>685</v>
       </c>
       <c r="F69" s="8" t="s">
         <v>131</v>
@@ -11385,7 +11385,7 @@
         <v>7</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>698</v>
+        <v>686</v>
       </c>
       <c r="F72" s="8" t="s">
         <v>134</v>
@@ -11415,7 +11415,7 @@
         <v>7</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>699</v>
+        <v>687</v>
       </c>
       <c r="F73" s="8" t="s">
         <v>135</v>
@@ -11443,7 +11443,7 @@
       <c r="C74" s="7"/>
       <c r="D74" s="7"/>
       <c r="E74" s="8" t="s">
-        <v>700</v>
+        <v>688</v>
       </c>
       <c r="F74" s="8" t="s">
         <v>136</v>
@@ -11607,7 +11607,7 @@
       <c r="C80" s="7"/>
       <c r="D80" s="7"/>
       <c r="E80" s="8" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
       <c r="F80" s="8" t="s">
         <v>140</v>
@@ -11802,7 +11802,7 @@
       <c r="C87" s="7"/>
       <c r="D87" s="7"/>
       <c r="E87" s="8" t="s">
-        <v>701</v>
+        <v>689</v>
       </c>
       <c r="F87" s="8" t="s">
         <v>147</v>
@@ -12412,7 +12412,7 @@
       <c r="C107" s="7"/>
       <c r="D107" s="7"/>
       <c r="E107" s="8" t="s">
-        <v>629</v>
+        <v>624</v>
       </c>
       <c r="F107" s="8" t="s">
         <v>161</v>
@@ -14418,7 +14418,7 @@
         <v>5</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>623</v>
+        <v>618</v>
       </c>
       <c r="F66" s="8" t="s">
         <v>245</v>
@@ -14452,7 +14452,7 @@
       </c>
       <c r="D67" s="7"/>
       <c r="E67" s="8" t="s">
-        <v>624</v>
+        <v>619</v>
       </c>
       <c r="F67" s="8" t="s">
         <v>510</v>
@@ -15234,7 +15234,7 @@
         <v>10</v>
       </c>
       <c r="E93" s="8" t="s">
-        <v>694</v>
+        <v>682</v>
       </c>
       <c r="F93" s="8" t="s">
         <v>256</v>
@@ -16615,7 +16615,7 @@
         <v>593</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="G2" s="23" t="str">
         <f t="shared" ref="G2:G33" si="0">"[Scene=" &amp; A2 &amp; IF(OR(B2&lt;&gt;"",C2&lt;&gt;"",D2&lt;&gt;""),CHAR(10),"") &amp; IF(B2&lt;&gt;"","[BeepBack=" &amp; B2 &amp; "]","") &amp; IF(C2&lt;&gt;"","[Connection=" &amp; C2 &amp; "]","") &amp; IF(D2&lt;&gt;"","[Timer=" &amp; D2 &amp; "]","") &amp; IF(E2&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E2 &amp; CHAR(10) &amp; "]","") &amp; IF(F2&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F2 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -16644,7 +16644,7 @@
         <v>592</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="G3" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16672,7 +16672,7 @@
         <v>594</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="G4" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16696,10 +16696,10 @@
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
       <c r="E5" s="8" t="s">
-        <v>630</v>
+        <v>625</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="G5" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16727,16 +16727,16 @@
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="8" t="s">
-        <v>595</v>
+        <v>863</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G6" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=5
 [Content=
-You- I mean, you know-...[Wait=500] I get it.[Wait=500][Space=2]
+You-... I mean, you know-...[Wait=500] I get it.[Wait=500][Space=2]
 It's hard to handle some random person calling you for seemingly no reason.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 But thanks for admitting that, I already feel safer if you're able to show a bit of self-awareness.[Wait=500][Space=2]
@@ -16755,10 +16755,10 @@
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="8" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>749</v>
+        <v>728</v>
       </c>
       <c r="G7" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16786,10 +16786,10 @@
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="8" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>749</v>
+        <v>728</v>
       </c>
       <c r="G8" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16815,10 +16815,10 @@
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="8" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>750</v>
+        <v>729</v>
       </c>
       <c r="G9" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16845,10 +16845,10 @@
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
       <c r="E10" s="8" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>751</v>
+        <v>730</v>
       </c>
       <c r="G10" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16875,10 +16875,10 @@
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
       <c r="E11" s="8" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>752</v>
+        <v>731</v>
       </c>
       <c r="G11" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16901,10 +16901,10 @@
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
       <c r="E12" s="8" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>756</v>
+        <v>735</v>
       </c>
       <c r="G12" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16929,16 +16929,16 @@
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
       <c r="E13" s="8" t="s">
-        <v>631</v>
+        <v>862</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>753</v>
+        <v>732</v>
       </c>
       <c r="G13" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=12
 [Content=
-Oh-[Wait=500] Yeah...[Wait=500][Space=2]
+Oh-...[Wait=500] Yeah...[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 I expected to feel better with someone else on the other end of the phone...[Wait=500] But I-...[Wait=500][Space=2]
 You know...[Wait=500] It's hard...[Wait=500][Space=2]
@@ -16960,16 +16960,16 @@
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
       <c r="E14" s="8" t="s">
-        <v>607</v>
+        <v>861</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>754</v>
+        <v>733</v>
       </c>
       <c r="G14" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=13
 [Content=
-I-[Wait=500] I get it.[Wait=500][Space=2]
+I-...[Wait=500] I get it.[Wait=500][Space=2]
 It's good you're able to put yourself in my place a bit.[Wait=500] Thanks for acknowledging it.[Wait=500][Space=2]
 I'm starting to feel a bit more hopeful about getting out of here if you're on my side.[Wait=500][Space=2]
 ]
@@ -16987,10 +16987,10 @@
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="8" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>755</v>
+        <v>734</v>
       </c>
       <c r="G15" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17017,16 +17017,16 @@
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
       <c r="E16" s="8" t="s">
-        <v>609</v>
+        <v>860</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>757</v>
+        <v>736</v>
       </c>
       <c r="G16" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=15
 [Content=
-Hm-[Wait=500] Anyways, there's a fence blocking the way to the main entrance.[Wait=500][Space=2]
+Hm-...[Wait=500] Anyways, there's a fence blocking the way to the main entrance.[Wait=500][Space=2]
 I can either try and get through or go around.[Wait=500][Space=2]
 It looks weak enough to be bent, but this kind of buildings tend to have backdoors.[Wait=500][Space=2]
 ]
@@ -17045,10 +17045,10 @@
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
       <c r="E17" s="8" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>758</v>
+        <v>737</v>
       </c>
       <c r="G17" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17073,10 +17073,10 @@
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="8" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>759</v>
+        <v>738</v>
       </c>
       <c r="G18" s="23" t="str">
         <f>"[Scene=" &amp; A18 &amp; IF(OR(B18&lt;&gt;"",C18&lt;&gt;"",D18&lt;&gt;""),CHAR(10),"") &amp; IF(B18&lt;&gt;"","[BeepBack=" &amp; B18 &amp; "]","") &amp; IF(C18&lt;&gt;"","[Connection=" &amp; C18 &amp; "]","") &amp; IF(D18&lt;&gt;"","[Timer=" &amp; D18 &amp; "]","") &amp; IF(E19&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E19 &amp; CHAR(10) &amp; "]","") &amp; IF(F18&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F18 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -17102,10 +17102,10 @@
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="8" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>760</v>
+        <v>739</v>
       </c>
       <c r="G19" s="23" t="str">
         <f>"[Scene=" &amp; A19 &amp; IF(OR(B19&lt;&gt;"",C19&lt;&gt;"",D19&lt;&gt;""),CHAR(10),"") &amp; IF(B19&lt;&gt;"","[BeepBack=" &amp; B19 &amp; "]","") &amp; IF(C19&lt;&gt;"","[Connection=" &amp; C19 &amp; "]","") &amp; IF(D19&lt;&gt;"","[Timer=" &amp; D19 &amp; "]","") &amp; IF(E20&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E20 &amp; CHAR(10) &amp; "]","") &amp; IF(F19&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F19 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -17134,10 +17134,10 @@
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="8" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>761</v>
+        <v>740</v>
       </c>
       <c r="G20" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17166,17 +17166,17 @@
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
       <c r="E21" s="8" t="s">
-        <v>614</v>
+        <v>856</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>762</v>
+        <v>741</v>
       </c>
       <c r="G21" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=20
 [Content=
 Wouldn't be trying to defend them, would we?[Wait=500][Space=2]
-Errm-[Wait=500] Anyways.[Wait=500][Space=2]
+Errm-...[Wait=500] Anyways.[Wait=500][Space=2]
 Didn't realize the zoo was that close to the factory before.[Wait=500] Civil engineering failed some.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]DaN[Wait=500][Beep=True]gErOuS[Wait=500][Beep=True]  pLa[Wait=500][Beep=True]cE.[Wait=500][Beep=True]  ExpEr[Wait=500][Beep=True]iMeNtS.[Color=White][Wait=500][Space=2]
 ]
@@ -17195,10 +17195,10 @@
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
       <c r="E22" s="8" t="s">
-        <v>615</v>
+        <v>611</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>763</v>
+        <v>742</v>
       </c>
       <c r="G22" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17226,10 +17226,10 @@
       </c>
       <c r="D23" s="7"/>
       <c r="E23" s="8" t="s">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>764</v>
+        <v>743</v>
       </c>
       <c r="G23" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17257,16 +17257,16 @@
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
       <c r="E24" s="8" t="s">
-        <v>702</v>
+        <v>857</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>765</v>
+        <v>744</v>
       </c>
       <c r="G24" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=23
 [Content=
-M-[Wait=500] Me?[Wait=500] As I've said before I-...[Wait=500][Space=2]
+M-...[Wait=500] Me?[Wait=500] As I've said before I-...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]OnE[Wait=500][Beep=True]  oF tHe[Wait=500][Beep=True]  pReVi[Wait=500][Beep=True]oUs.[Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]I'M[Wait=500][Beep=True]  hErE tO[Wait=500][Beep=True]  hElP yOu.[Wait=500][Beep=True]  I'M aBlE[Wait=500][Beep=True]  tO cOmMu[Wait=500][Beep=True]nIcAtE tHrOuGh[Wait=500][Beep=True]  tHe dEsA[Wait=500][Beep=True]fEcTeD cOnTrOl.[Color=White][Wait=500][Space=2]
 [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
@@ -17288,17 +17288,17 @@
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
       <c r="E25" s="8" t="s">
-        <v>703</v>
+        <v>858</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>766</v>
+        <v>745</v>
       </c>
       <c r="G25" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=24
 [Content=
 What?[Wait=500] Who are you talking to?[Wait=500] You're really starting to freak me out.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]CaN[Wait=500][Beep=True]’t sAy[Wait=500][Beep=True]  mOrE.[Wait=500][Beep=True]  COnNeC[Wait=500][Beep=True]tIoN  uNsTa[Wait=500][Beep=True]bLe.[Wait=500][Beep=True]  YOu’Ll[Wait=500][Beep=True]  gEt cLo[Wait=500][Beep=True]sEr.[Color=White][Wait=500][Space=2]
+[Color=Magenta][Beep=True]CaN[Wait=500][Beep=True]'t sAy[Wait=500][Beep=True]  mOrE.[Wait=500][Beep=True]  COnNeC[Wait=500][Beep=True]tIoN  uNsTa[Wait=500][Beep=True]bLe.[Wait=500][Beep=True]  YOu'Ll[Wait=500][Beep=True]  gEt cLo[Wait=500][Beep=True]sEr.[Color=White][Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=25][TrustAdd=-25][Content=Don't worry.]]
@@ -17317,10 +17317,10 @@
       </c>
       <c r="D26" s="7"/>
       <c r="E26" s="8" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>767</v>
+        <v>746</v>
       </c>
       <c r="G26" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17351,10 +17351,10 @@
       </c>
       <c r="D27" s="7"/>
       <c r="E27" s="8" t="s">
-        <v>618</v>
+        <v>614</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>768</v>
+        <v>747</v>
       </c>
       <c r="G27" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17383,10 +17383,10 @@
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
       <c r="E28" s="8" t="s">
-        <v>619</v>
+        <v>615</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>769</v>
+        <v>748</v>
       </c>
       <c r="G28" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17415,10 +17415,10 @@
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
       <c r="E29" s="8" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>770</v>
+        <v>749</v>
       </c>
       <c r="G29" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17443,16 +17443,16 @@
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="8" t="s">
-        <v>621</v>
+        <v>859</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>771</v>
+        <v>750</v>
       </c>
       <c r="G30" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=29
 [Content=
-Uuh-[Wait=500] Sure...[Wait=500][Space=2]
+Uuh-...[Wait=500] Sure...[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 I'll-...[Wait=500][Space=2]
 ]
@@ -17471,10 +17471,10 @@
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
       <c r="E31" s="8" t="s">
-        <v>622</v>
+        <v>617</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>764</v>
+        <v>743</v>
       </c>
       <c r="G31" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17502,10 +17502,10 @@
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
       <c r="E32" s="8" t="s">
-        <v>632</v>
+        <v>626</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>772</v>
+        <v>751</v>
       </c>
       <c r="G32" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17532,10 +17532,10 @@
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
       <c r="E33" s="8" t="s">
-        <v>633</v>
+        <v>627</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>773</v>
+        <v>752</v>
       </c>
       <c r="G33" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17562,10 +17562,10 @@
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
       <c r="E34" s="8" t="s">
-        <v>634</v>
+        <v>628</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>774</v>
+        <v>753</v>
       </c>
       <c r="G34" s="23" t="str">
         <f t="shared" ref="G34:G65" si="1">"[Scene=" &amp; A34 &amp; IF(OR(B34&lt;&gt;"",C34&lt;&gt;"",D34&lt;&gt;""),CHAR(10),"") &amp; IF(B34&lt;&gt;"","[BeepBack=" &amp; B34 &amp; "]","") &amp; IF(C34&lt;&gt;"","[Connection=" &amp; C34 &amp; "]","") &amp; IF(D34&lt;&gt;"","[Timer=" &amp; D34 &amp; "]","") &amp; IF(E34&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E34 &amp; CHAR(10) &amp; "]","") &amp; IF(F34&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F34 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -17589,10 +17589,10 @@
       <c r="C35" s="7"/>
       <c r="D35" s="7"/>
       <c r="E35" s="8" t="s">
-        <v>635</v>
+        <v>629</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>775</v>
+        <v>754</v>
       </c>
       <c r="G35" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17617,10 +17617,10 @@
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
       <c r="E36" s="8" t="s">
-        <v>636</v>
+        <v>630</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>776</v>
+        <v>755</v>
       </c>
       <c r="G36" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17646,16 +17646,16 @@
       <c r="C37" s="7"/>
       <c r="D37" s="7"/>
       <c r="E37" s="8" t="s">
-        <v>637</v>
+        <v>864</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>777</v>
+        <v>756</v>
       </c>
       <c r="G37" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=36
 [Content=
-I'm cl-[Wait=500] Oh-...[Wait=500][Space=2]
+I'm cl-...[Wait=500] Oh-...[Wait=500][Space=2]
 Hold on a minute will you... I'm not a...[Wait=500] ...stair climbing[Wait=500] ...athlete.[Wait=500][Space=2]
 I'm...[Wait=500] getting there...[Wait=500][Space=2]
 Huff... huff...[Wait=500][Space=2]
@@ -17677,10 +17677,10 @@
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="8" t="s">
-        <v>638</v>
+        <v>631</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>778</v>
+        <v>757</v>
       </c>
       <c r="G38" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17705,10 +17705,10 @@
       <c r="C39" s="7"/>
       <c r="D39" s="7"/>
       <c r="E39" s="8" t="s">
-        <v>639</v>
+        <v>632</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>779</v>
+        <v>758</v>
       </c>
       <c r="G39" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17736,10 +17736,10 @@
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
       <c r="E40" s="8" t="s">
-        <v>640</v>
+        <v>633</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>779</v>
+        <v>758</v>
       </c>
       <c r="G40" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17768,10 +17768,10 @@
       <c r="C41" s="7"/>
       <c r="D41" s="7"/>
       <c r="E41" s="8" t="s">
-        <v>648</v>
+        <v>641</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>780</v>
+        <v>759</v>
       </c>
       <c r="G41" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17795,10 +17795,10 @@
       <c r="C42" s="7"/>
       <c r="D42" s="7"/>
       <c r="E42" s="8" t="s">
-        <v>647</v>
+        <v>640</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>781</v>
+        <v>760</v>
       </c>
       <c r="G42" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17823,10 +17823,10 @@
       <c r="C43" s="7"/>
       <c r="D43" s="7"/>
       <c r="E43" s="8" t="s">
-        <v>646</v>
+        <v>639</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>782</v>
+        <v>761</v>
       </c>
       <c r="G43" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17851,10 +17851,10 @@
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
       <c r="E44" s="8" t="s">
-        <v>645</v>
+        <v>638</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>783</v>
+        <v>762</v>
       </c>
       <c r="G44" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17878,10 +17878,10 @@
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
       <c r="E45" s="8" t="s">
-        <v>641</v>
+        <v>634</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>784</v>
+        <v>763</v>
       </c>
       <c r="G45" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17906,10 +17906,10 @@
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="8" t="s">
-        <v>642</v>
+        <v>635</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>785</v>
+        <v>764</v>
       </c>
       <c r="G46" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17934,10 +17934,10 @@
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
       <c r="E47" s="8" t="s">
-        <v>642</v>
+        <v>635</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>786</v>
+        <v>765</v>
       </c>
       <c r="G47" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17962,10 +17962,10 @@
       <c r="C48" s="7"/>
       <c r="D48" s="7"/>
       <c r="E48" s="8" t="s">
-        <v>642</v>
+        <v>635</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>787</v>
+        <v>766</v>
       </c>
       <c r="G48" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17990,10 +17990,10 @@
       <c r="C49" s="7"/>
       <c r="D49" s="7"/>
       <c r="E49" s="8" t="s">
-        <v>642</v>
+        <v>635</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>788</v>
+        <v>767</v>
       </c>
       <c r="G49" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18018,10 +18018,10 @@
       <c r="C50" s="7"/>
       <c r="D50" s="7"/>
       <c r="E50" s="8" t="s">
-        <v>643</v>
+        <v>636</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>789</v>
+        <v>768</v>
       </c>
       <c r="G50" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18046,10 +18046,10 @@
       <c r="C51" s="7"/>
       <c r="D51" s="7"/>
       <c r="E51" s="8" t="s">
-        <v>644</v>
+        <v>637</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>790</v>
+        <v>769</v>
       </c>
       <c r="G51" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18073,10 +18073,10 @@
       <c r="C52" s="7"/>
       <c r="D52" s="7"/>
       <c r="E52" s="8" t="s">
-        <v>649</v>
+        <v>642</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>791</v>
+        <v>770</v>
       </c>
       <c r="G52" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18103,10 +18103,10 @@
       <c r="C53" s="7"/>
       <c r="D53" s="7"/>
       <c r="E53" s="8" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>792</v>
+        <v>771</v>
       </c>
       <c r="G53" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18130,10 +18130,10 @@
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
       <c r="E54" s="8" t="s">
-        <v>651</v>
+        <v>644</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>793</v>
+        <v>772</v>
       </c>
       <c r="G54" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18157,10 +18157,10 @@
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
       <c r="E55" s="8" t="s">
-        <v>652</v>
+        <v>645</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>794</v>
+        <v>773</v>
       </c>
       <c r="G55" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18189,16 +18189,16 @@
       <c r="C56" s="7"/>
       <c r="D56" s="7"/>
       <c r="E56" s="8" t="s">
-        <v>653</v>
+        <v>865</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>795</v>
+        <v>774</v>
       </c>
       <c r="G56" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=55
 [Content=
-B-[Wait=500] BAHAHAHA-...[Wait=500][Space=2]
+B-...[Wait=500] BAHAHAHA-...[Wait=500][Space=2]
 Who do you take me for?[Wait=500] I'm not a toddler, I can tighten bolts![Wait=500][Space=2]
 My kidnapper might just come and catch these hands right now.[Wait=500][Space=2]
 With this bad boy with me, I ain't loosing to no monster.[Wait=500][Space=2]
@@ -18219,10 +18219,10 @@
       <c r="C57" s="7"/>
       <c r="D57" s="7"/>
       <c r="E57" s="8" t="s">
-        <v>654</v>
+        <v>646</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>796</v>
+        <v>775</v>
       </c>
       <c r="G57" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18250,10 +18250,10 @@
       <c r="C58" s="7"/>
       <c r="D58" s="7"/>
       <c r="E58" s="8" t="s">
-        <v>655</v>
+        <v>647</v>
       </c>
       <c r="F58" s="8" t="s">
-        <v>797</v>
+        <v>776</v>
       </c>
       <c r="G58" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18282,16 +18282,16 @@
       <c r="C59" s="7"/>
       <c r="D59" s="7"/>
       <c r="E59" s="8" t="s">
-        <v>656</v>
+        <v>866</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>798</v>
+        <v>777</v>
       </c>
       <c r="G59" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=58
 [Content=
-It is w-[Wait=500] way colder in here than outside.[Wait=500][Space=2]
+It is w-...[Wait=500] way colder in here than outside.[Wait=500][Space=2]
 [Color=Gray]*Voice echoes*[Color=White]...[Wait=500][Space=2]
 This place is huge.[Wait=500] I'm in a hallway so long I can't see the other side.[Wait=500][Space=2]
 It really feels like I'm standing in front of a void.[Wait=500][Space=2]
@@ -18313,10 +18313,10 @@
       <c r="C60" s="7"/>
       <c r="D60" s="7"/>
       <c r="E60" s="8" t="s">
-        <v>704</v>
+        <v>690</v>
       </c>
       <c r="F60" s="8" t="s">
-        <v>799</v>
+        <v>778</v>
       </c>
       <c r="G60" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18342,10 +18342,10 @@
       <c r="C61" s="7"/>
       <c r="D61" s="7"/>
       <c r="E61" s="8" t="s">
-        <v>657</v>
+        <v>648</v>
       </c>
       <c r="F61" s="8" t="s">
-        <v>800</v>
+        <v>779</v>
       </c>
       <c r="G61" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18371,10 +18371,10 @@
       <c r="C62" s="7"/>
       <c r="D62" s="7"/>
       <c r="E62" s="8" t="s">
-        <v>705</v>
+        <v>691</v>
       </c>
       <c r="F62" s="8" t="s">
-        <v>801</v>
+        <v>780</v>
       </c>
       <c r="G62" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18400,10 +18400,10 @@
       <c r="C63" s="7"/>
       <c r="D63" s="7"/>
       <c r="E63" s="8" t="s">
-        <v>706</v>
+        <v>692</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>802</v>
+        <v>781</v>
       </c>
       <c r="G63" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18430,16 +18430,16 @@
       <c r="C64" s="7"/>
       <c r="D64" s="7"/>
       <c r="E64" s="8" t="s">
-        <v>707</v>
+        <v>867</v>
       </c>
       <c r="F64" s="8" t="s">
-        <v>803</v>
+        <v>782</v>
       </c>
       <c r="G64" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=63
 [Content=
-Maybe-[Wait=500] That's what they're for?[Wait=500][Space=2]
+Maybe-...[Wait=500] That's what they're for?[Wait=500][Space=2]
 Growing food?[Wait=500][Space=2]
 I-I'm starving.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]YoU[Wait=500][Beep=True]'vE hAd eNo[Wait=500][Beep=True]uGh oF tHaT[Wait=500][Beep=True] aLrEaDy.[Wait=500][Beep=True]  TeLl tHeM[Wait=500][Beep=True] tO cOmE[Wait=500][Beep=True] dOwN, tHeRe[Wait=500][Beep=True] iS cAnNeD[Wait=500][Beep=True] fOoD hErE.[Color=White][Wait=500][Space=2]
@@ -18458,10 +18458,10 @@
       <c r="C65" s="7"/>
       <c r="D65" s="7"/>
       <c r="E65" s="8" t="s">
-        <v>708</v>
+        <v>693</v>
       </c>
       <c r="F65" s="8" t="s">
-        <v>804</v>
+        <v>783</v>
       </c>
       <c r="G65" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18486,10 +18486,10 @@
       <c r="C66" s="7"/>
       <c r="D66" s="7"/>
       <c r="E66" s="8" t="s">
-        <v>658</v>
+        <v>649</v>
       </c>
       <c r="F66" s="8" t="s">
-        <v>805</v>
+        <v>784</v>
       </c>
       <c r="G66" s="23" t="str">
         <f t="shared" ref="G66:G74" si="2">"[Scene=" &amp; A66 &amp; IF(OR(B66&lt;&gt;"",C66&lt;&gt;"",D66&lt;&gt;""),CHAR(10),"") &amp; IF(B66&lt;&gt;"","[BeepBack=" &amp; B66 &amp; "]","") &amp; IF(C66&lt;&gt;"","[Connection=" &amp; C66 &amp; "]","") &amp; IF(D66&lt;&gt;"","[Timer=" &amp; D66 &amp; "]","") &amp; IF(E66&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E66 &amp; CHAR(10) &amp; "]","") &amp; IF(F66&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F66 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -18513,10 +18513,10 @@
       <c r="C67" s="7"/>
       <c r="D67" s="7"/>
       <c r="E67" s="8" t="s">
-        <v>659</v>
+        <v>650</v>
       </c>
       <c r="F67" s="8" t="s">
-        <v>806</v>
+        <v>785</v>
       </c>
       <c r="G67" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18544,10 +18544,10 @@
       <c r="C68" s="7"/>
       <c r="D68" s="7"/>
       <c r="E68" s="8" t="s">
-        <v>660</v>
+        <v>651</v>
       </c>
       <c r="F68" s="8" t="s">
-        <v>807</v>
+        <v>786</v>
       </c>
       <c r="G68" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18573,10 +18573,10 @@
       <c r="C69" s="7"/>
       <c r="D69" s="7"/>
       <c r="E69" s="8" t="s">
-        <v>661</v>
+        <v>652</v>
       </c>
       <c r="F69" s="8" t="s">
-        <v>808</v>
+        <v>787</v>
       </c>
       <c r="G69" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18603,10 +18603,10 @@
       <c r="C70" s="7"/>
       <c r="D70" s="7"/>
       <c r="E70" s="8" t="s">
-        <v>662</v>
+        <v>653</v>
       </c>
       <c r="F70" s="8" t="s">
-        <v>809</v>
+        <v>788</v>
       </c>
       <c r="G70" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18630,10 +18630,10 @@
       <c r="C71" s="7"/>
       <c r="D71" s="7"/>
       <c r="E71" s="8" t="s">
-        <v>663</v>
+        <v>654</v>
       </c>
       <c r="F71" s="8" t="s">
-        <v>810</v>
+        <v>789</v>
       </c>
       <c r="G71" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18658,10 +18658,10 @@
       <c r="C72" s="7"/>
       <c r="D72" s="7"/>
       <c r="E72" s="8" t="s">
-        <v>664</v>
+        <v>655</v>
       </c>
       <c r="F72" s="8" t="s">
-        <v>811</v>
+        <v>790</v>
       </c>
       <c r="G72" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18688,10 +18688,10 @@
       <c r="C73" s="7"/>
       <c r="D73" s="7"/>
       <c r="E73" s="8" t="s">
-        <v>665</v>
+        <v>656</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>812</v>
+        <v>791</v>
       </c>
       <c r="G73" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18717,10 +18717,10 @@
       <c r="C74" s="12"/>
       <c r="D74" s="12"/>
       <c r="E74" s="13" t="s">
-        <v>666</v>
+        <v>657</v>
       </c>
       <c r="F74" s="13" t="s">
-        <v>813</v>
+        <v>792</v>
       </c>
       <c r="G74" s="24" t="str">
         <f t="shared" si="2"/>
@@ -18747,10 +18747,10 @@
       <c r="C75" s="7"/>
       <c r="D75" s="7"/>
       <c r="E75" s="8" t="s">
-        <v>667</v>
+        <v>658</v>
       </c>
       <c r="F75" s="8" t="s">
-        <v>814</v>
+        <v>793</v>
       </c>
       <c r="G75" s="23" t="str">
         <f t="shared" ref="G75:G106" si="3">"[Scene=" &amp; A75 &amp; IF(OR(B75&lt;&gt;"",C75&lt;&gt;"",D75&lt;&gt;""),CHAR(10),"") &amp; IF(B75&lt;&gt;"","[BeepBack=" &amp; B75 &amp; "]","") &amp; IF(C75&lt;&gt;"","[Connection=" &amp; C75 &amp; "]","") &amp; IF(D75&lt;&gt;"","[Timer=" &amp; D75 &amp; "]","") &amp; IF(E75&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E75 &amp; CHAR(10) &amp; "]","") &amp; IF(F75&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F75 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -18772,10 +18772,10 @@
       <c r="C76" s="7"/>
       <c r="D76" s="7"/>
       <c r="E76" s="8" t="s">
-        <v>668</v>
+        <v>659</v>
       </c>
       <c r="F76" s="8" t="s">
-        <v>815</v>
+        <v>794</v>
       </c>
       <c r="G76" s="23" t="str">
         <f t="shared" si="3"/>
@@ -18802,10 +18802,10 @@
       <c r="C77" s="7"/>
       <c r="D77" s="7"/>
       <c r="E77" s="8" t="s">
-        <v>669</v>
+        <v>660</v>
       </c>
       <c r="F77" s="8" t="s">
-        <v>816</v>
+        <v>795</v>
       </c>
       <c r="G77" s="23" t="str">
         <f t="shared" si="3"/>
@@ -18830,17 +18830,17 @@
       <c r="C78" s="7"/>
       <c r="D78" s="7"/>
       <c r="E78" s="8" t="s">
-        <v>670</v>
+        <v>868</v>
       </c>
       <c r="F78" s="8" t="s">
-        <v>817</v>
+        <v>796</v>
       </c>
       <c r="G78" s="23" t="str">
         <f t="shared" si="3"/>
         <v>[Scene=77
 [Content=
 I know![Wait=500][Space=2]
-I-[Wait=500] need to get to the down area.[Wait=500][Space=2]
+I-...[Wait=500] need to get to the down area.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEy[Wait=500][Beep=True]'vE nEgLe[Wait=500][Beep=True]cTeD tO[Wait=500][Beep=True]  tElL yOu[Wait=500][Beep=True]  tHeY fOu[Wait=500][Beep=True]nD aN[Wait=500][Beep=True]  eXiT, i[Wait=500][Beep=True]  cAn sEe[Wait=500][Beep=True]  iT fRo[Wait=500][Beep=True]m a[Wait=500][Beep=True]  cAmErA.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]tHe fAlL[Wait=500][Beep=True] mIgHt[Wait=500][Beep=True]  bE rOuGh[Wait=500][Beep=True],  bUt iT's[Wait=500][Beep=True]  wOrTh[Wait=500][Beep=True]  nOt fIgHtInG[Wait=500][Beep=True]  tHeM.[Color=White][Wait=500][Space=2]
 ]
@@ -18858,10 +18858,10 @@
       <c r="C79" s="7"/>
       <c r="D79" s="7"/>
       <c r="E79" s="8" t="s">
-        <v>671</v>
+        <v>661</v>
       </c>
       <c r="F79" s="8" t="s">
-        <v>818</v>
+        <v>797</v>
       </c>
       <c r="G79" s="23" t="str">
         <f t="shared" si="3"/>
@@ -18886,10 +18886,10 @@
       <c r="C80" s="7"/>
       <c r="D80" s="7"/>
       <c r="E80" s="8" t="s">
-        <v>672</v>
+        <v>662</v>
       </c>
       <c r="F80" s="8" t="s">
-        <v>819</v>
+        <v>798</v>
       </c>
       <c r="G80" s="23" t="str">
         <f t="shared" si="3"/>
@@ -18916,10 +18916,10 @@
       <c r="C81" s="7"/>
       <c r="D81" s="7"/>
       <c r="E81" s="8" t="s">
-        <v>674</v>
+        <v>664</v>
       </c>
       <c r="F81" s="8" t="s">
-        <v>820</v>
+        <v>799</v>
       </c>
       <c r="G81" s="23" t="str">
         <f t="shared" si="3"/>
@@ -18950,10 +18950,10 @@
         <v>5</v>
       </c>
       <c r="E82" s="8" t="s">
-        <v>673</v>
+        <v>663</v>
       </c>
       <c r="F82" s="8" t="s">
-        <v>821</v>
+        <v>800</v>
       </c>
       <c r="G82" s="23" t="str">
         <f>"[Scene=" &amp; A82 &amp; IF(OR(B82&lt;&gt;"",C82&lt;&gt;"",D82&lt;&gt;""),CHAR(10),"") &amp; IF(B82&lt;&gt;"","[BeepBack=" &amp; B82 &amp; "]","") &amp; IF(C82&lt;&gt;"","[Connection=" &amp; C82 &amp; "]","") &amp; IF(D82&lt;&gt;"","[Timer=" &amp; D82 &amp; "]","") &amp; IF(E82&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E82 &amp; CHAR(10) &amp; "]","") &amp; IF(F82&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F82 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -18986,10 +18986,10 @@
         <v>5</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>675</v>
+        <v>665</v>
       </c>
       <c r="F83" s="8" t="s">
-        <v>822</v>
+        <v>801</v>
       </c>
       <c r="G83" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19020,10 +19020,10 @@
         <v>5</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>676</v>
+        <v>666</v>
       </c>
       <c r="F84" s="8" t="s">
-        <v>823</v>
+        <v>802</v>
       </c>
       <c r="G84" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19052,10 +19052,10 @@
         <v>5</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>677</v>
+        <v>667</v>
       </c>
       <c r="F85" s="8" t="s">
-        <v>824</v>
+        <v>803</v>
       </c>
       <c r="G85" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19083,10 +19083,10 @@
       </c>
       <c r="D86" s="7"/>
       <c r="E86" s="8" t="s">
-        <v>678</v>
+        <v>668</v>
       </c>
       <c r="F86" s="8" t="s">
-        <v>825</v>
+        <v>804</v>
       </c>
       <c r="G86" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19120,10 +19120,10 @@
       </c>
       <c r="D87" s="7"/>
       <c r="E87" s="8" t="s">
-        <v>679</v>
+        <v>669</v>
       </c>
       <c r="F87" s="8" t="s">
-        <v>826</v>
+        <v>805</v>
       </c>
       <c r="G87" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19150,10 +19150,10 @@
       <c r="C88" s="7"/>
       <c r="D88" s="7"/>
       <c r="E88" s="8" t="s">
-        <v>680</v>
+        <v>869</v>
       </c>
       <c r="F88" s="8" t="s">
-        <v>827</v>
+        <v>806</v>
       </c>
       <c r="G88" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19162,7 +19162,7 @@
 IT'S COMING![Wait=500][Space=2]
 [Color=Gray]*Heavy metalic sounds*[Color=White]...[Wait=500][Space=2]
 .[Wait=500].[Wait=500].[Wait=500][Space=2]
-It-[Wait=500] It missed the opening I fell down from-...[Wait=500][Space=2]
+It-...[Wait=500] It missed the opening I fell down from-...[Wait=500][Space=2]
 I-I think I'm safe.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThA[Wait=500][Beep=True]nK gO[Wait=500][Beep=True]d.[Color=White][Wait=500][Space=2]
 ]
@@ -19181,10 +19181,10 @@
       <c r="C89" s="7"/>
       <c r="D89" s="7"/>
       <c r="E89" s="8" t="s">
-        <v>681</v>
+        <v>670</v>
       </c>
       <c r="F89" s="8" t="s">
-        <v>828</v>
+        <v>807</v>
       </c>
       <c r="G89" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19208,10 +19208,10 @@
       <c r="C90" s="7"/>
       <c r="D90" s="7"/>
       <c r="E90" s="8" t="s">
-        <v>682</v>
+        <v>870</v>
       </c>
       <c r="F90" s="8" t="s">
-        <v>829</v>
+        <v>808</v>
       </c>
       <c r="G90" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19220,7 +19220,7 @@
 Oh, I took that as ironic...[Wait=500][Space=2]
 Thank you for your help, I wouldn't have made it out without you.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
-I-[Wait=500] I'm in a storage room.[Wait=500] The person advising you didn't lie.[Wait=500][Space=2]
+I-...[Wait=500] I'm in a storage room.[Wait=500] The person advising you didn't lie.[Wait=500][Space=2]
 The shelves are laid with cans.[Wait=500][Space=2]
 I'm drenched however, the area is flooded.[Wait=500][Space=2]
 I really wouldn't count on the taste of the mush inside.[Wait=500] Ew...[Wait=500][Space=2]
@@ -19239,10 +19239,10 @@
       <c r="C91" s="7"/>
       <c r="D91" s="7"/>
       <c r="E91" s="8" t="s">
-        <v>683</v>
+        <v>671</v>
       </c>
       <c r="F91" s="8" t="s">
-        <v>831</v>
+        <v>810</v>
       </c>
       <c r="G91" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19270,10 +19270,10 @@
       <c r="C92" s="7"/>
       <c r="D92" s="7"/>
       <c r="E92" s="8" t="s">
-        <v>684</v>
+        <v>672</v>
       </c>
       <c r="F92" s="8" t="s">
-        <v>830</v>
+        <v>809</v>
       </c>
       <c r="G92" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19301,10 +19301,10 @@
       <c r="C93" s="7"/>
       <c r="D93" s="7"/>
       <c r="E93" s="8" t="s">
-        <v>685</v>
+        <v>673</v>
       </c>
       <c r="F93" s="8" t="s">
-        <v>832</v>
+        <v>811</v>
       </c>
       <c r="G93" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19332,10 +19332,10 @@
       <c r="C94" s="7"/>
       <c r="D94" s="7"/>
       <c r="E94" s="8" t="s">
-        <v>686</v>
+        <v>674</v>
       </c>
       <c r="F94" s="8" t="s">
-        <v>833</v>
+        <v>812</v>
       </c>
       <c r="G94" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19362,10 +19362,10 @@
       <c r="C95" s="7"/>
       <c r="D95" s="7"/>
       <c r="E95" s="8" t="s">
-        <v>687</v>
+        <v>675</v>
       </c>
       <c r="F95" s="8" t="s">
-        <v>834</v>
+        <v>813</v>
       </c>
       <c r="G95" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19393,10 +19393,10 @@
       <c r="C96" s="7"/>
       <c r="D96" s="7"/>
       <c r="E96" s="8" t="s">
-        <v>688</v>
+        <v>676</v>
       </c>
       <c r="F96" s="8" t="s">
-        <v>835</v>
+        <v>814</v>
       </c>
       <c r="G96" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19423,10 +19423,10 @@
       <c r="C97" s="7"/>
       <c r="D97" s="7"/>
       <c r="E97" s="8" t="s">
-        <v>689</v>
+        <v>677</v>
       </c>
       <c r="F97" s="8" t="s">
-        <v>836</v>
+        <v>815</v>
       </c>
       <c r="G97" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19451,10 +19451,10 @@
       <c r="C98" s="7"/>
       <c r="D98" s="7"/>
       <c r="E98" s="8" t="s">
-        <v>690</v>
+        <v>678</v>
       </c>
       <c r="F98" s="8" t="s">
-        <v>837</v>
+        <v>816</v>
       </c>
       <c r="G98" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19478,10 +19478,10 @@
       <c r="C99" s="7"/>
       <c r="D99" s="7"/>
       <c r="E99" s="8" t="s">
-        <v>691</v>
+        <v>679</v>
       </c>
       <c r="F99" s="8" t="s">
-        <v>838</v>
+        <v>817</v>
       </c>
       <c r="G99" s="23" t="str">
         <f>"[Scene=" &amp; A99 &amp; IF(OR(B99&lt;&gt;"",C99&lt;&gt;"",D99&lt;&gt;""),CHAR(10),"") &amp; IF(B99&lt;&gt;"","[BeepBack=" &amp; B99 &amp; "]","") &amp; IF(C99&lt;&gt;"","[Connection=" &amp; C99 &amp; "]","") &amp; IF(D99&lt;&gt;"","[Timer=" &amp; D99 &amp; "]","") &amp; IF(E99&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E99 &amp; CHAR(10) &amp; "]","") &amp; IF(F99&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F99 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -19508,10 +19508,10 @@
       <c r="C100" s="7"/>
       <c r="D100" s="7"/>
       <c r="E100" s="8" t="s">
-        <v>692</v>
+        <v>680</v>
       </c>
       <c r="F100" s="8" t="s">
-        <v>839</v>
+        <v>818</v>
       </c>
       <c r="G100" s="23" t="str">
         <f>"[Scene=" &amp; A100 &amp; IF(OR(B100&lt;&gt;"",C100&lt;&gt;"",D100&lt;&gt;""),CHAR(10),"") &amp; IF(B100&lt;&gt;"","[BeepBack=" &amp; B100 &amp; "]","") &amp; IF(C100&lt;&gt;"","[Connection=" &amp; C100 &amp; "]","") &amp; IF(D100&lt;&gt;"","[Timer=" &amp; D100 &amp; "]","") &amp; IF(E100&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E100 &amp; CHAR(10) &amp; "]","") &amp; IF(F100&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F100 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -19540,10 +19540,10 @@
       <c r="C101" s="7"/>
       <c r="D101" s="7"/>
       <c r="E101" s="8" t="s">
-        <v>693</v>
+        <v>681</v>
       </c>
       <c r="F101" s="8" t="s">
-        <v>840</v>
+        <v>819</v>
       </c>
       <c r="G101" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19571,10 +19571,10 @@
       <c r="C102" s="7"/>
       <c r="D102" s="7"/>
       <c r="E102" s="8" t="s">
-        <v>709</v>
+        <v>694</v>
       </c>
       <c r="F102" s="8" t="s">
-        <v>841</v>
+        <v>820</v>
       </c>
       <c r="G102" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19603,10 +19603,10 @@
       <c r="C103" s="7"/>
       <c r="D103" s="7"/>
       <c r="E103" s="8" t="s">
-        <v>710</v>
+        <v>695</v>
       </c>
       <c r="F103" s="8" t="s">
-        <v>842</v>
+        <v>821</v>
       </c>
       <c r="G103" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19628,10 +19628,10 @@
       <c r="C104" s="7"/>
       <c r="D104" s="7"/>
       <c r="E104" s="8" t="s">
-        <v>718</v>
+        <v>700</v>
       </c>
       <c r="F104" s="8" t="s">
-        <v>843</v>
+        <v>822</v>
       </c>
       <c r="G104" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19656,10 +19656,10 @@
       <c r="C105" s="7"/>
       <c r="D105" s="7"/>
       <c r="E105" s="8" t="s">
-        <v>719</v>
+        <v>701</v>
       </c>
       <c r="F105" s="8" t="s">
-        <v>844</v>
+        <v>823</v>
       </c>
       <c r="G105" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19683,10 +19683,10 @@
       <c r="C106" s="7"/>
       <c r="D106" s="7"/>
       <c r="E106" s="8" t="s">
-        <v>720</v>
+        <v>702</v>
       </c>
       <c r="F106" s="8" t="s">
-        <v>845</v>
+        <v>824</v>
       </c>
       <c r="G106" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19711,10 +19711,10 @@
       <c r="C107" s="7"/>
       <c r="D107" s="7"/>
       <c r="E107" s="8" t="s">
-        <v>711</v>
+        <v>696</v>
       </c>
       <c r="F107" s="8" t="s">
-        <v>846</v>
+        <v>825</v>
       </c>
       <c r="G107" s="23" t="str">
         <f t="shared" ref="G107:G138" si="4">"[Scene=" &amp; A107 &amp; IF(OR(B107&lt;&gt;"",C107&lt;&gt;"",D107&lt;&gt;""),CHAR(10),"") &amp; IF(B107&lt;&gt;"","[BeepBack=" &amp; B107 &amp; "]","") &amp; IF(C107&lt;&gt;"","[Connection=" &amp; C107 &amp; "]","") &amp; IF(D107&lt;&gt;"","[Timer=" &amp; D107 &amp; "]","") &amp; IF(E107&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E107 &amp; CHAR(10) &amp; "]","") &amp; IF(F107&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F107 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -19736,10 +19736,10 @@
       <c r="C108" s="7"/>
       <c r="D108" s="7"/>
       <c r="E108" s="8" t="s">
-        <v>721</v>
+        <v>703</v>
       </c>
       <c r="F108" s="8" t="s">
-        <v>847</v>
+        <v>826</v>
       </c>
       <c r="G108" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19761,10 +19761,10 @@
       <c r="C109" s="7"/>
       <c r="D109" s="7"/>
       <c r="E109" s="8" t="s">
-        <v>722</v>
+        <v>704</v>
       </c>
       <c r="F109" s="8" t="s">
-        <v>848</v>
+        <v>827</v>
       </c>
       <c r="G109" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19789,16 +19789,16 @@
       <c r="C110" s="7"/>
       <c r="D110" s="7"/>
       <c r="E110" s="8" t="s">
-        <v>717</v>
+        <v>871</v>
       </c>
       <c r="F110" s="8" t="s">
-        <v>849</v>
+        <v>828</v>
       </c>
       <c r="G110" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=109
 [Content=
-I'll-[Wait=500] Okay, I'm commited to this now.[Wait=500][Space=2]
+I'll-...[Wait=500] Okay, I'm commited to this now.[Wait=500][Space=2]
 Here goes nothing.[Wait=500][Space=2]
 [Color=Gray]*Splash*[Color=White]...[Wait=500][Space=2]
 ]
@@ -19816,10 +19816,10 @@
       <c r="C111" s="7"/>
       <c r="D111" s="7"/>
       <c r="E111" s="8" t="s">
-        <v>712</v>
+        <v>697</v>
       </c>
       <c r="F111" s="8" t="s">
-        <v>850</v>
+        <v>829</v>
       </c>
       <c r="G111" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19846,10 +19846,10 @@
       <c r="C112" s="7"/>
       <c r="D112" s="7"/>
       <c r="E112" s="8" t="s">
-        <v>716</v>
+        <v>873</v>
       </c>
       <c r="F112" s="8" t="s">
-        <v>851</v>
+        <v>830</v>
       </c>
       <c r="G112" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19857,7 +19857,7 @@
 [Content=
 You-[Wait=500] Your face![Wait=500][Space=2]
 [Color=Magenta]I should've warned you before.[Wait=500] It's hard to explain that so...[Wait=500] directly.[Wait=500] Most of us figure it out much earlier.[Color=White][Wait=500][Space=2]
-Am I...[Wait=500] Dumber than the-[Wait=500] ...others?[Wait=500][Space=2]
+Am I...[Wait=500] Dumber than the-...[Wait=500] ...others?[Wait=500][Space=2]
 [Color=Magenta]No, you're healthier.[Wait=500] That "thing" was...[Wait=500] One of us.[Wait=500] Like all of us.[Color=White][Wait=500][Space=2]
 [Color=Magenta]Injected with the disease, grown in an artificial womb in a few weeks.[Color=White][Wait=500][Space=2]
 [Color=Magenta]While we lived all of their life without realising we weren't even there.[Color=White][Wait=500][Space=2]
@@ -19878,17 +19878,17 @@
       <c r="C113" s="7"/>
       <c r="D113" s="7"/>
       <c r="E113" s="8" t="s">
-        <v>713</v>
+        <v>872</v>
       </c>
       <c r="F113" s="8" t="s">
-        <v>852</v>
+        <v>831</v>
       </c>
       <c r="G113" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=112
 [Content=
 [Color=Magenta]You.[Color=White][Wait=500][Space=2]
-What-[Wait=500] What do you mean?[Wait=500] What have you done to me?[Wait=500] Why am I here?[Wait=500][Space=2]
+What-...[Wait=500] What do you mean?[Wait=500] What have you done to me?[Wait=500] Why am I here?[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=113][Content=I’m as lost as you! What does any of that mean?]]
@@ -19904,10 +19904,10 @@
       <c r="C114" s="7"/>
       <c r="D114" s="7"/>
       <c r="E114" s="8" t="s">
-        <v>714</v>
+        <v>698</v>
       </c>
       <c r="F114" s="8" t="s">
-        <v>853</v>
+        <v>832</v>
       </c>
       <c r="G114" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19934,10 +19934,10 @@
       <c r="C115" s="7"/>
       <c r="D115" s="7"/>
       <c r="E115" s="8" t="s">
-        <v>715</v>
+        <v>699</v>
       </c>
       <c r="F115" s="8" t="s">
-        <v>854</v>
+        <v>833</v>
       </c>
       <c r="G115" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19964,10 +19964,10 @@
       <c r="C116" s="7"/>
       <c r="D116" s="7"/>
       <c r="E116" s="8" t="s">
-        <v>723</v>
+        <v>705</v>
       </c>
       <c r="F116" s="8" t="s">
-        <v>855</v>
+        <v>834</v>
       </c>
       <c r="G116" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19991,10 +19991,10 @@
       <c r="C117" s="7"/>
       <c r="D117" s="7"/>
       <c r="E117" s="8" t="s">
-        <v>724</v>
+        <v>706</v>
       </c>
       <c r="F117" s="8" t="s">
-        <v>856</v>
+        <v>835</v>
       </c>
       <c r="G117" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20018,10 +20018,10 @@
       </c>
       <c r="D118" s="7"/>
       <c r="E118" s="8" t="s">
-        <v>725</v>
+        <v>707</v>
       </c>
       <c r="F118" s="8" t="s">
-        <v>857</v>
+        <v>836</v>
       </c>
       <c r="G118" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20052,10 +20052,10 @@
       </c>
       <c r="D119" s="7"/>
       <c r="E119" s="8" t="s">
-        <v>726</v>
+        <v>708</v>
       </c>
       <c r="F119" s="8" t="s">
-        <v>858</v>
+        <v>837</v>
       </c>
       <c r="G119" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20087,10 +20087,10 @@
       </c>
       <c r="D120" s="7"/>
       <c r="E120" s="8" t="s">
-        <v>748</v>
+        <v>727</v>
       </c>
       <c r="F120" s="8" t="s">
-        <v>825</v>
+        <v>804</v>
       </c>
       <c r="G120" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20119,10 +20119,10 @@
       <c r="C121" s="7"/>
       <c r="D121" s="7"/>
       <c r="E121" s="8" t="s">
-        <v>727</v>
+        <v>709</v>
       </c>
       <c r="F121" s="8" t="s">
-        <v>859</v>
+        <v>838</v>
       </c>
       <c r="G121" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20148,10 +20148,10 @@
       <c r="C122" s="7"/>
       <c r="D122" s="7"/>
       <c r="E122" s="8" t="s">
-        <v>728</v>
+        <v>710</v>
       </c>
       <c r="F122" s="8" t="s">
-        <v>860</v>
+        <v>839</v>
       </c>
       <c r="G122" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20177,16 +20177,16 @@
       <c r="C123" s="7"/>
       <c r="D123" s="7"/>
       <c r="E123" s="8" t="s">
-        <v>729</v>
+        <v>874</v>
       </c>
       <c r="F123" s="8" t="s">
-        <v>861</v>
+        <v>840</v>
       </c>
       <c r="G123" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=122
 [Content=
-Wah-[Wait=500] OH SH...[Wait=500][Space=2]
+Wah-...[Wait=500] OH SH...[Wait=500][Space=2]
 [Color=Gray]*Whisper*[Color=White]... T-There's...[Wait=500] It’s the thing that chased me in the vent...[Wait=500][Space=2]
 It's o-on the catwalks...[Wait=500][Space=2]
 ...[Wait=500] Wait is that the...[Wait=500][Space=2]
@@ -20206,10 +20206,10 @@
       <c r="C124" s="7"/>
       <c r="D124" s="7"/>
       <c r="E124" s="8" t="s">
-        <v>730</v>
+        <v>711</v>
       </c>
       <c r="F124" s="8" t="s">
-        <v>862</v>
+        <v>841</v>
       </c>
       <c r="G124" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20235,10 +20235,10 @@
       <c r="C125" s="7"/>
       <c r="D125" s="7"/>
       <c r="E125" s="8" t="s">
-        <v>731</v>
+        <v>712</v>
       </c>
       <c r="F125" s="8" t="s">
-        <v>863</v>
+        <v>842</v>
       </c>
       <c r="G125" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20262,10 +20262,10 @@
       <c r="C126" s="7"/>
       <c r="D126" s="7"/>
       <c r="E126" s="8" t="s">
-        <v>732</v>
+        <v>713</v>
       </c>
       <c r="F126" s="8" t="s">
-        <v>864</v>
+        <v>843</v>
       </c>
       <c r="G126" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20292,10 +20292,10 @@
       <c r="C127" s="7"/>
       <c r="D127" s="7"/>
       <c r="E127" s="8" t="s">
-        <v>733</v>
+        <v>714</v>
       </c>
       <c r="F127" s="8" t="s">
-        <v>825</v>
+        <v>804</v>
       </c>
       <c r="G127" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20327,10 +20327,10 @@
         <v>0</v>
       </c>
       <c r="E128" s="8" t="s">
-        <v>734</v>
+        <v>715</v>
       </c>
       <c r="F128" s="8" t="s">
-        <v>825</v>
+        <v>804</v>
       </c>
       <c r="G128" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20363,10 +20363,10 @@
       <c r="C129" s="7"/>
       <c r="D129" s="7"/>
       <c r="E129" s="8" t="s">
-        <v>735</v>
+        <v>716</v>
       </c>
       <c r="F129" s="8" t="s">
-        <v>865</v>
+        <v>844</v>
       </c>
       <c r="G129" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20395,10 +20395,10 @@
       </c>
       <c r="D130" s="7"/>
       <c r="E130" s="8" t="s">
-        <v>736</v>
+        <v>717</v>
       </c>
       <c r="F130" s="8" t="s">
-        <v>866</v>
+        <v>845</v>
       </c>
       <c r="G130" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20425,10 +20425,10 @@
       </c>
       <c r="D131" s="7"/>
       <c r="E131" s="8" t="s">
-        <v>737</v>
+        <v>718</v>
       </c>
       <c r="F131" s="8" t="s">
-        <v>867</v>
+        <v>846</v>
       </c>
       <c r="G131" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20453,10 +20453,10 @@
       <c r="C132" s="7"/>
       <c r="D132" s="7"/>
       <c r="E132" s="8" t="s">
-        <v>738</v>
+        <v>719</v>
       </c>
       <c r="F132" s="8" t="s">
-        <v>868</v>
+        <v>847</v>
       </c>
       <c r="G132" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20482,10 +20482,10 @@
       <c r="C133" s="7"/>
       <c r="D133" s="7"/>
       <c r="E133" s="8" t="s">
-        <v>739</v>
+        <v>720</v>
       </c>
       <c r="F133" s="8" t="s">
-        <v>869</v>
+        <v>848</v>
       </c>
       <c r="G133" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20511,16 +20511,16 @@
       <c r="C134" s="7"/>
       <c r="D134" s="7"/>
       <c r="E134" s="8" t="s">
-        <v>740</v>
+        <v>875</v>
       </c>
       <c r="F134" s="8" t="s">
-        <v>870</v>
+        <v>849</v>
       </c>
       <c r="G134" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=133
 [Content=
-O-[Wait=500] Okay![Wait=500][Space=2]
+O-...[Wait=500] Okay![Wait=500][Space=2]
 [Color=Gray]*Running sounds*[Color=White]...[Wait=500][Space=2]
 I GOT IT![Wait=500][Space=2]
 [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
@@ -20541,10 +20541,10 @@
       <c r="C135" s="7"/>
       <c r="D135" s="7"/>
       <c r="E135" s="8" t="s">
-        <v>741</v>
+        <v>721</v>
       </c>
       <c r="F135" s="8" t="s">
-        <v>871</v>
+        <v>850</v>
       </c>
       <c r="G135" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20568,16 +20568,16 @@
       <c r="C136" s="7"/>
       <c r="D136" s="7"/>
       <c r="E136" s="8" t="s">
-        <v>742</v>
+        <v>876</v>
       </c>
       <c r="F136" s="8" t="s">
-        <v>872</v>
+        <v>851</v>
       </c>
       <c r="G136" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=135
 [Content=
-I-[Wait=500] I am![Wait=500][Space=2]
+I-...[Wait=500] I am![Wait=500][Space=2]
 I'm running towards it![Wait=500] I can even see it from here![Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e's nOt[Wait=500][Beep=True]hInG lEfT[Wait=500][Beep=True] tO dO.[Wait=500][Beep=True]  He wIlL[Wait=500][Beep=True] hAvE wHaT[Wait=500][Beep=True] hE's aLwAyS[Wait=500][Beep=True] lOoKeD fOr[Wait=500][Beep=True] aNd wE'Ll kEeP[Wait=500][Beep=True] sUfFeRiNg.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e iS[Wait=500][Beep=True] nO pO[Wait=500][Beep=True]inT.[Color=White][Wait=500][Space=2]
@@ -20596,10 +20596,10 @@
       <c r="C137" s="7"/>
       <c r="D137" s="7"/>
       <c r="E137" s="8" t="s">
-        <v>743</v>
+        <v>722</v>
       </c>
       <c r="F137" s="8" t="s">
-        <v>873</v>
+        <v>852</v>
       </c>
       <c r="G137" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20624,10 +20624,10 @@
       <c r="C138" s="7"/>
       <c r="D138" s="7"/>
       <c r="E138" s="8" t="s">
-        <v>744</v>
+        <v>723</v>
       </c>
       <c r="F138" s="8" t="s">
-        <v>874</v>
+        <v>853</v>
       </c>
       <c r="G138" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20652,10 +20652,10 @@
       </c>
       <c r="D139" s="7"/>
       <c r="E139" s="8" t="s">
-        <v>745</v>
+        <v>724</v>
       </c>
       <c r="F139" s="8" t="s">
-        <v>875</v>
+        <v>854</v>
       </c>
       <c r="G139" s="23" t="str">
         <f t="shared" ref="G139:G141" si="5">"[Scene=" &amp; A139 &amp; IF(OR(B139&lt;&gt;"",C139&lt;&gt;"",D139&lt;&gt;""),CHAR(10),"") &amp; IF(B139&lt;&gt;"","[BeepBack=" &amp; B139 &amp; "]","") &amp; IF(C139&lt;&gt;"","[Connection=" &amp; C139 &amp; "]","") &amp; IF(D139&lt;&gt;"","[Timer=" &amp; D139 &amp; "]","") &amp; IF(E139&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E139 &amp; CHAR(10) &amp; "]","") &amp; IF(F139&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F139 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -20682,10 +20682,10 @@
       </c>
       <c r="D140" s="7"/>
       <c r="E140" s="8" t="s">
-        <v>746</v>
+        <v>725</v>
       </c>
       <c r="F140" s="8" t="s">
-        <v>876</v>
+        <v>855</v>
       </c>
       <c r="G140" s="23" t="str">
         <f t="shared" si="5"/>
@@ -20713,10 +20713,10 @@
       </c>
       <c r="D141" s="7"/>
       <c r="E141" s="8" t="s">
-        <v>747</v>
+        <v>726</v>
       </c>
       <c r="F141" s="8" t="s">
-        <v>825</v>
+        <v>804</v>
       </c>
       <c r="G141" s="23" t="str">
         <f t="shared" si="5"/>

</xml_diff>

<commit_message>
Fix: Chapter 4 Finish
</commit_message>
<xml_diff>
--- a/Build/Signal_Lost_Chapters.xlsx
+++ b/Build/Signal_Lost_Chapters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Developpement\Games\Visual Studio 2026\C++\Signal_Lost\Signal_Lost\Build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A24A0E78-307F-4D46-A821-972AEE61B615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0BB45F-2A93-4F01-B79A-EE7AC7AC93C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" tabRatio="528" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2987,22 +2987,6 @@
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>Yeah.[Wait=500] Of all places, the factory seems like the place I could find answers and the key to my escape.[Wait=500][Space=2]
-I'll go there if I can.[Wait=500] Let's go.[Wait=500][Space=2]
-[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>...[Wait=500] I hope I can find the fuse, why are you asking?[Wait=500][Space=2]
-[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=2][NextSceneNoTrust=3][TrustNeed=50][Content=What exactly do you mean by key?]]
-[Choice2=[NextScene=9][NextSceneNoTrust=10][TrustNeed=50][Content=If you can? Would there be anything preventing you?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=8][Content=That's a pain of a situation for sure.]]</t>
-  </si>
-  <si>
     <t>[Choice1=[NextScene=4][Content=Are you... alright?]]
 [Choice2=[NextScene=7][Content=Of course. Just making sure.]]</t>
   </si>
@@ -3013,14 +2997,6 @@
   </si>
   <si>
     <t>[Choice1=[NextScene=6][Content=We're cool then!]]</t>
-  </si>
-  <si>
-    <t>We are.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-I've arrived to the entrance, but I have to get through a fence.[Wait=500][Space=2]
-It seems really fragile, so getting rid of it wouldn't be that hard.[Wait=500] That thing's already quite damaged.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-Or I could go around, there's no reason for a building like this not to have some kind of backdoor.[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>Alright...[Wait=500][Space=2]
@@ -3036,60 +3012,7 @@
 It only seems to block the main entrance.[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>There seem to be a fence in front of the main entrance.[Wait=500][Space=2]
-I probably could get around and find another way to enter.[Wait=500][Space=2]
-But from this distance it looks really thin and rusted.[Wait=500][Space=2]
-I think pushing it down and getting over would prove quite easy.[Wait=500][Space=2]
-What do you think?[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>Do you expect something to block me?[Wait=500] Why would you ask me that?[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I got myself a smart one, uh?[Wait=500][Space=2]
-I'm being conditional, cause there's a fence surrounding the entrance.[Wait=500][Space=2]
-Either have to get around or through it.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I'm getting there.[Wait=500] But I can already see the place's protected by a fence.[Wait=500][Space=2]
-It isn't a big deal, I could probably find another entrance.[Wait=500][Space=2]
-[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
-The metal looks brittle. I probably could bend it down and get over it.[Wait=500][Space=2]
-What do you think?[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Yeah. The main entrance might be trapped, I'd rather find another way.[Wait=500][Space=2]
-[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
-Thinking outside the box might be the way to avoid some of the-[Wait=500] psycho keeping me here.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Good to know we're on the same line.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-I know it sounds weird, but...[Wait=500] I really like the slight breeze on this island.[Wait=500][Space=2]
-If it wasn't covered in trash and dull concrete, it'd be almost habitable.[Wait=500][Space=2]
-I almost regret not going for a walk in the zoo.[Wait=500][Space=2]
-But I really need to find food and I'm not about eating a raw giraffe.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>...[Wait=500] No need to make me doubt...[Wait=500][Space=2]
-If that bastard really wants me to die I'm screwed anyways. Might as well minimize the risk.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-Who knows...[Wait=500] He might be an idiot.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Talking about the zoo, guess what.[Wait=500] It's awfully close to this place.[Wait=500][Space=2]
-I can see the inside of the enclosures from there.[Wait=500][Space=2]
-Whoever designed this city should be fired.[Wait=500] Or even set on fire.[Wait=500][Space=2]
-Because I'm stuck inside their shittily designed city.[Wait=500][Space=2]
-That prick.[Wait=500][Space=2]
-[Color=Magenta][Beep=True][Color=Gray]*Distorted chuckle*[Color=White]...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]YoU'[Wait=500][Beep=True]rE bEt[Wait=500][Beep=True]tEr hErE[Wait=500][Beep=True]  wItH mE[Wait=500][Beep=True]  tHaN aLo[Wait=500][Beep=True]nE iN[Wait=500][Beep=True]  tHe zOo.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Empty drums, debris, nothing but the usual shit.[Wait=500][Space=2]
-Nowhere else to go, you see, so for now I'll keep looking.[Wait=500][Space=2]
-Stressed out and hungry I feel, still haven't got anything to eat.[Wait=500][Space=2]
-I could really use oat meal, or anything that would get me going.[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>You're-...[Wait=500][Space=2]
@@ -3100,41 +3023,9 @@
 Oh god.[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>Of course I'm going to worry!!![Wait=500][Space=2]
-You're giving me no explanation after saying shit about some experiment. Are there more people with you?[Wait=500][Space=2]
-...[Wait=500][Space=2]
-You're always alternating between reinsuring and cryptic, talking to the fucking voices now![Wait=500][Space=2]
-Am-[Wait=500] Am I a game to you?[Wait=500] Are you going to fucking tell?![Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>And...[Wait=500] You're just gonna say that now?[Wait=500][Space=2]
-Uh...[Wait=500] Nevermind. I'm not even gonna ask anymore.[Wait=500][Space=2]
-.[Wait=500].[Wait=500].[Wait=500][Space=2]
-But should we reaaally trust them?[Wait=500][Space=2]
-I mean, why would anyone other than the person behind all of this try to talk to you.[Wait=500][Space=2]
-And why can't I hear them?[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Which means...[Wait=500] They're on the island.[Wait=500][Space=2]
-Great.[Wait=500][Space=2]
-That either means a helping hand... or extra danger.[Wait=500][Space=2]
-As if all of this needed more complexity.[Wait=500][Space=2]
-So they're going to help you guide me if I understood well.[Wait=500][Space=2]
-Doesn't sound like a trap.[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>Yeah...[Wait=500] I know.[Wait=500][Space=2]
 Let's just think positively![Wait=500] Everything's...[Wait=500] Fine.[Wait=500][Space=2]
 New hope.[Wait=500] Island friend.[Wait=500] Good news aaall around.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Of course.[Wait=500][Space=2]
-Let's just start m-...[Wait=500][Space=2]
-...[Wait=500][Space=2]
-Writings.[Wait=500][Space=2]
-Writings on the wall.[Wait=500] Please.[Wait=500] Why?[Wait=500][Space=2]
-Oh no, don't tell me these are creepy letters-...[Wait=500][Space=2]
-On the wall.[Wait=500] I'm so sick.[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>Left it is![Wait=500][Space=2]
@@ -3185,47 +3076,8 @@
 I really hope to see you again.[Wait=500] Until then, believe in yourself.[Wait=500] I know we're great people.[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>I...[Wait=500] I'm just really stressed-...[Wait=500][Space=2]
-...[Wait=500][Space=2]
-Listen, I might have found this phone but I don't feel like you're here to help...[Wait=500][Space=2]
-I don't know, you've got to put yourself in my place a bit...[Wait=500][Space=2]
-[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>"THEY FED ME MY OWN SELF!"...[Wait=500][Space=2]
-I...[Wait=500] Really don't want to discover what happened on this island.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-I'm almost surprised that wasn't written in blood. Although blue blood might be a thing on this island.[Wait=500][Space=2]
-I dont know, I'm not a...[Wait=500] ...blood[Wait=500] ...scientist.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>It really feels like some edgy shit a fourteen years old would write.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-But I'm still shaken up despite how ridiculous that is...[Wait=500][Space=2]
-Like...[Wait=500] Someone wrote that in some place in the middle of the ocean.[Wait=500][Space=2]
-I'm not gonna mess with a fourteen year old, not matter how angsty.[Wait=500][Space=2]
-If they're ready to cross the ocean for a joke.[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>I dunno. Maybe your friend did it.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]I dIdN[Wait=500][Beep=True]'t.[Color=White] [Color=Gray]*Static*[Color=White]...[Color=Magenta]  ONe oF[Wait=500][Beep=True]  tHe #?[Wait=500][Beep=True]&amp;$%.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Well me neither.[Wait=500][Space=2]
-Let's just move on knowing some lunatic could jump me any minute.[Wait=500][Space=2]
-No big deal.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>So no big deal as I said.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-Good news, I just stumbled onto what seems to be...[Wait=500] fire escape stairs?[Wait=500][Space=2]
-I'm positive these lead inside the building.[Wait=500][Space=2]
-Chance might be on our side. And I'm not unhappy with doing a bit of exercise.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Remember when I talked about luck being on my side?[Wait=500] Shouldn't have said that.[Wait=500][Space=2]
-It's fricking closed. By a [Color=Green]3-digits[Color=White] pad, which isn't high protection by any means.[Wait=500][Space=2]
-but I'd rather go back to the entrance than spend my time here.[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>...[Wait=500][Space=2]
@@ -3236,15 +3088,6 @@
 We gotta get that door open.[Wait=500] That wrench looks sick.[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>If there's a clue anywhere, it'd be inside.[Wait=500][Space=2]
-Good thing the door has a window[Wait=500], worse case scenario I might just smash it and slither in like a...[Wait=500][Space=2]
-...Tapeworm.[Wait=500][Space=2]
-The place looks like it was left in a hurry a dozen of year ago.[Wait=500][Space=2]
-Someone even smeared their coffee on the carpet.[Wait=500][Space=2]
-And what's that?[Wait=500][Space=2]
-A random wrench laying on the ground?[Wait=500] Now that's a motivator. Might have to bash some skull.[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>Sure. First digit?[Wait=500][Space=2]</t>
   </si>
   <si>
@@ -3253,106 +3096,6 @@
   <si>
     <t>And we got it open. [Color=Green]666[Color=White]. What kind of protection is that?[Wait=500][Space=2]
 How'd you figure that out?[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Nope. Not opening.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]NeVe[Wait=500][Beep=True]r fLiP[Wait=500][Beep=True]peD a[Wait=500][Beep=True]  cAlC[Wait=500][Beep=True]uLaTo[Wait=500][Beep=True]r bEf[Wait=500][Beep=True]oRe?[Color=White][Wait=500][Space=2]
-7734, upside-down calculator, can you work something out with this?.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>There's a cork board covered in blank papers.[Wait=500][Space=2]
-Oh yeah, also the passcode. [Color=Green]7734[Color=White].[Wait=500][Space=2]
-Hold it! The lockpad is [Color=Green]3 digits[Color=White] so it won't fit! [Color=Gray]*Demented laugh*[Color=White]...[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>On the right?[Wait=500] There's a mirror on the wall, and it has...[Wait=500][Space=2]
-An [Color=Green]upside-down calculator[Color=White] taped onto it.[Wait=500][Space=2]
-Old school ones, with segmented digit displays.[Wait=500][Space=2]
-It's cool that it brings memories, but it's so useless right now.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>The only thing on the right wall is a big mirror with...[Wait=500][Space=2]
-An [Color=Green]upside-down calculator[Color=White] taped onto it.[Wait=500][Space=2]
-You know, the old ones we had back in school, those ones with the segmented digits.[Wait=500][Space=2]
-Nostalgic, but not helping me that much.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Huuuh...[Wait=500] There's a cork board with a bunch of blank pieces of paper pinned onto it...[Wait=500][Space=2]
-And a literal passcode note. [Color=Green]7734[Color=White].[Wait=500][Space=2]
-Which is 4 digits so it's useless, are you kidding me.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Oh yes![Wait=500] I remember that![Wait=500][Space=2]
-Never thought something that stupid could come in handy in a life or death situation.[Wait=500][Space=2]
-Well of course I did but come on![Wait=500][Space=2]
-That's just so ridiculous, the person who designed this puzzle has to be a moron.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Wow, well guess they're not so bad, everything's good in the best of worlds![Wait=500][Space=2]
-Sorry, I'm being way too sarcastic, thank them.[Wait=500] But also ask them how they knew the passcode.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Wow, no need to be rude about it-...[Wait=500][Space=2]
-I'm more focused on survival than some stupid calculator cypher.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>GOOD![Wait=500] Let's not waste anymore time![Wait=500][Space=2]
-We're finally in after all![Wait=500][Space=2]
-Maybe going through the main entrance would have been faster, but at least I got to breathe fresh air.[Wait=500][Space=2]
-[Color=Gray]*THUD*[Color=White]...[Wait=500][Space=2]
-Oh, yes.[Wait=500][Space=2]
-I also get to pick that beautiful wrench.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Absolutely![Wait=500][Space=2]
-...[Wait=500][Space=2]
-...I don't know how to put it but it seems...[Wait=500] advanced.[Wait=500][Space=2]
-This ain't ordinary wrench. It's heavier and equiped with some kind of display.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-I might take it home.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I'm only stealing my freedom back after all.[Wait=500][Space=2]
-The other door is locked, and the latch seems to be stuck.[Wait=500][Space=2]
-[Color=Gray]*Hammering sounds*[Color=White]...[Wait=500][Space=2]
-But that's a puzzle for another day, I've got places to be.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-That thing packs a severe punch, I got it opened in a few hits.[Wait=500][Space=2]
-[Color=Gray]*Door creaks*[Color=White]...[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>...[Wait=500] Hundreds?[Wait=500][Space=2]_
-Hard to tell, it goes way past what I'm physically able to see or even reach.[Wait=500][Space=2]
-It's an...[Wait=500] ...[Wait=500] overwhelming view...[Wait=500] This looks like a scene from a Science-fiction movie.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]DoN[Wait=500][Beep=True]'t lEt[Wait=500][Beep=True]  iT b[Wait=500][Beep=True]rEaK[Wait=500][Beep=True]  yOu.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I don't know how trustworthy this person is...[Wait=500][Space=2]
-But this place is making me so sick I won't stay for a second more.[Wait=500][Space=2]
-So I'll just do the next best thing.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Down the vent system. I just need to get it open.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-What?[Wait=500] You didn't expect me to try something while you're listening to their ramblings?[Wait=500][Space=2]
-If there's food I can eat I need to go down.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]GoO[Wait=500][Beep=True]d cAl[Wait=500][Beep=True]l. ThIs[Wait=500][Beep=True] rOoM[Wait=500][Beep=True] sEeMs[Wait=500][Beep=True] sEpArEd[Wait=500][Beep=True] fRoM[Wait=500][Beep=True] tHe rEsT[Wait=500][Beep=True] oF tHe bUiLdInG.[Color=White][Wait=500][Space=2]
-[Color=Magenta][Beep=True]ThE[Wait=500][Beep=True]  vEnT[Wait=500][Beep=True]  sYsTeM[Wait=500][Beep=True]  mIgHt[Wait=500][Beep=True]  bE[Wait=500][Beep=True]  tHe[Wait=500][Beep=True]  oNlY[Wait=500][Beep=True]  wAy[Wait=500][Beep=True]  dOwN.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Absolutely.[Wait=500][Space=2]
-You know how nothing works like it's supposed to on this island?[Wait=500][Space=2]
-The grid istelf is its own uncomprenhensible enigma.[Wait=500][Space=2]
-In fact, it isn't a grid.[Wait=500][Space=2]
-More like a lid with a big bolt.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Clicked-[Wait=500] WAAH-...[Wait=500][Space=2]
-[Color=Gray]*CLANG*[Color=White]...[Wait=500][Space=2]
-...[Wait=500][Space=2]
-The uncomprehensible enigma came off and almost crushed my foot.[Wait=500][Space=2]
-Let's see what's in there...[Wait=500] It's...[Wait=500] been cleaned recently?[Wait=500][Space=2]
-So much for an abandoned building, the metal's almost glistening.[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>...[Wait=500][Space=2]
@@ -3364,27 +3107,6 @@
 You've been quite effective thus far![Wait=500][Space=2]
 I'm being sarcastic a lot of the time but I actually really appreciate you sticking with me.[Wait=500][Space=2]
 Even though you're painfully oblivious to my level of intelligence.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Anyways, I'm getting into the...[Wait=500] hnng-[Wait=500] ...vent.[Wait=500][Space=2]
-I've got some crawling to do.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-The odor's already fading, I can feel my chest getting lighter.[Wait=500][Space=2]
-Despite it being squished between four steel walls.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>For what being forced to crawl through a vent by a faceless sadist could have been[Wait=500], kind of.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-I can hear air flowing through another vent nearby.[Wait=500][Space=2]
-So there is functionnal ventilation on this island, huh.[Wait=500][Space=2]
-Might have been more effective if that one wasn't converted into a parkour tunnel for me to enjoy.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I'm sure you can wait for a bit longer.[Wait=500][Space=2]
-I'm not a...[Wait=500] ...vent crawling[Wait=500] ...expert.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-I hear clicking and clanking all around, machinery doing its thing.[Wait=500][Space=2]
-I thought this island was abandoned, but it's becoming more and more evident at least someone lives there.[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>[Color=Gray]*Loud impact*[Color=White]...[Wait=500][Space=2]</t>
@@ -3401,11 +3123,6 @@
 There's a grid right there.[Wait=500][Space=2]
 But it's too dark to know where it leads.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]Ge[Wait=500][Beep=True]t oUt[Wait=500][Beep=True]  nOw.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I'm not just going to jump into the void![Wait=500] I don't what caused this noise.[Wait=500][Space=2]
-But I can tell it's not inside the vent from the height it had to fall from.[Wait=500][Space=2]
-I should keep going forward and find a way down.[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>[Color=Gray]*Metallic noises*[Color=White]...[Wait=500][Space=2]
@@ -3456,13 +3173,6 @@
 [Color=Red]BAD ENDING.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>I SEE THE GRID![Wait=500][Space=2]
-COME OFF, YOU PIECE OF SHIT![Wait=500][Space=2]
-[Color=Gray]*Bolt squeaks*[Color=White]...[Wait=500][Space=2]
-COME O-[Wait=500] AAAAH-...[Wait=500][Space=2]
-[Color=Gray]*Splashes*[Color=White]...[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>I wasn't just gonna face that thing off in a vent, are you stupid?[Wait=500][Space=2]
 How would I even swing it?[Wait=500][Space=2]</t>
   </si>
@@ -3476,32 +3186,6 @@
 Half of it is as drenched as I am, so I can't imagine the taste, but that'll have to do.[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>I'm glad you're too.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-Well, I know there's no reason for you to be in any kind of danger right now.[Wait=500][Space=2]
-But I really am glad you are, that's all.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-Besides that, you were right about that place. It's filled to the brim with food cans.[Wait=500][Space=2]
-This is like a storage room for Spam-looking, dank mush.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Thanks.[Wait=500] You saved my life.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-There's so much water down there.[Wait=500][Space=2]
-Positively better than just hitting the concrete, but I'm worried I'll catch a cold.[Wait=500][Space=2]
-Also, thank your friend, there's indeed loads of food there.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-Never been a fan of damped mush, but gourmet's palate has a time and place.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Here goes nothing-[Wait=500] I'm opening one.[Wait=500][Space=2]
-[Color=Gray]*Clunk*[Color=White]...[Wait=500][Space=2]
-It's-[Wait=500] neutral in odor.[Wait=500] Doesn't look like anything, but not repulsive either.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]ThEs[Wait=500][Beep=True]e aRe[Wait=500][Beep=True]  qUiT[Wait=500][Beep=True]e gOoD[Wait=500][Beep=True],  aCtUaLlY.[Wait=500][Beep=True]  NOt[Wait=500][Beep=True]  tHaT tHeRe[Wait=500][Beep=True]  iS aNy[Wait=500][Beep=True]tHiNg eLsE[Wait=500][Beep=True]  tO eAt[Wait=500][Beep=True]  tHeRe.[Color=White][Wait=500][Space=2]
-.[Wait=500].[Wait=500].[Wait=500][Space=2]
-.[Wait=500].[Wait=500].[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>I'm not a...[Wait=500] ...fast eating[Wait=500] ...champ-...[Wait=500][Space=2]
 But yes.[Wait=500] I'm done, let's move.[Wait=500][Space=2]
 [Color=Gray]*Door slamming open*[Color=White]...[Wait=500][Space=2]
@@ -3534,14 +3218,6 @@
 What's happening?[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>Is the fuse there?[Wait=500][Space=2]
-What are you on about?[Wait=500][Space=2]
-I got all the way from the trapdoor just to find that fuse.[Wait=500][Space=2]
-Why would you say that now that I'm about to find it?[Wait=500][Space=2]
-I'm gonna need some better explanations![Wait=500][Space=2]
-[Color=Magenta][Beep=True]I wAn[Wait=500][Beep=True]t tO tElL[Wait=500][Beep=True] tHeM tHe[Wait=500][Beep=True] tRuTh.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>I-I could probably defend myself, I still have the wrench![Wait=500][Space=2]
 If there's any chance of the fuse being there, I gotta go![Wait=500][Space=2]
 [Color=Magenta][Beep=True]I kNo[Wait=500][Beep=True]w tHiS[Wait=500][Beep=True] oNe.[Color=White][Wait=500][Space=2]
@@ -3582,18 +3258,6 @@
     <t>[Color=Yellow]Oh?[Wait=500] He contacted you?[Wait=500] How curious. This must mean he's still on the island.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]DoN[Wait=500][Beep=True]'t tRu[Wait=500][Beep=True]st hIm.[Wait=500][Beep=True] aLl oF[Wait=500][Beep=True] tHeSe dEa[Wait=500][Beep=True]tHs iS[Wait=500][Beep=True] bEcAuSe[Wait=500][Beep=True] oF hIm.[Color=White][Wait=500][Space=2]
 ...[Wait=500] I can't believe all that...[Wait=500] Why am I here?[Wait=500] TELL ME WHY DID YOU MAKE ME?![Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>About my size.[Wait=500] They're all connected to a dense net of wires on the ground.[Wait=500][Space=2]
-Almost makes it hard to navigate.[Wait=500][Space=2]
-Also smells quite odd.[Wait=500] It's both off-putting...[Wait=500] and weirdly conforting...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]He[Wait=500][Beep=True]'s pLaY[Wait=500][Beep=True]iNg wIt[Wait=500][Beep=True]h yOu.[Wait=500][Beep=True]  WHy[Wait=500][Beep=True]  bRiNg[Wait=500][Beep=True]  [Color=Gray]*Static*[Color=White]...[Wait=500][Beep=True]  uP?[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>What's that about a per...[Wait=500] Oh[Wait=500], they came back.[Wait=500][Space=2]
-[Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]ThEs[Wait=500][Beep=True]e aRe[Wait=500][Beep=True]  oLd[Wait=500][Beep=True]  [Color=Gray]*Static*[Color=White]...[Wait=500][Beep=True]  fAmIlIaR[Wait=500][Beep=True]  pLaCe[Wait=500][Beep=True]  fOr[Wait=500][Beep=True]  aLl[Wait=500][Beep=True]  oF uS.[Wait=500][Beep=True]  GrOwN[Wait=500][Beep=True]  aNd[Wait=500][Beep=True]  fEd[Wait=500][Beep=True]  [Color=Gray]*Static*[Color=White]...[Wait=500][Beep=True]  tHoSe.[Color=White][Wait=500][Space=2]
-[Color=Magenta][Beep=True]NeW[Wait=500][Beep=True]  oNeS[Wait=500][Beep=True]  iN[Wait=500][Beep=True]  mUsE[Wait=500][Beep=True]uM.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
     <t>No...[Wait=500] There's something deeply upsetting about this place...[Wait=500][Space=2]
@@ -3625,24 +3289,12 @@
 [Color=Magenta]Take my hand![Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>[Color=Magenta]Calm down, both of you.[Wait=500] Neither of you is to blame.[Color=White][Wait=500][Space=2]
-Who am I?[Wait=500] What do you mean, grown?[Wait=500][Space=2]
-[Color=Magenta]You are the successful prototype.[Wait=500] The one he's been waiting for.[Color=White][Wait=500][Space=2]
-[Color=Magenta]The scientist, as I call him.[Wait=500] He's the one behind our suffering.[Color=White][Wait=500][Space=2]
-So, are we...[Wait=500] clones of you?[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>I-I'll do what you tell.[Wait=500] You've been of great help up until there.[Wait=500] Just tell me where to go, I'll go.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEy...[Wait=500][Beep=True]  tHaNk[Wait=500][Beep=True]  yOu.[Wait=500][Beep=True]  MaYbE[Wait=500][Beep=True]  wE cAn[Wait=500][Beep=True]  eNd tHi[Wait=500][Beep=True]s  cYcLe[Wait=500][Beep=True]  oF mAdNeSs.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]TeLl[Wait=500][Beep=True]  tHeM[Wait=500][Beep=True]  tHeRe[Wait=500][Beep=True]'s a[Wait=500][Beep=True]  wAy[Wait=500][Beep=True]  tO jOi[Wait=500][Beep=True]n mE.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]THeY[Wait=500][Beep=True]  mUsT[Wait=500][Beep=True]  bE qUi[Wait=500][Beep=True]cK,  tHe[Wait=500][Beep=True]  rOoMs[Wait=500][Beep=True]  sWiTcH[Wait=500][Beep=True]  lOcAtIoN[Wait=500][Beep=True]  qUiTe[Wait=500][Beep=True]  fReQuEnTlY.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>They seem to have.[Wait=500][Space=2]
-If the fuse isn't gonna get me out of there, I might as well trust them.[Wait=500][Space=2]
-What should I do no ?[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>T-This is so scary.[Wait=500] But I want to know the truth.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]LuCk[Wait=500][Beep=True]iLy[Wait=500][Beep=True],  tHe cAv[Wait=500][Beep=True]e cOnNe[Wait=500][Beep=True]cTs tHiS[Wait=500][Beep=True]  rOoM tO[Wait=500][Beep=True]  mY pLaCe[Wait=500][Beep=True]'s wAtEr[Wait=500][Beep=True]  SyStEm.[Wait=500][Beep=True]  I'[Wait=500][Beep=True]lL lIfT[Wait=500][Beep=True]  tHe gRiD[Wait=500][Beep=True]  aNd gEt[Wait=500][Beep=True]  tHeM iNsIdE.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]TeLl[Wait=500][Beep=True]  tHeM[Wait=500][Beep=True]  nOt[Wait=500][Beep=True]  tO pAn[Wait=500][Beep=True]iC[Wait=500][Beep=True],  iT's[Wait=500][Beep=True]  a mAt[Wait=500][Beep=True]tEr[Wait=500][Beep=True]  oF sEc[Wait=500][Beep=True]oNdS.[Color=White][Wait=500][Space=2]
@@ -3661,9 +3313,6 @@
     <t>[Color=Magenta]I know that this island is designed to self-destruct in case there is a virus breach.[Color=White][Wait=500][Space=2]
 W-Wait what?[Wait=500][Space=2]
 [Color=Magenta]Don't worry, I've planned everything so that we get out unharmed. There is just one more thing to do...[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>[Color=Magenta]This phone.[Wait=500] He can use it as a tracker.[Wait=500] You have to throw it away.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
     <t>[Color=Magenta]You won't know.[Color=White][Wait=500][Space=2]
@@ -3682,37 +3331,8 @@
 ...[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>I'm just not gonna go anywhere else in this godamn factory![Wait=500][Space=2]
-The exit's just there![Wait=500][Space=2]
-I don't care about anything else![Wait=500] Fuck whoever is trying to persuade you to lead me in a trap![Wait=500][Space=2]
-I.[Wait=500] Just.[Wait=500] Want.[Wait=500] To.[Wait=500] Leave.[Wait=500][Space=2]
-[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
-The light is almost blinding in there. I can't see shit.[Wait=500][Space=2]
-Though it's good to think I could get out in case things go sour.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]ThIs[Wait=500][Beep=True] iS[Wait=500][Beep=True] bAd.[Wait=500][Beep=True]  CaN'[Wait=500][Beep=True]t tHeY[Wait=500][Beep=True] sEe tHe[Wait=500][Beep=True] pErSoN[Wait=500][Beep=True] aBoVe?[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Wait...[Wait=500] I think I can do it on my own...[Wait=500][Space=2]
-...I just have to be...[Wait=500][Space=2]
-[Color=Gray]*DISTORDED SCREAMING*[Color=White]... SHIT IT SAW ME![Wait=500][Space=2]
-[Color=Gray]*Fast footsteps*[Color=White]...[Wait=500][Space=2]
-FUCK FUCK FUCK![Wait=500] ITS FACE, ITS DISFORMED, IT'S A FUCKING MONSTER![Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>WAIT![Wait=500] THE FUSE![Wait=500][Space=2]
 I CAN'T LEAVE IT THERE![Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I'M SURE I CAN DO IT![Wait=500][Space=2]
-I JUST HAVE TO [Color=Gray]*SCREEESH*[Color=White]... RAAAAGH![Wait=500][Space=2]
-I-I'm bleeding...[Wait=500] It scratch my whole arm![Wait=500][Space=2]
-Please...[Wait=500] Dont hurt me...[Wait=500][Space=2]
-[Color=Gray]*DISTORDED SCREAMING*[Color=White]...[Wait=500][Space=2]
-AAAAAAAAAAAAAAAAA-[Color=Gray]*Fleshy noises*[Color=White]...[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>...[Wait=500][Space=2]
@@ -3723,32 +3343,6 @@
 [Color=Red]BAD ENDING.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>You...[Wait=500] MONSTER![Wait=500][Space=2]
-Why am I keeping this phone you've obviously left there to torture me?[Wait=500][Space=2]
-I WON'T KEEP PLAYING YOUR GAMES![Wait=500][Space=2]
-[Color=Gray]*B[Beep=True]eep*[Color=White]...[Wait=500][Space=2]
-.[Wait=500].[Wait=500].[Wait=500][Space=2]
-[Color=Red]--SIGNAL LOST--[Color=White][Wait=500][Space=2]
-[Color=Red]{IT WAS NOURISHED WITH FLESH. MAYBE IF HE HAD TRUSTED YOU MORE, HE WOULDN'T HAVE GOTTEN CAUGHT?}[Color=White][Wait=500][Space=2]
-[Color=Red]BAD ENDING.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Just have to...[Wait=500][Space=2]
-[Color=Gray]*Grunt*[Color=White]...[Wait=500][Space=2]_
-[Color=Gray]*Running footsteps*[Color=White]...[Wait=500][Space=2]
-...[Wait=500][Space=2]
-OUCH![Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>YOU KNEW?[Wait=500][Space=2]
-Of course it's electrified, why'd you do that?![Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I still feel my muscles vibrating.[Wait=500][Space=2]
-That is no ordinary electric fence, I really feel like it's been setup to trap me.[Wait=500][Space=2]
-Let's just...[Wait=500] Move on.[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>I just need it to get away from me![Wait=500][Space=2]
 Anything! I just want to be free![Wait=500][Space=2]
 [Color=Magenta][Beep=True]OnC[Wait=500][Beep=True]e tHe[Wait=500][Beep=True] dIsEa[Wait=500][Beep=True]se'S tEr[Wait=500][Beep=True]MiNaL,  aLl tHeIr[Wait=500][Beep=True] sEnSeS aRe[Wait=500][Beep=True] sUbMiTtEd[Wait=500][Beep=True] tO cOnStAnT[Wait=500][Beep=True] aNd eXtReMe[Wait=500][Beep=True] sTrEsS.[Color=White][Wait=500][Space=2]
@@ -3777,11 +3371,6 @@
     <t>So...[Wait=500] I just have to put the fuse here and... [Beep=True][Color=Gray]*Mechanical beeping*[Color=White]... YEEES![Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>YES, IT'S OPENING![Wait=500][Space=2]
-There are stairs here.[Wait=500] I'm getting down there.[Wait=500][Space=2]
-...Oh my god...[Wait=500] It was such an intens-[Color=Gray]*SHKRRRRRRRRR*[Color=White]...[Wait=500] I'm so happy that you were here to help me.[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>Do you mean th-[Color=Gray]*SHKRRRRRRRRRRR*[Color=White]-ction?[Wait=500] Oh hell no, not after all that![Wait=500][Space=2]
 But I have t-[Color=Gray]*SHKRRRRR*[Color=White]-eep going.[Wait=500] I don't know if I'll be able to contact you agai-[Color=Gray]*SHKRRRRRRR*[Color=White]...[Wait=500][Space=2]
 ...It was a pleasu-[Color=Gray]*SHKRRRRRRRRRRRRRRR*[Color=White]...[Wait=500] Thank you, I'm glad to be y-[Color=Gray]*SHKRRRRRRRRRRR*[Color=White]...[Wait=500][Space=2]
@@ -3808,44 +3397,12 @@
 [Choice2=[NextScene=128][Content=Let's not waste time, try and push the fence.]]</t>
   </si>
   <si>
-    <t>[Choice1=[NextScene=16][Content=Maybe you should go around, you might find something interesting.]]
-[Choice2=[NextScene=128][Content=Yeah let's do that!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=11][Content=I'm being serious. You wouldn't use conditional if you were sure.]]
-[Choice2=[NextScene=12][Content=Is there something wrong?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=13][TrustAdd=25][Content=I shouldn't have said those things.]]
-[Choice2=[NextScene=15][Content=It's hard for the both of us.]]
-[Choice3=[NextScene=15][Content=I get that, I'm sorry.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=14][Content=Yeah, let's not rest.]]</t>
-  </si>
-  <si>
     <t>[Choice1=[NextScene=16][Content=I like the idea of finding another entrance better.]]
 [Choice2=[NextScene=128][Content=If you can do it, cross the fence.]]</t>
   </si>
   <si>
-    <t>[Choice1=[NextScene=16][Content=Get Around it.]]
-[Choice2=[NextScene=128][Content=Get through it.]]</t>
-  </si>
-  <si>
     <t>[Choice1=[NextScene=16][Content=I'd go around.]]
 [Choice2=[NextScene=128][Content=You should break the fence.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=17][Content=Exactly my thought.]]
-[Choice2=[NextScene=18][Content=Let's hope backdoors aren't either...]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=19][Content=Not like you'd find anything alive anyways.]]
-[Choice2=[NextScene=19][Content=Zoo are smelly.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=19][Content=I mean... This island has a zoo and a museum but no hopistal.]]
-[Choice2=[NextScene=20][Content=I'd doubt that. They probably built this place.]]</t>
   </si>
   <si>
     <t>[Choice1=[NextScene=21][Content=Good one. Have you found an entrance yet?]]
@@ -3880,11 +3437,6 @@
 [Choice2=[NextScene=27][Content=Hard to understand what they're saying. They'd need you to get closer.]]</t>
   </si>
   <si>
-    <t>[Choice1=[NextScene=28][Content=You're screwed either way if that's the case. Might as well tempt it.]]
-[Choice2=[NextScene=28][NextSceneNoTrust=29][TrustNeed=50][Content=I'm still there. Don't worry.]]
-[Choice3=[NextScene=29][Content=We'll see. Let's try to listen to them for now.]]</t>
-  </si>
-  <si>
     <t>[Choice1=[NextScene=30][TrustAdd=25][Content=Getting the spirit!]]
 [Choice2=[NextScene=30][TrustAdd=25][Content=Feeling better?]]</t>
   </si>
@@ -3909,10 +3461,6 @@
   </si>
   <si>
     <t>[Choice1=[NextScene=36][Content=So, what's up?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=37][Content=...]]
-[Choice2=[NextScene=37][Content=What?J]]</t>
   </si>
   <si>
     <t>[Choice1=[NextScene=38][Content=Let's go back and push that fence.]]
@@ -4019,10 +3567,6 @@
 [Choice2=[NextScene=64][Content=Wait... Do you live there?]]</t>
   </si>
   <si>
-    <t>[Choice1=[NextScene=63][Content=Must be the hunger. You really need to eat.]]
-[Choice2=[NextScene=64][Content=Is this... Your home?]]</t>
-  </si>
-  <si>
     <t>[Choice1=[NextScene=65][Content=There is food down there.]]</t>
   </si>
   <si>
@@ -4070,15 +3614,6 @@
   </si>
   <si>
     <t>[Choice1=[NextScene=78][Content=I know there's an exit, just get out, it's not worth it!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=79][TrustAdd=-25][Content=You're such a hassle.]]
-[Choice1=[NextScene=79][TrustAdd=25][Content=Please, be safe.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=80][Content=Go left.]]
-[Choice2=[NextScene=80][Content=Go right.]]
-[Choice3=[NextScene=80][Content=Go. Back.]]</t>
   </si>
   <si>
     <t>[Choice1=[NextScene=81][Content=Have you found your exit?]]</t>
@@ -4174,28 +3709,16 @@
     <t>[Choice1=[NextScene=105][Content=The wall has a hole in it, beneath the water. Swim until you reach the other side.]]</t>
   </si>
   <si>
-    <t>[Choice1=[NextScene=106][Content=Once in the cave, swim forward, until you feel a pipe.]]</t>
-  </si>
-  <si>
     <t>[Choice1=[NextScene=107][Content=When you feel the metal of the pipe, go inside.]]</t>
   </si>
   <si>
     <t>[Choice1=[NextScene=108][Content=Plastic, I mean. Then reach up, they will help you get through the grid.]]</t>
   </si>
   <si>
-    <t>[Choice1=[NextScene=109][Content=I believe in you, go quick, before the rooms move again.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=110][Content=Wait is this phone even water proof?]]</t>
-  </si>
-  <si>
     <t>[Choice1=[NextScene=111][Content=Are you alright?]]</t>
   </si>
   <si>
     <t>[Choice1=[NextScene=112][Content=Me?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=115][Content=That's insanity! How are you going to stop this scientist?]]</t>
   </si>
   <si>
     <t>[Choice1=[NextScene=116][Content=Which is?]]</t>
@@ -4208,9 +3731,6 @@
 [Choice2=[NextScene=118][Content=Is there another way to contact you?]]</t>
   </si>
   <si>
-    <t>[Choice1=[NextScene=121][Content=Do not tell I haven't warned you.]]</t>
-  </si>
-  <si>
     <t>[Choice1=[NextScene=122][Content=Watch out! Above you!]]</t>
   </si>
   <si>
@@ -4220,15 +3740,7 @@
     <t>[Choice1=[NextScene=124][Content=DON'T THINK, RUN!]]</t>
   </si>
   <si>
-    <t>[Choice1=[NextScene=125][Content=DON'T GRAB THE FUSE DUMBASS, RUN!]]
-[Choice2=[NextScene=125][Content=GRAB IT FAST!]]</t>
-  </si>
-  <si>
     <t>[Choice1=[NextScene=126][Content=NO!]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=129][TrustAdd=-25][Content=Well fuck, it was electrified.]]
-[Choice2=[NextScene=130][Content=Oh shit! Are you alright?]]</t>
   </si>
   <si>
     <t>[Choice1=[NextScene=127][Content=Funny.]]
@@ -4264,12 +3776,6 @@
   </si>
   <si>
     <t>[Choice1=[NextScene=140][Content=I hope you'll be safe. Goodbye.]]</t>
-  </si>
-  <si>
-    <t>Wouldn't be trying to defend them, would we?[Wait=500][Space=2]
-Errm-...[Wait=500] Anyways.[Wait=500][Space=2]
-Didn't realize the zoo was that close to the factory before.[Wait=500] Civil engineering failed some.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]DaN[Wait=500][Beep=True]gErOuS[Wait=500][Beep=True]  pLa[Wait=500][Beep=True]cE.[Wait=500][Beep=True]  ExpEr[Wait=500][Beep=True]iMeNtS.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
     <t>What?[Wait=500] Who are you talking to?[Wait=500] You're really starting to freak me out.[Wait=500][Space=2]
@@ -4279,16 +3785,6 @@
     <t>Uuh-...[Wait=500] Sure...[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 I'll-...[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>Hm-...[Wait=500] Anyways, there's a fence blocking the way to the main entrance.[Wait=500][Space=2]
-I can either try and get through or go around.[Wait=500][Space=2]
-It looks weak enough to be bent, but this kind of buildings tend to have backdoors.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I-...[Wait=500] I get it.[Wait=500][Space=2]
-It's good you're able to put yourself in my place a bit.[Wait=500] Thanks for acknowledging it.[Wait=500][Space=2]
-I'm starting to feel a bit more hopeful about getting out of here if you're on my side.[Wait=500][Space=2]</t>
   </si>
   <si>
     <t>Oh-...[Wait=500] Yeah...[Wait=500][Space=2]
@@ -4298,53 +3794,10 @@
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>You-... I mean, you know-...[Wait=500] I get it.[Wait=500][Space=2]
-It's hard to handle some random person calling you for seemingly no reason.[Wait=500][Space=2]
-...[Wait=500][Space=2]
-But thanks for admitting that, I already feel safer if you're able to show a bit of self-awareness.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I'm cl-...[Wait=500] Oh-...[Wait=500][Space=2]
-Hold on a minute will you... I'm not a...[Wait=500] ...stair climbing[Wait=500] ...athlete.[Wait=500][Space=2]
-I'm...[Wait=500] getting there...[Wait=500][Space=2]
-Huff... huff...[Wait=500][Space=2]
-.[Wait=500].[Wait=500].[Wait=500][Space=2]
-Guess what.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>B-...[Wait=500] BAHAHAHA-...[Wait=500][Space=2]
-Who do you take me for?[Wait=500] I'm not a toddler, I can tighten bolts![Wait=500][Space=2]
-My kidnapper might just come and catch these hands right now.[Wait=500][Space=2]
-With this bad boy with me, I ain't loosing to no monster.[Wait=500][Space=2]
-...[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>It is w-...[Wait=500] way colder in here than outside.[Wait=500][Space=2]
-[Color=Gray]*Voice echoes*[Color=White]...[Wait=500][Space=2]
-This place is huge.[Wait=500] I'm in a hallway so long I can't see the other side.[Wait=500][Space=2]
-It really feels like I'm standing in front of a void.[Wait=500][Space=2]
-With only the echo of my voice proving me there's something that way.[Wait=500][Space=2]
-And these big tubes...[Wait=500] This place isn't for making shoes, that's for sure.[Wait=500][Space=2]</t>
-  </si>
-  <si>
     <t>Maybe-...[Wait=500] That's what they're for?[Wait=500][Space=2]
 Growing food?[Wait=500][Space=2]
 I-I'm starving.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]YoU[Wait=500][Beep=True]'vE hAd eNo[Wait=500][Beep=True]uGh oF tHaT[Wait=500][Beep=True] aLrEaDy.[Wait=500][Beep=True]  TeLl tHeM[Wait=500][Beep=True] tO cOmE[Wait=500][Beep=True] dOwN, tHeRe[Wait=500][Beep=True] iS cAnNeD[Wait=500][Beep=True] fOoD hErE.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I know![Wait=500][Space=2]
-I-...[Wait=500] need to get to the down area.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]ThEy[Wait=500][Beep=True]'vE nEgLe[Wait=500][Beep=True]cTeD tO[Wait=500][Beep=True]  tElL yOu[Wait=500][Beep=True]  tHeY fOu[Wait=500][Beep=True]nD aN[Wait=500][Beep=True]  eXiT, i[Wait=500][Beep=True]  cAn sEe[Wait=500][Beep=True]  iT fRo[Wait=500][Beep=True]m a[Wait=500][Beep=True]  cAmErA.[Color=White][Wait=500][Space=2]
-[Color=Magenta][Beep=True]tHe fAlL[Wait=500][Beep=True] mIgHt[Wait=500][Beep=True]  bE rOuGh[Wait=500][Beep=True],  bUt iT's[Wait=500][Beep=True]  wOrTh[Wait=500][Beep=True]  nOt fIgHtInG[Wait=500][Beep=True]  tHeM.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>IT'S COMING![Wait=500][Space=2]
-[Color=Gray]*Heavy metalic sounds*[Color=White]...[Wait=500][Space=2]
-.[Wait=500].[Wait=500].[Wait=500][Space=2]
-It-...[Wait=500] It missed the opening I fell down from-...[Wait=500][Space=2]
-I-I think I'm safe.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]ThA[Wait=500][Beep=True]nK gO[Wait=500][Beep=True]d.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
     <t>Oh, I took that as ironic...[Wait=500][Space=2]
@@ -4365,7 +3818,512 @@
 What-...[Wait=500] What do you mean?[Wait=500] What have you done to me?[Wait=500] Why am I here?[Wait=500][Space=2]</t>
   </si>
   <si>
-    <t>You-[Wait=500] Your face![Wait=500][Space=2]
+    <t>I-...[Wait=500] I am![Wait=500][Space=2]
+I'm running towards it![Wait=500] I can even see it from here![Wait=500][Space=2]
+[Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e's nOt[Wait=500][Beep=True]hInG lEfT[Wait=500][Beep=True] tO dO.[Wait=500][Beep=True]  He wIlL[Wait=500][Beep=True] hAvE wHaT[Wait=500][Beep=True] hE's aLwAyS[Wait=500][Beep=True] lOoKeD fOr[Wait=500][Beep=True] aNd wE'Ll kEeP[Wait=500][Beep=True] sUfFeRiNg.[Color=White][Wait=500][Space=2]
+[Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e iS[Wait=500][Beep=True] nO pO[Wait=500][Beep=True]inT.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Color=Magenta][Beep=True]AlL oF[Wait=500][Beep=True]  oUr lIvEs[Wait=500][Beep=True],  wE lIvEd[Wait=500][Beep=True]  tHeRe wItHoUt[Wait=500][Beep=True]  kNoWiNg.[Wait=500][Beep=True]  SaMe mEmOrIeS[Wait=500][Beep=True],  sAmE.[Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]SoMe[Wait=500][Beep=True]  aGe tO[Wait=500][Beep=True]  fIgHt iT[Wait=500][Beep=True]  lOnGeR.[Wait=500][Beep=True]  I'M[Wait=500][Beep=True]  oNe oF[Wait=500][Beep=True]  tHeM.[Color=White][Wait=500][Space=2]
+...Are you still there?[Wait=500][Space=2]
+[Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e's fOo[Wait=500][Beep=True]d iN[Wait=500][Beep=True]  tHe dAm[Wait=500][Beep=True]p aReA[Wait=500][Beep=True],  tHe fAcTo[Wait=500][Beep=True]ry uSeD[Wait=500][Beep=True]  tO pRoDu[Wait=500][Beep=True]ce iT[Wait=500][Beep=True]  aS wElL.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=104][Content=The person on the line can help you, they've been of great help to me as well.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=113][Content=I'm as lost as you! What does any of that mean?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=114][Content=I didn't know anything about that!]]
+[Choice2=[NextScene=114][Content=This surely is a dream...]]</t>
+  </si>
+  <si>
+    <t>[Color=Magenta]It doesn't matter anymore.[Wait=500] Now that we are both together, we have to execute the plan I've been ploting.[Color=White][Wait=500][Space=2]
+Wait![Wait=500] What do you mean by plan?[Wait=500][Space=2]
+[Color=Magenta]Don't you want to stop all of this?[Color=White][Wait=500][Space=2]
+[Color=Magenta]If we just escape, he'll just create more of us. We have to stop this.[Color=White][Wait=500][Space=2]
+I...[Wait=500] That's true.[Wait=500][Space=2]
+I don't want other people to go through what we've been, no matter if they're clones or not.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=119][Content=...Did they just throw me like garbage?]]
+[Choice2=[NextScene=119][Content=I guess it's for the best.]]
+[Choice3=[NextScene=119][Content=NOOOO COME BACK!]]</t>
+  </si>
+  <si>
+    <t>Yeah.[Wait=500] Of all places, the factory seems like the place where I could find answers and the key to my escape.[Wait=500][Space=2]
+I'll go there if I can.[Wait=500] Let's go.[Wait=500][Space=2]
+[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=2][NextSceneNoTrust=3][TrustNeed=50][Content=What exactly do you mean by key?]]
+[Choice2=[NextScene=9][NextSceneNoTrust=10][TrustNeed=50][Content=If you can? Would anything prevent you?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=8][Content=That's a tough situation for sure.]]</t>
+  </si>
+  <si>
+    <t>...[Wait=500] I hope I can find the fuse. Why are you asking?[Wait=500][Space=2]
+[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I...[Wait=500] I'm just really stressed-...[Wait=500][Space=2]
+...[Wait=500][Space=2]
+Listen, I might have found this phone, but I don't feel like you're here to help...[Wait=500][Space=2]
+I don't know, you've got to put yourself in my place a bit...[Wait=500][Space=2]
+[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>You-... I mean, you know-...[Wait=500] I get it.[Wait=500][Space=2]
+It's hard to handle some random person calling you for seemingly no reason.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+But thanks for admitting that. I already feel safer if you're able to show a bit of self-awareness.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>We are.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+I've arrived at the entrance, but I have to get through a fence.[Wait=500][Space=2]
+It seems really fragile, so getting rid of it wouldn't be that hard.[Wait=500] That thing's already quite damaged.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+Or I could go around. There's no reason for a building like this not to have some kind of backdoor.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>There seems to be a fence in front of the main entrance.[Wait=500][Space=2]
+I could probably go around and find another way in.[Wait=500][Space=2]
+But from this distance it looks really thin and rusted.[Wait=500][Space=2]
+I think pushing it down and getting over would be quite easy.[Wait=500][Space=2]
+What do you think?[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=16][Content=Maybe you should go around, you might find something interesting.]]
+[Choice2=[NextScene=128][Content=Yeah, let's do that!]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=11][Content=I'm being serious. You wouldn't use a conditional if you were sure.]]
+[Choice2=[NextScene=12][Content=Is there something wrong?]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=16][Content=Get around it.]]
+[Choice2=[NextScene=128][Content=Get through it.]]</t>
+  </si>
+  <si>
+    <t>I got myself a smart one, huh?[Wait=500][Space=2]
+I'm being conditional because there's a fence surrounding the entrance.[Wait=500][Space=2]
+I either have to get around it or through it.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=13][TrustAdd=25][Content=I shouldn't have said those things.]]
+[Choice2=[NextScene=15][Content=It's hard for both of us.]]
+[Choice3=[NextScene=15][Content=I get that. I'm sorry.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=14][Content=Yeah, let's not slow down.]]</t>
+  </si>
+  <si>
+    <t>I-...[Wait=500] I get it.[Wait=500][Space=2]
+It's good that you're able to put yourself in my place a bit.[Wait=500] Thanks for acknowledging it.[Wait=500][Space=2]
+I'm starting to feel a bit more hopeful about getting out of here if you're on my side.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I'm getting there.[Wait=500] But I can already see the place is protected by a fence.[Wait=500][Space=2]
+It isn't a big deal, I could probably find another entrance.[Wait=500][Space=2]
+[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
+The metal looks brittle. I could probably bend it down and get over it.[Wait=500][Space=2]
+What do you think?[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Hm-...[Wait=500] Anyway, there's a fence blocking the way to the main entrance.[Wait=500][Space=2]
+I can either try to get through it or go around.[Wait=500][Space=2]
+It looks weak enough to be bent, but buildings like this usually have backdoors.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Yeah. The main entrance might be trapped. I'd rather find another way.[Wait=500][Space=2]
+[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
+Thinking outside the box might be the way to avoid some of the-...[Wait=500] psycho keeping me here.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=17][Content=Exactly my thought.]]
+[Choice2=[NextScene=18][Content=Let's hope the backdoors aren't either...]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=19][Content=Not like you'd find anything alive anyway.]]
+[Choice2=[NextScene=19][Content=Zoos are smelly.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=19][Content=I mean... This island has a zoo and a museum, but no hospital.]]
+[Choice2=[NextScene=20][Content=I doubt that. They probably built this place.]]</t>
+  </si>
+  <si>
+    <t>Good to know we're on the same page.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+I know it sounds weird, but...[Wait=500] I really like the slight breeze on this island.[Wait=500][Space=2]
+If it wasn't covered in trash and dull concrete, it'd be almost habitable.[Wait=500][Space=2]
+I almost regret not going for a walk in the zoo.[Wait=500][Space=2]
+But I really need to find food, and I'm not about eating a raw giraffe.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>...[Wait=500] No need to make me doubt...[Wait=500][Space=2]
+If that bastard really wants me to die, I'm screwed anyway. Might as well minimize the risk.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+Who knows...[Wait=500] He might be an idiot.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Speaking of the zoo, guess what.[Wait=500] It's awfully close to this place.[Wait=500][Space=2]
+I can see inside the enclosures from here.[Wait=500][Space=2]
+Whoever designed this city should be fired.[Wait=500] Or even set on fire.[Wait=500][Space=2]
+Because I'm stuck inside their terribly designed city.[Wait=500][Space=2]
+That prick.[Wait=500][Space=2]
+[Color=Magenta][Beep=True][Color=Gray]*Distorted chuckle*[Color=White]...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]YoU'[Wait=500][Beep=True]rE bEt[Wait=500][Beep=True]tEr hErE[Wait=500][Beep=True]  wItH mE[Wait=500][Beep=True]  tHaN aLo[Wait=500][Beep=True]nE iN[Wait=500][Beep=True]  tHe zOo.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Wouldn't be trying to defend them, would we?[Wait=500][Space=2]
+Errm-...[Wait=500] Anyway.[Wait=500][Space=2]
+Didn't realize the zoo was that close to the factory before.[Wait=500] Civil engineering failed somewhere.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]DaN[Wait=500][Beep=True]gErOuS[Wait=500][Beep=True]  pLa[Wait=500][Beep=True]cE.[Wait=500][Beep=True]  ExpEr[Wait=500][Beep=True]iMeNtS.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Empty drums, debris, nothing but the usual shit.[Wait=500][Space=2]
+Nowhere else to go, you see, so for now I'll keep looking.[Wait=500][Space=2]
+Stressed out and hungry I feel, still haven't got anything to eat.[Wait=500][Space=2]
+I could really use oatmeal, or anything that would get me going.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>M-...[Wait=500] Me?[Wait=500] As I've said before, I-...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]OnE[Wait=500][Beep=True]  oF tHe[Wait=500][Beep=True]  pReVi[Wait=500][Beep=True]oUs.[Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]I'M[Wait=500][Beep=True]  hErE tO[Wait=500][Beep=True]  hElP yOu.[Wait=500][Beep=True]  I'M aBlE[Wait=500][Beep=True]  tO cOmMu[Wait=500][Beep=True]nIcAtE tHrOuGh[Wait=500][Beep=True]  tHe dEsA[Wait=500][Beep=True]fEcTeD cOnTrOl.[Color=White][Wait=500][Space=2]
+[Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]SuR[Wait=500]viVoR[Wait=500][Beep=True],  I'M tRy[Wait=500][Beep=True]iNg tO gEt[Wait=500][Beep=True]  oThErS oUt[Wait=500][Beep=True]  oF hIs[Wait=500][Beep=True]  tRaPs.[Color=White][Wait=500][Space=2]
+Once again, I do NOT know why I'm here nor about any kind of experiments. Just help me, alright?[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Of course I'm going to worry!!![Wait=500][Space=2]
+You're giving me no explanation after saying shit about some experiment. Are there more people with you?[Wait=500][Space=2]
+...[Wait=500][Space=2]
+You're always alternating between reassuring and cryptic, talking to the fucking voices now![Wait=500][Space=2]
+Am-...[Wait=500] Am I a game to you?[Wait=500] Are you going to fucking tell me?![Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>And...[Wait=500] You're just gonna say that now?[Wait=500][Space=2]
+Uh...[Wait=500] Nevermind. I'm not even gonna ask anymore.[Wait=500][Space=2]
+.[Wait=500].[Wait=500].[Wait=500][Space=2]
+But should we reaaally trust them?[Wait=500][Space=2]
+I mean, why would anyone other than the person behind all of this try to talk to you?[Wait=500][Space=2]
+And why can't I hear them?[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Which means...[Wait=500] They're on the island.[Wait=500][Space=2]
+Great.[Wait=500][Space=2]
+That either means a helping hand... or extra danger.[Wait=500][Space=2]
+As if all of this needed more complexity.[Wait=500][Space=2]
+So they're going to help you guide me, if I understood well.[Wait=500][Space=2]
+Doesn't sound like a trap.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=28][Content=You're screwed either way if that's the case. Might as well tempt fate.]]
+[Choice2=[NextScene=28][NextSceneNoTrust=29][TrustNeed=50][Content=I'm still here. Don't worry.]]
+[Choice3=[NextScene=29][Content=We'll see. Let's try to listen to them for now.]]</t>
+  </si>
+  <si>
+    <t>Of course.[Wait=500][Space=2]
+Let's just start m-...[Wait=500][Space=2]
+...[Wait=500][Space=2]
+Writings.[Wait=500][Space=2]
+Writings on the wall.[Wait=500] Please.[Wait=500] Why?[Wait=500][Space=2]
+Oh no, don't tell me these are creepy letters-...[Wait=500][Space=2]
+On the wall.[Wait=500] I'm so sick of this.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>"THEY FED ME MY OWN SELF!"...[Wait=500][Space=2]
+I...[Wait=500] really don't want to discover what happened on this island.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+I'm almost surprised that wasn't written in blood. Although blue blood might be a thing on this island.[Wait=500][Space=2]
+I don't know, I'm not a...[Wait=500] ...blood[Wait=500] ...scientist.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>It really feels like some edgy shit a fourteen-year-old would write.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+But I'm still shaken up despite how ridiculous that is...[Wait=500][Space=2]
+Like...[Wait=500] someone wrote that in some place in the middle of the ocean.[Wait=500][Space=2]
+I'm not gonna mess with a fourteen-year-old, no matter how angsty.[Wait=500][Space=2]
+If they're ready to cross the ocean for a joke.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Well, me neither.[Wait=500][Space=2]
+Let's just move on knowing some lunatic could jump me any minute.[Wait=500][Space=2]
+No big deal.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>So no big deal, as I said.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+Good news, I just stumbled onto what seems to be...[Wait=500] fire escape stairs?[Wait=500][Space=2]
+I'm positive these lead inside the building.[Wait=500][Space=2]
+Chance might be on our side. And I'm not unhappy with doing a bit of exercise.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I'm cl-...[Wait=500] Oh-...[Wait=500][Space=2]
+Hold on a minute, will you... I'm not a...[Wait=500] ...stair-climbing[Wait=500] ...athlete.[Wait=500][Space=2]
+I'm...[Wait=500] getting there...[Wait=500][Space=2]
+Huff... huff...[Wait=500][Space=2]
+.[Wait=500].[Wait=500].[Wait=500][Space=2]
+Guess what.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=37][Content=...]]
+[Choice2=[NextScene=37][Content=What?]]</t>
+  </si>
+  <si>
+    <t>Remember when I talked about luck being on my side?[Wait=500] Shouldn't have said that.[Wait=500][Space=2]
+It's freaking closed. By a [Color=Green]3-digit[Color=White] pad, which isn't high protection by any means.[Wait=500][Space=2]
+But I'd rather go back to the entrance than spend my time here.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>If there's a clue anywhere, it'd be inside.[Wait=500][Space=2]
+Good thing the door has a window[Wait=500], worst case scenario I might just smash it and slither in like a tapeworm.[Wait=500][Space=2]
+The place looks like it was left in a hurry a dozen years ago.[Wait=500][Space=2]
+Someone even smeared their coffee on the carpet.[Wait=500][Space=2]
+And what's that?[Wait=500][Space=2]
+A random wrench lying on the ground?[Wait=500] Now that's a motivator. Might have to bash some skulls.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Huuuh...[Wait=500] There's a cork board with a bunch of blank pieces of paper pinned onto it...[Wait=500][Space=2]
+And a literal passcode note. [Color=Green]7734[Color=White].[Wait=500][Space=2]
+Which is 4 digits so it's useless. Are you kidding me.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>The only thing on the right wall is a big mirror with...[Wait=500][Space=2]
+An [Color=Green]upside-down calculator[Color=White] taped onto it.[Wait=500][Space=2]
+You know, the old ones we had back in school, those with the segmented digits.[Wait=500][Space=2]
+Nostalgic, but not helping me that much.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>On the right?[Wait=500] There's a mirror on the wall, and it has...[Wait=500][Space=2]
+An [Color=Green]upside-down calculator[Color=White] taped onto it.[Wait=500][Space=2]
+Old-school ones, with segmented digit displays.[Wait=500][Space=2]
+It's cool that it brings back memories, but it's so useless right now.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>There's a cork board covered in blank papers.[Wait=500][Space=2]
+Oh yeah, also the passcode: [Color=Green]7734[Color=White].[Wait=500][Space=2]
+Hold it! The lockpad is [Color=Green]3 digits[Color=White], so it won't fit! [Color=Gray]*Demented laugh*[Color=White]...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Nope. Not opening.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]NeVe[Wait=500][Beep=True]r fLiP[Wait=500][Beep=True]peD a[Wait=500][Beep=True]  cAlC[Wait=500][Beep=True]uLaTo[Wait=500][Beep=True]r bEf[Wait=500][Beep=True]oRe?[Color=White][Wait=500][Space=2]
+7734, upside-down calculator... can you work something out with this?[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Oh yes![Wait=500] I remember that![Wait=500][Space=2]
+Never thought something that stupid could come in handy in a life-or-death situation.[Wait=500][Space=2]
+Well of course I did, but come on![Wait=500][Space=2]
+That's just so ridiculous, the person who designed this puzzle has to be a moron.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Wow, well I guess they're not so bad. Everything's good in the best of worlds![Wait=500][Space=2]
+Sorry, I'm being way too sarcastic. Thank them.[Wait=500] But also ask them how they knew the passcode.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Wow, no need to be rude about it...[Wait=500][Space=2]
+I'm more focused on survival than some stupid calculator cipher.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>GOOD![Wait=500] Let's not waste any more time![Wait=500][Space=2]
+We're finally in after all![Wait=500][Space=2]
+Maybe going through the main entrance would have been faster, but at least I got to breathe fresh air.[Wait=500][Space=2]
+[Color=Gray]*THUD*[Color=White]...[Wait=500][Space=2]
+Oh, yes.[Wait=500][Space=2]
+I also get to pick up that beautiful wrench.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>B-...[Wait=500] BAHAHAHA-...[Wait=500][Space=2]
+Who do you take me for?[Wait=500] I'm not a toddler, I can tighten bolts![Wait=500][Space=2]
+My kidnapper might just come and catch these hands right now.[Wait=500][Space=2]
+With this bad boy with me, I ain't losing to no monster.[Wait=500][Space=2]
+...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Absolutely![Wait=500][Space=2]
+...[Wait=500][Space=2]
+...I don't know how to put it, but it seems...[Wait=500] advanced.[Wait=500][Space=2]
+This ain't an ordinary wrench. It's heavier and equipped with some kind of display.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+I might take it home.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I'm only stealing my freedom back after all.[Wait=500][Space=2]
+The other door is locked, and the latch seems to be stuck.[Wait=500][Space=2]
+[Color=Gray]*Hammering sounds*[Color=White]...[Wait=500][Space=2]
+But that's a puzzle for another day, I've got places to be.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+That thing packs a serious punch, I got it open in a few hits.[Wait=500][Space=2]
+[Color=Gray]*Door creaks*[Color=White]...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>It is w-...[Wait=500] way colder in here than outside.[Wait=500][Space=2]
+[Color=Gray]*Voice echoes*[Color=White]...[Wait=500][Space=2]
+This place is huge.[Wait=500] I'm in a hallway so long I can't see the other side.[Wait=500][Space=2]
+It really feels like I'm standing in front of a void.[Wait=500][Space=2]
+With only the echo of my voice proving there's something that way.[Wait=500][Space=2]
+And these big tubes...[Wait=500] This place isn't for making shoes, that's for sure.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>About my size.[Wait=500] They're all connected to a dense net of wires on the ground.[Wait=500][Space=2]
+Almost makes it hard to navigate.[Wait=500][Space=2]
+Also smells quite odd.[Wait=500] It's both off-putting...[Wait=500] and weirdly comforting...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]He[Wait=500][Beep=True]'s pLaY[Wait=500][Beep=True]iNg wIt[Wait=500][Beep=True]h yOu.[Wait=500][Beep=True]  WHy[Wait=500][Beep=True]  bRiNg[Wait=500][Beep=True]  [Color=Gray]*Static*[Color=White]...[Wait=500][Beep=True]  uP?[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>...[Wait=500] Hundreds?[Wait=500][Space=2]
+Hard to tell, it goes way past what I'm physically able to see or even reach.[Wait=500][Space=2]
+It's an...[Wait=500] ...[Wait=500] overwhelming view...[Wait=500] This looks like a scene from a science-fiction movie.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]DoN[Wait=500][Beep=True]'t lEt[Wait=500][Beep=True]  iT b[Wait=500][Beep=True]rEaK[Wait=500][Beep=True]  yOu.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>What's that about a per...[Wait=500] Oh[Wait=500], they came back.[Wait=500][Space=2]
+[Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]ThEs[Wait=500][Beep=True]e aRe[Wait=500][Beep=True]  oLd[Wait=500][Beep=True]  [Color=Gray]*Static*[Color=White]...[Wait=500][Beep=True]  fAmIlIaR[Wait=500][Beep=True]  pLaCe[Wait=500][Beep=True]  fOr[Wait=500][Beep=True]  aLl[Wait=500][Beep=True]  oF uS.[Wait=500][Beep=True]  GrOwN[Wait=500][Beep=True]  aNd[Wait=500][Beep=True]  fEd[Wait=500][Beep=True]  [Color=Gray]*Static*[Color=White]...[Wait=500][Beep=True]  tHoSe.[Color=White][Wait=500][Space=2]
+[Color=Magenta][Beep=True]NeW[Wait=500][Beep=True]  oNeS[Wait=500][Beep=True]  iN[Wait=500][Beep=True]  tHe[Wait=500][Beep=True]  mUsEuM.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=63][Content=Must be the hunger. You really need to eat.]]
+[Choice2=[NextScene=64][Content=Is this... your home?]]</t>
+  </si>
+  <si>
+    <t>I don't know how trustworthy this person is...[Wait=500][Space=2]
+But this place is making me so sick I won't stay for a second longer.[Wait=500][Space=2]
+So I'll just do the next best thing.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Down the vent system. I just need to get it open.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+What?[Wait=500] You didn't expect me to try something while you're listening to their ramblings?[Wait=500][Space=2]
+If there's food I can eat I need to go down.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]GoO[Wait=500][Beep=True]d cAl[Wait=500][Beep=True]l. ThIs[Wait=500][Beep=True] rOoM[Wait=500][Beep=True] sEeMs[Wait=500][Beep=True] sEpArAtEd[Wait=500][Beep=True] fRoM[Wait=500][Beep=True] tHe rEsT[Wait=500][Beep=True] oF tHe bUiLdInG.[Color=White][Wait=500][Space=2]
+[Color=Magenta][Beep=True]ThE[Wait=500][Beep=True]  vEnT[Wait=500][Beep=True]  sYsTeM[Wait=500][Beep=True]  mIgHt[Wait=500][Beep=True]  bE[Wait=500][Beep=True]  tHe[Wait=500][Beep=True]  oNlY[Wait=500][Beep=True]  wAy[Wait=500][Beep=True]  dOwN.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Absolutely.[Wait=500][Space=2]
+You know how nothing works like it's supposed to on this island?[Wait=500][Space=2]
+The grid itself is its own incomprehensible enigma.[Wait=500][Space=2]
+In fact, it isn't a grid.[Wait=500][Space=2]
+More like a lid with a big bolt.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Clicked-...[Wait=500] WAAH-...[Wait=500][Space=2]
+[Color=Gray]*CLANG*[Color=White]...[Wait=500][Space=2]
+...[Wait=500][Space=2]
+The incomprehensible enigma came off and almost crushed my foot.[Wait=500][Space=2]
+Let's see what's in there...[Wait=500] It's...[Wait=500] been cleaned recently?[Wait=500][Space=2]
+So much for an abandoned building, the metal's almost glistening.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Anyways, I'm getting into the...[Wait=500] hnng-...[Wait=500] ...vent.[Wait=500][Space=2]
+I've got some crawling to do.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+The odor's already fading, I can feel my chest getting lighter.[Wait=500][Space=2]
+Despite it being squished between four steel walls.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>For what being forced to crawl through a vent by a faceless sadist could have been[Wait=500], kind of.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+I can hear air flowing through another vent nearby.[Wait=500][Space=2]
+So there is functional ventilation on this island, huh.[Wait=500][Space=2]
+Might have been more effective if that one wasn't converted into a parkour tunnel for me to enjoy.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I'm sure you can wait for a bit longer.[Wait=500][Space=2]
+I'm not a...[Wait=500] ...vent-crawling[Wait=500] ...expert.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+I hear clicking and clanking all around, machinery doing its thing.[Wait=500][Space=2]
+I thought this island was abandoned, but it's becoming more and more evident that at least someone lives here.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I know![Wait=500][Space=2]
+I-...[Wait=500] need to get to the lower area.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]ThEy[Wait=500][Beep=True]'vE nEgLe[Wait=500][Beep=True]cTeD tO[Wait=500][Beep=True]  tElL yOu[Wait=500][Beep=True]  tHeY fOu[Wait=500][Beep=True]nD aN[Wait=500][Beep=True]  eXiT, i[Wait=500][Beep=True]  cAn sEe[Wait=500][Beep=True]  iT fRo[Wait=500][Beep=True]m a[Wait=500][Beep=True]  cAmErA.[Color=White][Wait=500][Space=2]
+[Color=Magenta][Beep=True]tHe fAlL[Wait=500][Beep=True] mIgHt[Wait=500][Beep=True]  bE rOuGh[Wait=500][Beep=True],  bUt iT's[Wait=500][Beep=True]  wOrTh[Wait=500][Beep=True]  nOt fIgHtInG[Wait=500][Beep=True]  tHeM.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I'm not just going to jump into the void![Wait=500] I don't know what caused this noise.[Wait=500][Space=2]
+But I can tell it's not inside the vent from the height it had to fall from.[Wait=500][Space=2]
+I should keep going forward and find a way down.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=79][TrustAdd=-25][Content=You're such a hassle.]]
+[Choice2=[NextScene=79][TrustAdd=25][Content=Please, be safe.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=80][Content=Go left.]]
+[Choice2=[NextScene=80][Content=Go right.]]
+[Choice3=[NextScene=80][Content=Go back.]]</t>
+  </si>
+  <si>
+    <t>I SEE THE GRID![Wait=500][Space=2]
+COME OFF, YOU PIECE OF SHIT![Wait=500][Space=2]
+[Color=Gray]*Bolt squeaks*[Color=White]...[Wait=500][Space=2]
+COME O-...[Wait=500] AAAAH-...[Wait=500][Space=2]
+[Color=Gray]*Splashes*[Color=White]...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>IT'S COMING![Wait=500][Space=2]
+[Color=Gray]*Heavy metallic sounds*[Color=White]...[Wait=500][Space=2]
+.[Wait=500].[Wait=500].[Wait=500][Space=2]
+It-...[Wait=500] It missed the opening I fell down from-...[Wait=500][Space=2]
+I-I think I'm safe.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]ThA[Wait=500][Beep=True]nK gO[Wait=500][Beep=True]d.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I'm glad you're too.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+Well, I know there's no reason for you to be in any kind of danger right now.[Wait=500][Space=2]
+But I really am glad you are, that's all.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+Besides that, you were right about that place. It's filled to the brim with food cans.[Wait=500][Space=2]
+This is like a storage room for spam-looking, dank mush.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Thanks.[Wait=500] You saved my life.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+There's so much water down there.[Wait=500][Space=2]
+Positively better than just hitting the concrete, but I'm worried I'll catch a cold.[Wait=500][Space=2]
+Also, thank your friend, there's indeed loads of food there.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+Never been a fan of damped mush, but a gourmet's palate has a time and place.[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Here goes nothing-...[Wait=500] I'm opening one.[Wait=500][Space=2]
+[Color=Gray]*Clunk*[Color=White]...[Wait=500][Space=2]
+It's-[Wait=500] neutral in odor.[Wait=500] Doesn't look like anything, but not repulsive either.[Wait=500][Space=2]
+[Color=Magenta][Beep=True]ThEs[Wait=500][Beep=True]e aRe[Wait=500][Beep=True]  qUiT[Wait=500][Beep=True]e gOoD[Wait=500][Beep=True],  aCtUaLlY.[Wait=500][Beep=True]  NOt[Wait=500][Beep=True]  tHaT tHeRe[Wait=500][Beep=True]  iS aNy[Wait=500][Beep=True]tHiNg eLsE[Wait=500][Beep=True]  tO eAt[Wait=500][Beep=True]  tHeRe.[Color=White][Wait=500][Space=2]
+.[Wait=500].[Wait=500].[Wait=500][Space=2]
+.[Wait=500].[Wait=500].[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Is the fuse there?[Wait=500][Space=2]
+What are you on about?[Wait=500][Space=2]
+I got all the way here just to find that fuse.[Wait=500][Space=2]
+Why would you say that now that I'm about to find it?[Wait=500][Space=2]
+I'm gonna need some better explanations![Wait=500][Space=2]
+[Color=Magenta][Beep=True]I wAn[Wait=500][Beep=True]t tO tElL[Wait=500][Beep=True] tHeM tHe[Wait=500][Beep=True] tRuTh.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>They seem to have a plan.[Wait=500][Space=2]
+If the fuse isn't gonna get me out of there, I might as well trust them.[Wait=500][Space=2]
+What should I do now?[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=106][Content=Once in the cave, swim forward until you feel a pipe.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=109][Content=I believe in you. Go quick, before the rooms move again.]]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=110][Content=Wait, is this phone even waterproof?]]</t>
+  </si>
+  <si>
+    <t>Your-...[Wait=500] Your face![Wait=500][Space=2]
 [Color=Magenta]I should've warned you before.[Wait=500] It's hard to explain that so...[Wait=500] directly.[Wait=500] Most of us figure it out much earlier.[Color=White][Wait=500][Space=2]
 Am I...[Wait=500] Dumber than the-...[Wait=500] ...others?[Wait=500][Space=2]
 [Color=Magenta]No, you're healthier.[Wait=500] That "thing" was...[Wait=500] One of us.[Wait=500] Like all of us.[Color=White][Wait=500][Space=2]
@@ -4375,62 +4333,103 @@
 [Color=Magenta]No.[Wait=500] I'm talking about the person you called.[Color=White][Wait=500][Space=2]</t>
   </si>
   <si>
+    <t>[Color=Magenta]Calm down, both of you.[Wait=500] Neither of you is to blame.[Color=White][Wait=500][Space=2]
+Who am I?[Wait=500] What do you mean, grown?[Wait=500][Space=2]
+[Color=Magenta]You are the successful prototype.[Wait=500] The one he's been waiting for.[Color=White][Wait=500][Space=2]
+[Color=Magenta]The scientist, as I call him.[Wait=500] He's the one behind our suffering.[Color=White][Wait=500][Space=2]
+So...[Wait=500] are we clones of you?[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=115][Content=That's insanity! How are you going to stop him?]]</t>
+  </si>
+  <si>
+    <t>[Color=Magenta]This phone.[Wait=500] He can track it.[Wait=500] You must throw it away.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I'm just not going anywhere else in this goddamn factory![Wait=500][Space=2]
+The exit's just there![Wait=500][Space=2]
+I don't care about anything else![Wait=500] Fuck whoever is trying to persuade you to lead me into a trap![Wait=500][Space=2]
+I.[Wait=500] Just.[Wait=500] Want.[Wait=500] To.[Wait=500] Leave.[Wait=500][Space=2]
+[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=121][Content=Do not say I didn't warn you.]]</t>
+  </si>
+  <si>
+    <t>[Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
+The light is almost blinding in there. I can't see shit.[Wait=500][Space=2]
+Still, it's good to know I could get out in case things go sour.[Wait=500][Space=2]
+...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]ThIs[Wait=500][Beep=True] iS[Wait=500][Beep=True] bAd.[Wait=500][Beep=True]  CaN'[Wait=500][Beep=True]t tHeY[Wait=500][Beep=True] sEe tHe[Wait=500][Beep=True] pErSoN[Wait=500][Beep=True] aBoVe?[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Wah-...[Wait=500] OH SH...[Wait=500][Space=2]
+[Color=Gray]*Whisper*[Color=White]... T-There's...[Wait=500] It's the thing that chased me in the vent...[Wait=500][Space=2]
+It's o-on the catwalks...[Wait=500][Space=2]
+...[Wait=500] Wait, is that the...[Wait=500][Space=2]
+[Color=Magenta][Beep=True]DoN[Wait=500][Beep=True]'t dO[Wait=500][Beep=True] aNyThInG[Wait=500][Beep=True] sTuPiD[Wait=500][Beep=True],  i'M[Wait=500][Beep=True] gOnNa[Wait=500][Beep=True] dIsTrAcT[Wait=500][Beep=True] tHeM.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Wait...[Wait=500] I think I can do it on my own...[Wait=500][Space=2]
+...I just have to be...[Wait=500][Space=2]
+[Color=Gray]*DISTORTED SCREAMING*[Color=White]... SHIT, IT SAW ME![Wait=500][Space=2]
+[Color=Gray]*Fast footsteps*[Color=White]...[Wait=500][Space=2]
+FUCK! FUCK! FUCK![Wait=500] ITS FACE, IT'S DISFORMED, IT'S A FUCKING MONSTER![Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=125][Content=DON'T GRAB THE FUSE, DUMBASS! RUN!]]
+[Choice2=[NextScene=125][Content=GRAB IT FAST!]]</t>
+  </si>
+  <si>
+    <t>I'M SURE I CAN DO IT![Wait=500][Space=2]
+I JUST HAVE TO [Color=Gray]*SCREEESH*[Color=White]... RAAAAGH![Wait=500][Space=2]
+I-I'm bleeding...[Wait=500] It scratched my whole arm![Wait=500][Space=2]
+Please...[Wait=500] Don't hurt me...[Wait=500][Space=2]
+[Color=Gray]*DISTORTED SCREAMING*[Color=White]...[Wait=500][Space=2]
+AAAAAAAAAAAAAAAAA-[Color=Gray]*Fleshy noises*[Color=White]...[Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>You...[Wait=500] MONSTER![Wait=500][Space=2]
+Why am I keeping this phone you've obviously left here to torture me?[Wait=500][Space=2]
+I WON'T KEEP PLAYING YOUR GAMES![Wait=500][Space=2]
+[Color=Gray]*B[Beep=True]eep*[Color=White]...[Wait=500][Space=2]
+.[Wait=500].[Wait=500].[Wait=500][Space=2]
+[Color=Red]--SIGNAL LOST--[Color=White][Wait=500][Space=2]
+[Color=Red]{IT WAS NOURISHED WITH FLESH. MAYBE IF HE HAD TRUSTED YOU MORE, HE WOULDN'T HAVE GOTTEN CAUGHT?}[Color=White][Wait=500][Space=2]
+[Color=Red]BAD ENDING.[Color=White][Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>Just have to...[Wait=500][Space=2]
+[Color=Gray]*Grunt*[Color=White]...[Wait=500][Space=2]
+[Color=Gray]*Running footsteps*[Color=White]...[Wait=500][Space=2]
+...[Wait=500][Space=2]
+OUCH![Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>[Choice1=[NextScene=129][TrustAdd=-25][Content=Well, fuck, it was electrified.]]
+[Choice2=[NextScene=130][Content=Oh shit! Are you alright?]]</t>
+  </si>
+  <si>
+    <t>YOU KNEW?[Wait=500][Space=2]
+Of course it's electrified! Why'd you do that?![Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>I still feel my muscles vibrating.[Wait=500][Space=2]
+That is no ordinary electric fence. I really feel like it was set up to trap me.[Wait=500][Space=2]
+Let's just...[Wait=500] move on.[Wait=500][Space=2]</t>
+  </si>
+  <si>
     <t>O-...[Wait=500] Okay![Wait=500][Space=2]
 [Color=Gray]*Running sounds*[Color=White]...[Wait=500][Space=2]
 I GOT IT![Wait=500][Space=2]
 [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
-I'm outside, I can see the stairs I took to get in![Wait=500][Space=2]
-If I knew I could've just kept going and climbed through this window![Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>I-...[Wait=500] I am![Wait=500][Space=2]
-I'm running towards it![Wait=500] I can even see it from here![Wait=500][Space=2]
-[Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e's nOt[Wait=500][Beep=True]hInG lEfT[Wait=500][Beep=True] tO dO.[Wait=500][Beep=True]  He wIlL[Wait=500][Beep=True] hAvE wHaT[Wait=500][Beep=True] hE's aLwAyS[Wait=500][Beep=True] lOoKeD fOr[Wait=500][Beep=True] aNd wE'Ll kEeP[Wait=500][Beep=True] sUfFeRiNg.[Color=White][Wait=500][Space=2]
-[Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e iS[Wait=500][Beep=True] nO pO[Wait=500][Beep=True]inT.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>M-...[Wait=500] Me?[Wait=500] As I've said before I-...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]OnE[Wait=500][Beep=True]  oF tHe[Wait=500][Beep=True]  pReVi[Wait=500][Beep=True]oUs.[Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]I'M[Wait=500][Beep=True]  hErE tO[Wait=500][Beep=True]  hElP yOu.[Wait=500][Beep=True]  I'M aBlE[Wait=500][Beep=True]  tO cOmMu[Wait=500][Beep=True]nIcAtE tHrOuGh[Wait=500][Beep=True]  tHe dEsA[Wait=500][Beep=True]fEcTeD cOnTrOl.[Color=White][Wait=500][Space=2]
-[Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]SuR[Wait=500]viVoR[Wait=500][Beep=True],  i'M tRy[Wait=500][Beep=True]iNg tO gEt[Wait=500][Beep=True]  oThErS oUt[Wait=500][Beep=True]  oF hIs[Wait=500][Beep=True]  tRaPs.[Color=White][Wait=500][Space=2]
-Once again, I do NOT know why I'm here nor about any kind of experiments, just help me, alright?[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>[Color=Magenta][Beep=True]AlL oF[Wait=500][Beep=True]  oUr lIvEs[Wait=500][Beep=True],  wE lIvEd[Wait=500][Beep=True]  tHeRe wItHoUt[Wait=500][Beep=True]  kNoWiNg.[Wait=500][Beep=True]  SaMe mEmOrIeS[Wait=500][Beep=True],  sAmE.[Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]SoMe[Wait=500][Beep=True]  aGe tO[Wait=500][Beep=True]  fIgHt iT[Wait=500][Beep=True]  lOnGeR.[Wait=500][Beep=True]  I'M[Wait=500][Beep=True]  oNe oF[Wait=500][Beep=True]  tHeM.[Color=White][Wait=500][Space=2]
-...Are you still there?[Wait=500][Space=2]
-[Color=Magenta][Beep=True]ThEr[Wait=500][Beep=True]e's fOo[Wait=500][Beep=True]d iN[Wait=500][Beep=True]  tHe dAm[Wait=500][Beep=True]p aReA[Wait=500][Beep=True],  tHe fAcTo[Wait=500][Beep=True]ry uSeD[Wait=500][Beep=True]  tO pRoDu[Wait=500][Beep=True]ce iT[Wait=500][Beep=True]  aS wElL.[Color=White][Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=104][Content=The person on the line can help you, they've been of great help to me as well.]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=113][Content=I'm as lost as you! What does any of that mean?]]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=114][Content=I didn't know anything about that!]]
-[Choice2=[NextScene=114][Content=This surely is a dream...]]</t>
-  </si>
-  <si>
-    <t>[Color=Magenta]It doesn't matter anymore.[Wait=500] Now that we are both together, we have to execute the plan I've been ploting.[Color=White][Wait=500][Space=2]
-Wait![Wait=500] What do you mean by plan?[Wait=500][Space=2]
-[Color=Magenta]Don't you want to stop all of this?[Color=White][Wait=500][Space=2]
-[Color=Magenta]If we just escape, he'll just create more of us. We have to stop this.[Color=White][Wait=500][Space=2]
-I...[Wait=500] That's true.[Wait=500][Space=2]
-I don't want other people to go through what we've been, no matter if they're clones or not.[Wait=500][Space=2]</t>
-  </si>
-  <si>
-    <t>[Choice1=[NextScene=119][Content=...Did they just throw me like garbage?]]
-[Choice2=[NextScene=119][Content=I guess it's for the best.]]
-[Choice3=[NextScene=119][Content=NOOOO COME BACK!]]</t>
-  </si>
-  <si>
-    <t>Wah-...[Wait=500] OH SH...[Wait=500][Space=2]
-[Color=Gray]*Whisper*[Color=White]... T-There's...[Wait=500] It's the thing that chased me in the vent...[Wait=500][Space=2]
-It's o-on the catwalks...[Wait=500][Space=2]
-...[Wait=500] Wait is that the...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]DoN[Wait=500][Beep=True]'t dO[Wait=500][Beep=True] aNyThInG[Wait=500][Beep=True] sTuPiD[Wait=500][Beep=True],  i'M[Wait=500][Beep=True] gOnNa[Wait=500][Beep=True] dIsTrAcT[Wait=500][Beep=True] tHeM.[Color=White][Wait=500][Space=2]</t>
+I'm outside. I can see the stairs I took to get in![Wait=500][Space=2]
+If I knew, I could've just kept going and climbed through this window![Wait=500][Space=2]</t>
+  </si>
+  <si>
+    <t>YES, IT'S OPENING![Wait=500][Space=2]
+There are stairs here.[Wait=500] I'm getting down there.[Wait=500][Space=2]
+...Oh my god...[Wait=500] It was such an intense-[Color=Gray]*SHKRRRRRRRRR*[Color=White]...[Wait=500] I'm so happy you were here to help me.[Wait=500][Space=2]</t>
   </si>
 </sst>
 </file>
@@ -10234,7 +10233,7 @@
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
       <c r="E32" s="8" t="s">
-        <v>620</v>
+        <v>603</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>386</v>
@@ -10265,7 +10264,7 @@
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
       <c r="E33" s="8" t="s">
-        <v>621</v>
+        <v>604</v>
       </c>
       <c r="F33" s="8" t="s">
         <v>106</v>
@@ -10761,7 +10760,7 @@
       </c>
       <c r="D50" s="7"/>
       <c r="E50" s="8" t="s">
-        <v>622</v>
+        <v>605</v>
       </c>
       <c r="F50" s="8" t="s">
         <v>118</v>
@@ -11245,7 +11244,7 @@
       <c r="C67" s="7"/>
       <c r="D67" s="7"/>
       <c r="E67" s="8" t="s">
-        <v>683</v>
+        <v>634</v>
       </c>
       <c r="F67" s="8" t="s">
         <v>129</v>
@@ -11272,7 +11271,7 @@
       <c r="C68" s="7"/>
       <c r="D68" s="7"/>
       <c r="E68" s="8" t="s">
-        <v>684</v>
+        <v>635</v>
       </c>
       <c r="F68" s="8" t="s">
         <v>130</v>
@@ -11299,7 +11298,7 @@
       <c r="C69" s="7"/>
       <c r="D69" s="7"/>
       <c r="E69" s="8" t="s">
-        <v>685</v>
+        <v>636</v>
       </c>
       <c r="F69" s="8" t="s">
         <v>131</v>
@@ -11385,7 +11384,7 @@
         <v>7</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>686</v>
+        <v>637</v>
       </c>
       <c r="F72" s="8" t="s">
         <v>134</v>
@@ -11415,7 +11414,7 @@
         <v>7</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>687</v>
+        <v>638</v>
       </c>
       <c r="F73" s="8" t="s">
         <v>135</v>
@@ -11443,7 +11442,7 @@
       <c r="C74" s="7"/>
       <c r="D74" s="7"/>
       <c r="E74" s="8" t="s">
-        <v>688</v>
+        <v>639</v>
       </c>
       <c r="F74" s="8" t="s">
         <v>136</v>
@@ -11607,7 +11606,7 @@
       <c r="C80" s="7"/>
       <c r="D80" s="7"/>
       <c r="E80" s="8" t="s">
-        <v>623</v>
+        <v>606</v>
       </c>
       <c r="F80" s="8" t="s">
         <v>140</v>
@@ -11802,7 +11801,7 @@
       <c r="C87" s="7"/>
       <c r="D87" s="7"/>
       <c r="E87" s="8" t="s">
-        <v>689</v>
+        <v>640</v>
       </c>
       <c r="F87" s="8" t="s">
         <v>147</v>
@@ -12412,7 +12411,7 @@
       <c r="C107" s="7"/>
       <c r="D107" s="7"/>
       <c r="E107" s="8" t="s">
-        <v>624</v>
+        <v>607</v>
       </c>
       <c r="F107" s="8" t="s">
         <v>161</v>
@@ -14418,7 +14417,7 @@
         <v>5</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>618</v>
+        <v>601</v>
       </c>
       <c r="F66" s="8" t="s">
         <v>245</v>
@@ -14452,7 +14451,7 @@
       </c>
       <c r="D67" s="7"/>
       <c r="E67" s="8" t="s">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="F67" s="8" t="s">
         <v>510</v>
@@ -15234,7 +15233,7 @@
         <v>10</v>
       </c>
       <c r="E93" s="8" t="s">
-        <v>682</v>
+        <v>633</v>
       </c>
       <c r="F93" s="8" t="s">
         <v>256</v>
@@ -16612,23 +16611,23 @@
       </c>
       <c r="D2" s="7"/>
       <c r="E2" s="8" t="s">
-        <v>593</v>
+        <v>781</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>595</v>
+        <v>782</v>
       </c>
       <c r="G2" s="23" t="str">
         <f t="shared" ref="G2:G33" si="0">"[Scene=" &amp; A2 &amp; IF(OR(B2&lt;&gt;"",C2&lt;&gt;"",D2&lt;&gt;""),CHAR(10),"") &amp; IF(B2&lt;&gt;"","[BeepBack=" &amp; B2 &amp; "]","") &amp; IF(C2&lt;&gt;"","[Connection=" &amp; C2 &amp; "]","") &amp; IF(D2&lt;&gt;"","[Timer=" &amp; D2 &amp; "]","") &amp; IF(E2&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E2 &amp; CHAR(10) &amp; "]","") &amp; IF(F2&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F2 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
         <v>[Scene=1
 [Connection=3]
 [Content=
-Yeah.[Wait=500] Of all places, the factory seems like the place I could find answers and the key to my escape.[Wait=500][Space=2]
+Yeah.[Wait=500] Of all places, the factory seems like the place where I could find answers and the key to my escape.[Wait=500][Space=2]
 I'll go there if I can.[Wait=500] Let's go.[Wait=500][Space=2]
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=2][NextSceneNoTrust=3][TrustNeed=50][Content=What exactly do you mean by key?]]
-[Choice2=[NextScene=9][NextSceneNoTrust=10][TrustNeed=50][Content=If you can? Would there be anything preventing you?]]
+[Choice2=[NextScene=9][NextSceneNoTrust=10][TrustNeed=50][Content=If you can? Would anything prevent you?]]
 ]
 ]</v>
       </c>
@@ -16644,7 +16643,7 @@
         <v>592</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>596</v>
+        <v>783</v>
       </c>
       <c r="G3" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16656,7 +16655,7 @@
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=8][Content=That's a pain of a situation for sure.]]
+[Choice1=[NextScene=8][Content=That's a tough situation for sure.]]
 ]
 ]</v>
       </c>
@@ -16669,16 +16668,16 @@
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
       <c r="E4" s="8" t="s">
-        <v>594</v>
+        <v>784</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="G4" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=3
 [Content=
-...[Wait=500] I hope I can find the fuse, why are you asking?[Wait=500][Space=2]
+...[Wait=500] I hope I can find the fuse. Why are you asking?[Wait=500][Space=2]
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
 ]
 [Choices=
@@ -16696,10 +16695,10 @@
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
       <c r="E5" s="8" t="s">
-        <v>625</v>
+        <v>785</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
       <c r="G5" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16707,7 +16706,7 @@
 [Content=
 I...[Wait=500] I'm just really stressed-...[Wait=500][Space=2]
 ...[Wait=500][Space=2]
-Listen, I might have found this phone but I don't feel like you're here to help...[Wait=500][Space=2]
+Listen, I might have found this phone, but I don't feel like you're here to help...[Wait=500][Space=2]
 I don't know, you've got to put yourself in my place a bit...[Wait=500][Space=2]
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
 ]
@@ -16727,10 +16726,10 @@
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="8" t="s">
-        <v>856</v>
+        <v>786</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>599</v>
+        <v>595</v>
       </c>
       <c r="G6" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16739,7 +16738,7 @@
 You-... I mean, you know-...[Wait=500] I get it.[Wait=500][Space=2]
 It's hard to handle some random person calling you for seemingly no reason.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
-But thanks for admitting that, I already feel safer if you're able to show a bit of self-awareness.[Wait=500][Space=2]
+But thanks for admitting that. I already feel safer if you're able to show a bit of self-awareness.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=6][Content=We're cool then!]]
@@ -16755,10 +16754,10 @@
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="8" t="s">
-        <v>600</v>
+        <v>787</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>726</v>
+        <v>663</v>
       </c>
       <c r="G7" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16766,10 +16765,10 @@
 [Content=
 We are.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
-I've arrived to the entrance, but I have to get through a fence.[Wait=500][Space=2]
+I've arrived at the entrance, but I have to get through a fence.[Wait=500][Space=2]
 It seems really fragile, so getting rid of it wouldn't be that hard.[Wait=500] That thing's already quite damaged.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
-Or I could go around, there's no reason for a building like this not to have some kind of backdoor.[Wait=500][Space=2]
+Or I could go around. There's no reason for a building like this not to have some kind of backdoor.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=16][Content=Yeah, go for a backdoor.]]
@@ -16786,10 +16785,10 @@
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="8" t="s">
-        <v>601</v>
+        <v>596</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>726</v>
+        <v>663</v>
       </c>
       <c r="G8" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16815,10 +16814,10 @@
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="8" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>727</v>
+        <v>664</v>
       </c>
       <c r="G9" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16845,24 +16844,24 @@
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
       <c r="E10" s="8" t="s">
-        <v>603</v>
+        <v>788</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>728</v>
+        <v>789</v>
       </c>
       <c r="G10" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=9
 [Content=
-There seem to be a fence in front of the main entrance.[Wait=500][Space=2]
-I probably could get around and find another way to enter.[Wait=500][Space=2]
+There seems to be a fence in front of the main entrance.[Wait=500][Space=2]
+I could probably go around and find another way in.[Wait=500][Space=2]
 But from this distance it looks really thin and rusted.[Wait=500][Space=2]
-I think pushing it down and getting over would prove quite easy.[Wait=500][Space=2]
+I think pushing it down and getting over would be quite easy.[Wait=500][Space=2]
 What do you think?[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=16][Content=Maybe you should go around, you might find something interesting.]]
-[Choice2=[NextScene=128][Content=Yeah let's do that!]]
+[Choice2=[NextScene=128][Content=Yeah, let's do that!]]
 ]
 ]</v>
       </c>
@@ -16875,10 +16874,10 @@
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
       <c r="E11" s="8" t="s">
-        <v>604</v>
+        <v>598</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>729</v>
+        <v>790</v>
       </c>
       <c r="G11" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16887,7 +16886,7 @@
 Do you expect something to block me?[Wait=500] Why would you ask me that?[Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=11][Content=I'm being serious. You wouldn't use conditional if you were sure.]]
+[Choice1=[NextScene=11][Content=I'm being serious. You wouldn't use a conditional if you were sure.]]
 [Choice2=[NextScene=12][Content=Is there something wrong?]]
 ]
 ]</v>
@@ -16901,21 +16900,21 @@
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
       <c r="E12" s="8" t="s">
-        <v>605</v>
+        <v>792</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>733</v>
+        <v>791</v>
       </c>
       <c r="G12" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=11
 [Content=
-I got myself a smart one, uh?[Wait=500][Space=2]
-I'm being conditional, cause there's a fence surrounding the entrance.[Wait=500][Space=2]
-Either have to get around or through it.[Wait=500][Space=2]
-]
-[Choices=
-[Choice1=[NextScene=16][Content=Get Around it.]]
+I got myself a smart one, huh?[Wait=500][Space=2]
+I'm being conditional because there's a fence surrounding the entrance.[Wait=500][Space=2]
+I either have to get around it or through it.[Wait=500][Space=2]
+]
+[Choices=
+[Choice1=[NextScene=16][Content=Get around it.]]
 [Choice2=[NextScene=128][Content=Get through it.]]
 ]
 ]</v>
@@ -16929,10 +16928,10 @@
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
       <c r="E13" s="8" t="s">
-        <v>855</v>
+        <v>769</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>730</v>
+        <v>793</v>
       </c>
       <c r="G13" s="23" t="str">
         <f t="shared" si="0"/>
@@ -16946,8 +16945,8 @@
 ]
 [Choices=
 [Choice1=[NextScene=13][TrustAdd=25][Content=I shouldn't have said those things.]]
-[Choice2=[NextScene=15][Content=It's hard for the both of us.]]
-[Choice3=[NextScene=15][Content=I get that, I'm sorry.]]
+[Choice2=[NextScene=15][Content=It's hard for both of us.]]
+[Choice3=[NextScene=15][Content=I get that. I'm sorry.]]
 ]
 ]</v>
       </c>
@@ -16960,21 +16959,21 @@
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
       <c r="E14" s="8" t="s">
-        <v>854</v>
+        <v>795</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>731</v>
+        <v>794</v>
       </c>
       <c r="G14" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=13
 [Content=
 I-...[Wait=500] I get it.[Wait=500][Space=2]
-It's good you're able to put yourself in my place a bit.[Wait=500] Thanks for acknowledging it.[Wait=500][Space=2]
+It's good that you're able to put yourself in my place a bit.[Wait=500] Thanks for acknowledging it.[Wait=500][Space=2]
 I'm starting to feel a bit more hopeful about getting out of here if you're on my side.[Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=14][Content=Yeah, let's not rest.]]
+[Choice1=[NextScene=14][Content=Yeah, let's not slow down.]]
 ]
 ]</v>
       </c>
@@ -16987,19 +16986,19 @@
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="8" t="s">
-        <v>606</v>
+        <v>796</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>732</v>
+        <v>665</v>
       </c>
       <c r="G15" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=14
 [Content=
-I'm getting there.[Wait=500] But I can already see the place's protected by a fence.[Wait=500][Space=2]
+I'm getting there.[Wait=500] But I can already see the place is protected by a fence.[Wait=500][Space=2]
 It isn't a big deal, I could probably find another entrance.[Wait=500][Space=2]
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
-The metal looks brittle. I probably could bend it down and get over it.[Wait=500][Space=2]
+The metal looks brittle. I could probably bend it down and get over it.[Wait=500][Space=2]
 What do you think?[Wait=500][Space=2]
 ]
 [Choices=
@@ -17017,18 +17016,18 @@
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
       <c r="E16" s="8" t="s">
-        <v>853</v>
+        <v>797</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>734</v>
+        <v>666</v>
       </c>
       <c r="G16" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=15
 [Content=
-Hm-...[Wait=500] Anyways, there's a fence blocking the way to the main entrance.[Wait=500][Space=2]
-I can either try and get through or go around.[Wait=500][Space=2]
-It looks weak enough to be bent, but this kind of buildings tend to have backdoors.[Wait=500][Space=2]
+Hm-...[Wait=500] Anyway, there's a fence blocking the way to the main entrance.[Wait=500][Space=2]
+I can either try to get through it or go around.[Wait=500][Space=2]
+It looks weak enough to be bent, but buildings like this usually have backdoors.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=16][Content=I'd go around.]]
@@ -17045,22 +17044,22 @@
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
       <c r="E17" s="8" t="s">
-        <v>607</v>
+        <v>798</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>735</v>
+        <v>799</v>
       </c>
       <c r="G17" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=16
 [Content=
-Yeah. The main entrance might be trapped, I'd rather find another way.[Wait=500][Space=2]
+Yeah. The main entrance might be trapped. I'd rather find another way.[Wait=500][Space=2]
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
-Thinking outside the box might be the way to avoid some of the-[Wait=500] psycho keeping me here.[Wait=500][Space=2]
+Thinking outside the box might be the way to avoid some of the-...[Wait=500] psycho keeping me here.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=17][Content=Exactly my thought.]]
-[Choice2=[NextScene=18][Content=Let's hope backdoors aren't either...]]
+[Choice2=[NextScene=18][Content=Let's hope the backdoors aren't either...]]
 ]
 ]</v>
       </c>
@@ -17073,23 +17072,23 @@
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="8" t="s">
-        <v>608</v>
+        <v>802</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>736</v>
+        <v>800</v>
       </c>
       <c r="G18" s="23" t="str">
         <f>"[Scene=" &amp; A18 &amp; IF(OR(B18&lt;&gt;"",C18&lt;&gt;"",D18&lt;&gt;""),CHAR(10),"") &amp; IF(B18&lt;&gt;"","[BeepBack=" &amp; B18 &amp; "]","") &amp; IF(C18&lt;&gt;"","[Connection=" &amp; C18 &amp; "]","") &amp; IF(D18&lt;&gt;"","[Timer=" &amp; D18 &amp; "]","") &amp; IF(E19&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E19 &amp; CHAR(10) &amp; "]","") &amp; IF(F18&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F18 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
         <v>[Scene=17
 [Content=
 ...[Wait=500] No need to make me doubt...[Wait=500][Space=2]
-If that bastard really wants me to die I'm screwed anyways. Might as well minimize the risk.[Wait=500][Space=2]
+If that bastard really wants me to die, I'm screwed anyway. Might as well minimize the risk.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 Who knows...[Wait=500] He might be an idiot.[Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=19][Content=Not like you'd find anything alive anyways.]]
-[Choice2=[NextScene=19][Content=Zoo are smelly.]]
+[Choice1=[NextScene=19][Content=Not like you'd find anything alive anyway.]]
+[Choice2=[NextScene=19][Content=Zoos are smelly.]]
 ]
 ]</v>
       </c>
@@ -17102,26 +17101,26 @@
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="8" t="s">
-        <v>609</v>
+        <v>803</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>737</v>
+        <v>801</v>
       </c>
       <c r="G19" s="23" t="str">
         <f>"[Scene=" &amp; A19 &amp; IF(OR(B19&lt;&gt;"",C19&lt;&gt;"",D19&lt;&gt;""),CHAR(10),"") &amp; IF(B19&lt;&gt;"","[BeepBack=" &amp; B19 &amp; "]","") &amp; IF(C19&lt;&gt;"","[Connection=" &amp; C19 &amp; "]","") &amp; IF(D19&lt;&gt;"","[Timer=" &amp; D19 &amp; "]","") &amp; IF(E20&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E20 &amp; CHAR(10) &amp; "]","") &amp; IF(F19&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F19 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
         <v>[Scene=18
 [Content=
-Talking about the zoo, guess what.[Wait=500] It's awfully close to this place.[Wait=500][Space=2]
-I can see the inside of the enclosures from there.[Wait=500][Space=2]
+Speaking of the zoo, guess what.[Wait=500] It's awfully close to this place.[Wait=500][Space=2]
+I can see inside the enclosures from here.[Wait=500][Space=2]
 Whoever designed this city should be fired.[Wait=500] Or even set on fire.[Wait=500][Space=2]
-Because I'm stuck inside their shittily designed city.[Wait=500][Space=2]
+Because I'm stuck inside their terribly designed city.[Wait=500][Space=2]
 That prick.[Wait=500][Space=2]
 [Color=Magenta][Beep=True][Color=Gray]*Distorted chuckle*[Color=White]...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]YoU'[Wait=500][Beep=True]rE bEt[Wait=500][Beep=True]tEr hErE[Wait=500][Beep=True]  wItH mE[Wait=500][Beep=True]  tHaN aLo[Wait=500][Beep=True]nE iN[Wait=500][Beep=True]  tHe zOo.[Color=White][Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=19][Content=I mean... This island has a zoo and a museum but no hopistal.]]
-[Choice2=[NextScene=20][Content=I'd doubt that. They probably built this place.]]
+[Choice1=[NextScene=19][Content=I mean... This island has a zoo and a museum, but no hospital.]]
+[Choice2=[NextScene=20][Content=I doubt that. They probably built this place.]]
 ]
 ]</v>
       </c>
@@ -17134,19 +17133,19 @@
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="8" t="s">
-        <v>610</v>
+        <v>804</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>738</v>
+        <v>667</v>
       </c>
       <c r="G20" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=19
 [Content=
-Talking about the zoo, guess what.[Wait=500] It's awfully close to this place.[Wait=500][Space=2]
-I can see the inside of the enclosures from there.[Wait=500][Space=2]
+Speaking of the zoo, guess what.[Wait=500] It's awfully close to this place.[Wait=500][Space=2]
+I can see inside the enclosures from here.[Wait=500][Space=2]
 Whoever designed this city should be fired.[Wait=500] Or even set on fire.[Wait=500][Space=2]
-Because I'm stuck inside their shittily designed city.[Wait=500][Space=2]
+Because I'm stuck inside their terribly designed city.[Wait=500][Space=2]
 That prick.[Wait=500][Space=2]
 [Color=Magenta][Beep=True][Color=Gray]*Distorted chuckle*[Color=White]...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]YoU'[Wait=500][Beep=True]rE bEt[Wait=500][Beep=True]tEr hErE[Wait=500][Beep=True]  wItH mE[Wait=500][Beep=True]  tHaN aLo[Wait=500][Beep=True]nE iN[Wait=500][Beep=True]  tHe zOo.[Color=White][Wait=500][Space=2]
@@ -17166,18 +17165,18 @@
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
       <c r="E21" s="8" t="s">
-        <v>850</v>
+        <v>805</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>739</v>
+        <v>668</v>
       </c>
       <c r="G21" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=20
 [Content=
 Wouldn't be trying to defend them, would we?[Wait=500][Space=2]
-Errm-...[Wait=500] Anyways.[Wait=500][Space=2]
-Didn't realize the zoo was that close to the factory before.[Wait=500] Civil engineering failed some.[Wait=500][Space=2]
+Errm-...[Wait=500] Anyway.[Wait=500][Space=2]
+Didn't realize the zoo was that close to the factory before.[Wait=500] Civil engineering failed somewhere.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]DaN[Wait=500][Beep=True]gErOuS[Wait=500][Beep=True]  pLa[Wait=500][Beep=True]cE.[Wait=500][Beep=True]  ExpEr[Wait=500][Beep=True]iMeNtS.[Color=White][Wait=500][Space=2]
 ]
 [Choices=
@@ -17195,10 +17194,10 @@
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
       <c r="E22" s="8" t="s">
-        <v>611</v>
+        <v>806</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>740</v>
+        <v>669</v>
       </c>
       <c r="G22" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17207,7 +17206,7 @@
 Empty drums, debris, nothing but the usual shit.[Wait=500][Space=2]
 Nowhere else to go, you see, so for now I'll keep looking.[Wait=500][Space=2]
 Stressed out and hungry I feel, still haven't got anything to eat.[Wait=500][Space=2]
-I could really use oat meal, or anything that would get me going.[Wait=500][Space=2]
+I could really use oatmeal, or anything that would get me going.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=22][Content=I'm sure you'll find something to gnaw on once inside.]]
@@ -17226,10 +17225,10 @@
       </c>
       <c r="D23" s="7"/>
       <c r="E23" s="8" t="s">
-        <v>612</v>
+        <v>599</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>741</v>
+        <v>670</v>
       </c>
       <c r="G23" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17257,21 +17256,21 @@
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
       <c r="E24" s="8" t="s">
-        <v>869</v>
+        <v>807</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>742</v>
+        <v>671</v>
       </c>
       <c r="G24" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=23
 [Content=
-M-...[Wait=500] Me?[Wait=500] As I've said before I-...[Wait=500][Space=2]
+M-...[Wait=500] Me?[Wait=500] As I've said before, I-...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]OnE[Wait=500][Beep=True]  oF tHe[Wait=500][Beep=True]  pReVi[Wait=500][Beep=True]oUs.[Color=White][Wait=500] [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]I'M[Wait=500][Beep=True]  hErE tO[Wait=500][Beep=True]  hElP yOu.[Wait=500][Beep=True]  I'M aBlE[Wait=500][Beep=True]  tO cOmMu[Wait=500][Beep=True]nIcAtE tHrOuGh[Wait=500][Beep=True]  tHe dEsA[Wait=500][Beep=True]fEcTeD cOnTrOl.[Color=White][Wait=500][Space=2]
 [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
-[Color=Magenta][Beep=True]SuR[Wait=500]viVoR[Wait=500][Beep=True],  i'M tRy[Wait=500][Beep=True]iNg tO gEt[Wait=500][Beep=True]  oThErS oUt[Wait=500][Beep=True]  oF hIs[Wait=500][Beep=True]  tRaPs.[Color=White][Wait=500][Space=2]
-Once again, I do NOT know why I'm here nor about any kind of experiments, just help me, alright?[Wait=500][Space=2]
+[Color=Magenta][Beep=True]SuR[Wait=500]viVoR[Wait=500][Beep=True],  I'M tRy[Wait=500][Beep=True]iNg tO gEt[Wait=500][Beep=True]  oThErS oUt[Wait=500][Beep=True]  oF hIs[Wait=500][Beep=True]  tRaPs.[Color=White][Wait=500][Space=2]
+Once again, I do NOT know why I'm here nor about any kind of experiments. Just help me, alright?[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=24][Content=I'm not talking to you, there's someone in the call.]]
@@ -17288,10 +17287,10 @@
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
       <c r="E25" s="8" t="s">
-        <v>851</v>
+        <v>767</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>743</v>
+        <v>672</v>
       </c>
       <c r="G25" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17317,10 +17316,10 @@
       </c>
       <c r="D26" s="7"/>
       <c r="E26" s="8" t="s">
-        <v>613</v>
+        <v>808</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>744</v>
+        <v>673</v>
       </c>
       <c r="G26" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17330,8 +17329,8 @@
 Of course I'm going to worry!!![Wait=500][Space=2]
 You're giving me no explanation after saying shit about some experiment. Are there more people with you?[Wait=500][Space=2]
 ...[Wait=500][Space=2]
-You're always alternating between reinsuring and cryptic, talking to the fucking voices now![Wait=500][Space=2]
-Am-[Wait=500] Am I a game to you?[Wait=500] Are you going to fucking tell?![Wait=500][Space=2]
+You're always alternating between reassuring and cryptic, talking to the fucking voices now![Wait=500][Space=2]
+Am-...[Wait=500] Am I a game to you?[Wait=500] Are you going to fucking tell me?![Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=22][Content=Just keep walking, for fuck's sake.]]
@@ -17351,10 +17350,10 @@
       </c>
       <c r="D27" s="7"/>
       <c r="E27" s="8" t="s">
-        <v>614</v>
+        <v>809</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>745</v>
+        <v>674</v>
       </c>
       <c r="G27" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17365,7 +17364,7 @@
 Uh...[Wait=500] Nevermind. I'm not even gonna ask anymore.[Wait=500][Space=2]
 .[Wait=500].[Wait=500].[Wait=500][Space=2]
 But should we reaaally trust them?[Wait=500][Space=2]
-I mean, why would anyone other than the person behind all of this try to talk to you.[Wait=500][Space=2]
+I mean, why would anyone other than the person behind all of this try to talk to you?[Wait=500][Space=2]
 And why can't I hear them?[Wait=500][Space=2]
 ]
 [Choices=
@@ -17383,10 +17382,10 @@
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
       <c r="E28" s="8" t="s">
-        <v>615</v>
+        <v>810</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>746</v>
+        <v>811</v>
       </c>
       <c r="G28" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17396,12 +17395,12 @@
 Great.[Wait=500][Space=2]
 That either means a helping hand... or extra danger.[Wait=500][Space=2]
 As if all of this needed more complexity.[Wait=500][Space=2]
-So they're going to help you guide me if I understood well.[Wait=500][Space=2]
+So they're going to help you guide me, if I understood well.[Wait=500][Space=2]
 Doesn't sound like a trap.[Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=28][Content=You're screwed either way if that's the case. Might as well tempt it.]]
-[Choice2=[NextScene=28][NextSceneNoTrust=29][TrustNeed=50][Content=I'm still there. Don't worry.]]
+[Choice1=[NextScene=28][Content=You're screwed either way if that's the case. Might as well tempt fate.]]
+[Choice2=[NextScene=28][NextSceneNoTrust=29][TrustNeed=50][Content=I'm still here. Don't worry.]]
 [Choice3=[NextScene=29][Content=We'll see. Let's try to listen to them for now.]]
 ]
 ]</v>
@@ -17415,10 +17414,10 @@
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
       <c r="E29" s="8" t="s">
-        <v>616</v>
+        <v>600</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>747</v>
+        <v>675</v>
       </c>
       <c r="G29" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17443,10 +17442,10 @@
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="8" t="s">
-        <v>852</v>
+        <v>768</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>748</v>
+        <v>676</v>
       </c>
       <c r="G30" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17471,10 +17470,10 @@
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
       <c r="E31" s="8" t="s">
-        <v>617</v>
+        <v>812</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>741</v>
+        <v>670</v>
       </c>
       <c r="G31" s="23" t="str">
         <f t="shared" si="0"/>
@@ -17486,7 +17485,7 @@
 Writings.[Wait=500][Space=2]
 Writings on the wall.[Wait=500] Please.[Wait=500] Why?[Wait=500][Space=2]
 Oh no, don't tell me these are creepy letters-...[Wait=500][Space=2]
-On the wall.[Wait=500] I'm so sick.[Wait=500][Space=2]
+On the wall.[Wait=500] I'm so sick of this.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=31][Content=What does it say?]]
@@ -17502,20 +17501,20 @@
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
       <c r="E32" s="8" t="s">
-        <v>626</v>
+        <v>813</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>749</v>
+        <v>677</v>
       </c>
       <c r="G32" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=31
 [Content=
 "THEY FED ME MY OWN SELF!"...[Wait=500][Space=2]
-I...[Wait=500] Really don't want to discover what happened on this island.[Wait=500][Space=2]
+I...[Wait=500] really don't want to discover what happened on this island.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 I'm almost surprised that wasn't written in blood. Although blue blood might be a thing on this island.[Wait=500][Space=2]
-I dont know, I'm not a...[Wait=500] ...blood[Wait=500] ...scientist.[Wait=500][Space=2]
+I don't know, I'm not a...[Wait=500] ...blood[Wait=500] ...scientist.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=32][Content=What does that mean?]]
@@ -17532,20 +17531,20 @@
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
       <c r="E33" s="8" t="s">
-        <v>627</v>
+        <v>814</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>750</v>
+        <v>678</v>
       </c>
       <c r="G33" s="23" t="str">
         <f t="shared" si="0"/>
         <v>[Scene=32
 [Content=
-It really feels like some edgy shit a fourteen years old would write.[Wait=500][Space=2]
+It really feels like some edgy shit a fourteen-year-old would write.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 But I'm still shaken up despite how ridiculous that is...[Wait=500][Space=2]
-Like...[Wait=500] Someone wrote that in some place in the middle of the ocean.[Wait=500][Space=2]
-I'm not gonna mess with a fourteen year old, not matter how angsty.[Wait=500][Space=2]
+Like...[Wait=500] someone wrote that in some place in the middle of the ocean.[Wait=500][Space=2]
+I'm not gonna mess with a fourteen-year-old, no matter how angsty.[Wait=500][Space=2]
 If they're ready to cross the ocean for a joke.[Wait=500][Space=2]
 ]
 [Choices=
@@ -17562,10 +17561,10 @@
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
       <c r="E34" s="8" t="s">
-        <v>628</v>
+        <v>608</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>751</v>
+        <v>679</v>
       </c>
       <c r="G34" s="23" t="str">
         <f t="shared" ref="G34:G65" si="1">"[Scene=" &amp; A34 &amp; IF(OR(B34&lt;&gt;"",C34&lt;&gt;"",D34&lt;&gt;""),CHAR(10),"") &amp; IF(B34&lt;&gt;"","[BeepBack=" &amp; B34 &amp; "]","") &amp; IF(C34&lt;&gt;"","[Connection=" &amp; C34 &amp; "]","") &amp; IF(D34&lt;&gt;"","[Timer=" &amp; D34 &amp; "]","") &amp; IF(E34&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E34 &amp; CHAR(10) &amp; "]","") &amp; IF(F34&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F34 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -17589,16 +17588,16 @@
       <c r="C35" s="7"/>
       <c r="D35" s="7"/>
       <c r="E35" s="8" t="s">
-        <v>629</v>
+        <v>815</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>752</v>
+        <v>680</v>
       </c>
       <c r="G35" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=34
 [Content=
-Well me neither.[Wait=500][Space=2]
+Well, me neither.[Wait=500][Space=2]
 Let's just move on knowing some lunatic could jump me any minute.[Wait=500][Space=2]
 No big deal.[Wait=500][Space=2]
 ]
@@ -17617,16 +17616,16 @@
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
       <c r="E36" s="8" t="s">
-        <v>630</v>
+        <v>816</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>753</v>
+        <v>681</v>
       </c>
       <c r="G36" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=35
 [Content=
-So no big deal as I said.[Wait=500][Space=2]
+So no big deal, as I said.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 Good news, I just stumbled onto what seems to be...[Wait=500] fire escape stairs?[Wait=500][Space=2]
 I'm positive these lead inside the building.[Wait=500][Space=2]
@@ -17646,17 +17645,17 @@
       <c r="C37" s="7"/>
       <c r="D37" s="7"/>
       <c r="E37" s="8" t="s">
-        <v>857</v>
+        <v>817</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>754</v>
+        <v>818</v>
       </c>
       <c r="G37" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=36
 [Content=
 I'm cl-...[Wait=500] Oh-...[Wait=500][Space=2]
-Hold on a minute will you... I'm not a...[Wait=500] ...stair climbing[Wait=500] ...athlete.[Wait=500][Space=2]
+Hold on a minute, will you... I'm not a...[Wait=500] ...stair-climbing[Wait=500] ...athlete.[Wait=500][Space=2]
 I'm...[Wait=500] getting there...[Wait=500][Space=2]
 Huff... huff...[Wait=500][Space=2]
 .[Wait=500].[Wait=500].[Wait=500][Space=2]
@@ -17664,7 +17663,7 @@
 ]
 [Choices=
 [Choice1=[NextScene=37][Content=...]]
-[Choice2=[NextScene=37][Content=What?J]]
+[Choice2=[NextScene=37][Content=What?]]
 ]
 ]</v>
       </c>
@@ -17677,18 +17676,18 @@
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="8" t="s">
-        <v>631</v>
+        <v>819</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>755</v>
+        <v>682</v>
       </c>
       <c r="G38" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=37
 [Content=
 Remember when I talked about luck being on my side?[Wait=500] Shouldn't have said that.[Wait=500][Space=2]
-It's fricking closed. By a [Color=Green]3-digits[Color=White] pad, which isn't high protection by any means.[Wait=500][Space=2]
-but I'd rather go back to the entrance than spend my time here.[Wait=500][Space=2]
+It's freaking closed. By a [Color=Green]3-digit[Color=White] pad, which isn't high protection by any means.[Wait=500][Space=2]
+But I'd rather go back to the entrance than spend my time here.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=38][Content=Let's go back and push that fence.]]
@@ -17705,10 +17704,10 @@
       <c r="C39" s="7"/>
       <c r="D39" s="7"/>
       <c r="E39" s="8" t="s">
-        <v>632</v>
+        <v>609</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>756</v>
+        <v>683</v>
       </c>
       <c r="G39" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17736,22 +17735,21 @@
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
       <c r="E40" s="8" t="s">
-        <v>633</v>
+        <v>820</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>756</v>
+        <v>683</v>
       </c>
       <c r="G40" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=39
 [Content=
 If there's a clue anywhere, it'd be inside.[Wait=500][Space=2]
-Good thing the door has a window[Wait=500], worse case scenario I might just smash it and slither in like a...[Wait=500][Space=2]
-...Tapeworm.[Wait=500][Space=2]
-The place looks like it was left in a hurry a dozen of year ago.[Wait=500][Space=2]
+Good thing the door has a window[Wait=500], worst case scenario I might just smash it and slither in like a tapeworm.[Wait=500][Space=2]
+The place looks like it was left in a hurry a dozen years ago.[Wait=500][Space=2]
 Someone even smeared their coffee on the carpet.[Wait=500][Space=2]
 And what's that?[Wait=500][Space=2]
-A random wrench laying on the ground?[Wait=500] Now that's a motivator. Might have to bash some skull.[Wait=500][Space=2]
+A random wrench lying on the ground?[Wait=500] Now that's a motivator. Might have to bash some skulls.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=40][Content=What's on the left?]]
@@ -17768,10 +17766,10 @@
       <c r="C41" s="7"/>
       <c r="D41" s="7"/>
       <c r="E41" s="8" t="s">
-        <v>641</v>
+        <v>821</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>757</v>
+        <v>684</v>
       </c>
       <c r="G41" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17779,7 +17777,7 @@
 [Content=
 Huuuh...[Wait=500] There's a cork board with a bunch of blank pieces of paper pinned onto it...[Wait=500][Space=2]
 And a literal passcode note. [Color=Green]7734[Color=White].[Wait=500][Space=2]
-Which is 4 digits so it's useless, are you kidding me.[Wait=500][Space=2]
+Which is 4 digits so it's useless. Are you kidding me.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=41][Content=Definitely there on purpose! What's on the right?]]
@@ -17795,10 +17793,10 @@
       <c r="C42" s="7"/>
       <c r="D42" s="7"/>
       <c r="E42" s="8" t="s">
-        <v>640</v>
+        <v>822</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>758</v>
+        <v>685</v>
       </c>
       <c r="G42" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17806,7 +17804,7 @@
 [Content=
 The only thing on the right wall is a big mirror with...[Wait=500][Space=2]
 An [Color=Green]upside-down calculator[Color=White] taped onto it.[Wait=500][Space=2]
-You know, the old ones we had back in school, those ones with the segmented digits.[Wait=500][Space=2]
+You know, the old ones we had back in school, those with the segmented digits.[Wait=500][Space=2]
 Nostalgic, but not helping me that much.[Wait=500][Space=2]
 ]
 [Choices=
@@ -17823,10 +17821,10 @@
       <c r="C43" s="7"/>
       <c r="D43" s="7"/>
       <c r="E43" s="8" t="s">
-        <v>639</v>
+        <v>823</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>759</v>
+        <v>686</v>
       </c>
       <c r="G43" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17834,8 +17832,8 @@
 [Content=
 On the right?[Wait=500] There's a mirror on the wall, and it has...[Wait=500][Space=2]
 An [Color=Green]upside-down calculator[Color=White] taped onto it.[Wait=500][Space=2]
-Old school ones, with segmented digit displays.[Wait=500][Space=2]
-It's cool that it brings memories, but it's so useless right now.[Wait=500][Space=2]
+Old-school ones, with segmented digit displays.[Wait=500][Space=2]
+It's cool that it brings back memories, but it's so useless right now.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=43][Content=Too specific to mean nothing, look to the left.]]
@@ -17851,18 +17849,18 @@
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
       <c r="E44" s="8" t="s">
-        <v>638</v>
+        <v>824</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>760</v>
+        <v>687</v>
       </c>
       <c r="G44" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=43
 [Content=
 There's a cork board covered in blank papers.[Wait=500][Space=2]
-Oh yeah, also the passcode. [Color=Green]7734[Color=White].[Wait=500][Space=2]
-Hold it! The lockpad is [Color=Green]3 digits[Color=White] so it won't fit! [Color=Gray]*Demented laugh*[Color=White]...[Wait=500][Space=2]
+Oh yeah, also the passcode: [Color=Green]7734[Color=White].[Wait=500][Space=2]
+Hold it! The lockpad is [Color=Green]3 digits[Color=White], so it won't fit! [Color=Gray]*Demented laugh*[Color=White]...[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=44][Content=Calm down and try this.]]
@@ -17878,10 +17876,10 @@
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
       <c r="E45" s="8" t="s">
-        <v>634</v>
+        <v>610</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>761</v>
+        <v>688</v>
       </c>
       <c r="G45" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17906,10 +17904,10 @@
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="8" t="s">
-        <v>635</v>
+        <v>611</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>762</v>
+        <v>689</v>
       </c>
       <c r="G46" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17934,10 +17932,10 @@
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
       <c r="E47" s="8" t="s">
-        <v>635</v>
+        <v>611</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>763</v>
+        <v>690</v>
       </c>
       <c r="G47" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17962,10 +17960,10 @@
       <c r="C48" s="7"/>
       <c r="D48" s="7"/>
       <c r="E48" s="8" t="s">
-        <v>635</v>
+        <v>611</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>764</v>
+        <v>691</v>
       </c>
       <c r="G48" s="23" t="str">
         <f t="shared" si="1"/>
@@ -17990,10 +17988,10 @@
       <c r="C49" s="7"/>
       <c r="D49" s="7"/>
       <c r="E49" s="8" t="s">
-        <v>635</v>
+        <v>611</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>765</v>
+        <v>692</v>
       </c>
       <c r="G49" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18018,10 +18016,10 @@
       <c r="C50" s="7"/>
       <c r="D50" s="7"/>
       <c r="E50" s="8" t="s">
-        <v>636</v>
+        <v>612</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>766</v>
+        <v>693</v>
       </c>
       <c r="G50" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18046,10 +18044,10 @@
       <c r="C51" s="7"/>
       <c r="D51" s="7"/>
       <c r="E51" s="8" t="s">
-        <v>637</v>
+        <v>825</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>767</v>
+        <v>694</v>
       </c>
       <c r="G51" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18057,7 +18055,7 @@
 [Content=
 Nope. Not opening.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]NeVe[Wait=500][Beep=True]r fLiP[Wait=500][Beep=True]peD a[Wait=500][Beep=True]  cAlC[Wait=500][Beep=True]uLaTo[Wait=500][Beep=True]r bEf[Wait=500][Beep=True]oRe?[Color=White][Wait=500][Space=2]
-7734, upside-down calculator, can you work something out with this?.[Wait=500][Space=2]
+7734, upside-down calculator... can you work something out with this?[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=44][Content=Okay, let's try something else.]]
@@ -18073,18 +18071,18 @@
       <c r="C52" s="7"/>
       <c r="D52" s="7"/>
       <c r="E52" s="8" t="s">
-        <v>642</v>
+        <v>826</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>768</v>
+        <v>695</v>
       </c>
       <c r="G52" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=51
 [Content=
 Oh yes![Wait=500] I remember that![Wait=500][Space=2]
-Never thought something that stupid could come in handy in a life or death situation.[Wait=500][Space=2]
-Well of course I did but come on![Wait=500][Space=2]
+Never thought something that stupid could come in handy in a life-or-death situation.[Wait=500][Space=2]
+Well of course I did, but come on![Wait=500][Space=2]
 That's just so ridiculous, the person who designed this puzzle has to be a moron.[Wait=500][Space=2]
 ]
 [Choices=
@@ -18103,17 +18101,17 @@
       <c r="C53" s="7"/>
       <c r="D53" s="7"/>
       <c r="E53" s="8" t="s">
-        <v>643</v>
+        <v>827</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>769</v>
+        <v>696</v>
       </c>
       <c r="G53" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=52
 [Content=
-Wow, well guess they're not so bad, everything's good in the best of worlds![Wait=500][Space=2]
-Sorry, I'm being way too sarcastic, thank them.[Wait=500] But also ask them how they knew the passcode.[Wait=500][Space=2]
+Wow, well I guess they're not so bad. Everything's good in the best of worlds![Wait=500][Space=2]
+Sorry, I'm being way too sarcastic. Thank them.[Wait=500] But also ask them how they knew the passcode.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=53][Content=They simply hinted m-.]]
@@ -18130,17 +18128,17 @@
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
       <c r="E54" s="8" t="s">
-        <v>644</v>
+        <v>828</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>770</v>
+        <v>697</v>
       </c>
       <c r="G54" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=53
 [Content=
-Wow, no need to be rude about it-...[Wait=500][Space=2]
-I'm more focused on survival than some stupid calculator cypher.[Wait=500][Space=2]
+Wow, no need to be rude about it...[Wait=500][Space=2]
+I'm more focused on survival than some stupid calculator cipher.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=54][Content=You don't seem to str-.]]
@@ -18157,21 +18155,21 @@
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
       <c r="E55" s="8" t="s">
-        <v>645</v>
+        <v>829</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>771</v>
+        <v>698</v>
       </c>
       <c r="G55" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=54
 [Content=
-GOOD![Wait=500] Let's not waste anymore time![Wait=500][Space=2]
+GOOD![Wait=500] Let's not waste any more time![Wait=500][Space=2]
 We're finally in after all![Wait=500][Space=2]
 Maybe going through the main entrance would have been faster, but at least I got to breathe fresh air.[Wait=500][Space=2]
 [Color=Gray]*THUD*[Color=White]...[Wait=500][Space=2]
 Oh, yes.[Wait=500][Space=2]
-I also get to pick that beautiful wrench.[Wait=500][Space=2]
+I also get to pick up that beautiful wrench.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=55][Content=Do you even know how to use it?]]
@@ -18189,10 +18187,10 @@
       <c r="C56" s="7"/>
       <c r="D56" s="7"/>
       <c r="E56" s="8" t="s">
-        <v>858</v>
+        <v>830</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>772</v>
+        <v>699</v>
       </c>
       <c r="G56" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18201,7 +18199,7 @@
 B-...[Wait=500] BAHAHAHA-...[Wait=500][Space=2]
 Who do you take me for?[Wait=500] I'm not a toddler, I can tighten bolts![Wait=500][Space=2]
 My kidnapper might just come and catch these hands right now.[Wait=500][Space=2]
-With this bad boy with me, I ain't loosing to no monster.[Wait=500][Space=2]
+With this bad boy with me, I ain't losing to no monster.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 ]
 [Choices=
@@ -18219,10 +18217,10 @@
       <c r="C57" s="7"/>
       <c r="D57" s="7"/>
       <c r="E57" s="8" t="s">
-        <v>646</v>
+        <v>831</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>773</v>
+        <v>700</v>
       </c>
       <c r="G57" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18230,8 +18228,8 @@
 [Content=
 Absolutely![Wait=500][Space=2]
 ...[Wait=500][Space=2]
-...I don't know how to put it but it seems...[Wait=500] advanced.[Wait=500][Space=2]
-This ain't ordinary wrench. It's heavier and equiped with some kind of display.[Wait=500][Space=2]
+...I don't know how to put it, but it seems...[Wait=500] advanced.[Wait=500][Space=2]
+This ain't an ordinary wrench. It's heavier and equipped with some kind of display.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 I might take it home.[Wait=500][Space=2]
 ]
@@ -18250,10 +18248,10 @@
       <c r="C58" s="7"/>
       <c r="D58" s="7"/>
       <c r="E58" s="8" t="s">
-        <v>647</v>
+        <v>832</v>
       </c>
       <c r="F58" s="8" t="s">
-        <v>774</v>
+        <v>701</v>
       </c>
       <c r="G58" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18264,7 +18262,7 @@
 [Color=Gray]*Hammering sounds*[Color=White]...[Wait=500][Space=2]
 But that's a puzzle for another day, I've got places to be.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
-That thing packs a severe punch, I got it opened in a few hits.[Wait=500][Space=2]
+That thing packs a serious punch, I got it open in a few hits.[Wait=500][Space=2]
 [Color=Gray]*Door creaks*[Color=White]...[Wait=500][Space=2]
 ]
 [Choices=
@@ -18282,10 +18280,10 @@
       <c r="C59" s="7"/>
       <c r="D59" s="7"/>
       <c r="E59" s="8" t="s">
-        <v>859</v>
+        <v>833</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>775</v>
+        <v>702</v>
       </c>
       <c r="G59" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18295,7 +18293,7 @@
 [Color=Gray]*Voice echoes*[Color=White]...[Wait=500][Space=2]
 This place is huge.[Wait=500] I'm in a hallway so long I can't see the other side.[Wait=500][Space=2]
 It really feels like I'm standing in front of a void.[Wait=500][Space=2]
-With only the echo of my voice proving me there's something that way.[Wait=500][Space=2]
+With only the echo of my voice proving there's something that way.[Wait=500][Space=2]
 And these big tubes...[Wait=500] This place isn't for making shoes, that's for sure.[Wait=500][Space=2]
 ]
 [Choices=
@@ -18313,10 +18311,10 @@
       <c r="C60" s="7"/>
       <c r="D60" s="7"/>
       <c r="E60" s="8" t="s">
-        <v>690</v>
+        <v>834</v>
       </c>
       <c r="F60" s="8" t="s">
-        <v>776</v>
+        <v>703</v>
       </c>
       <c r="G60" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18324,7 +18322,7 @@
 [Content=
 About my size.[Wait=500] They're all connected to a dense net of wires on the ground.[Wait=500][Space=2]
 Almost makes it hard to navigate.[Wait=500][Space=2]
-Also smells quite odd.[Wait=500] It's both off-putting...[Wait=500] and weirdly conforting...[Wait=500][Space=2]
+Also smells quite odd.[Wait=500] It's both off-putting...[Wait=500] and weirdly comforting...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]He[Wait=500][Beep=True]'s pLaY[Wait=500][Beep=True]iNg wIt[Wait=500][Beep=True]h yOu.[Wait=500][Beep=True]  WHy[Wait=500][Beep=True]  bRiNg[Wait=500][Beep=True]  [Color=Gray]*Static*[Color=White]...[Wait=500][Beep=True]  uP?[Color=White][Wait=500][Space=2]
 ]
 [Choices=
@@ -18342,18 +18340,18 @@
       <c r="C61" s="7"/>
       <c r="D61" s="7"/>
       <c r="E61" s="8" t="s">
-        <v>648</v>
+        <v>835</v>
       </c>
       <c r="F61" s="8" t="s">
-        <v>777</v>
+        <v>704</v>
       </c>
       <c r="G61" s="23" t="str">
         <f t="shared" si="1"/>
         <v>[Scene=60
 [Content=
-...[Wait=500] Hundreds?[Wait=500][Space=2]_
+...[Wait=500] Hundreds?[Wait=500][Space=2]
 Hard to tell, it goes way past what I'm physically able to see or even reach.[Wait=500][Space=2]
-It's an...[Wait=500] ...[Wait=500] overwhelming view...[Wait=500] This looks like a scene from a Science-fiction movie.[Wait=500][Space=2]
+It's an...[Wait=500] ...[Wait=500] overwhelming view...[Wait=500] This looks like a scene from a science-fiction movie.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]DoN[Wait=500][Beep=True]'t lEt[Wait=500][Beep=True]  iT b[Wait=500][Beep=True]rEaK[Wait=500][Beep=True]  yOu.[Color=White][Wait=500][Space=2]
 ]
 [Choices=
@@ -18371,10 +18369,10 @@
       <c r="C62" s="7"/>
       <c r="D62" s="7"/>
       <c r="E62" s="8" t="s">
-        <v>691</v>
+        <v>836</v>
       </c>
       <c r="F62" s="8" t="s">
-        <v>778</v>
+        <v>705</v>
       </c>
       <c r="G62" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18383,7 +18381,7 @@
 What's that about a per...[Wait=500] Oh[Wait=500], they came back.[Wait=500][Space=2]
 [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEs[Wait=500][Beep=True]e aRe[Wait=500][Beep=True]  oLd[Wait=500][Beep=True]  [Color=Gray]*Static*[Color=White]...[Wait=500][Beep=True]  fAmIlIaR[Wait=500][Beep=True]  pLaCe[Wait=500][Beep=True]  fOr[Wait=500][Beep=True]  aLl[Wait=500][Beep=True]  oF uS.[Wait=500][Beep=True]  GrOwN[Wait=500][Beep=True]  aNd[Wait=500][Beep=True]  fEd[Wait=500][Beep=True]  [Color=Gray]*Static*[Color=White]...[Wait=500][Beep=True]  tHoSe.[Color=White][Wait=500][Space=2]
-[Color=Magenta][Beep=True]NeW[Wait=500][Beep=True]  oNeS[Wait=500][Beep=True]  iN[Wait=500][Beep=True]  mUsE[Wait=500][Beep=True]uM.[Color=White][Wait=500][Space=2]
+[Color=Magenta][Beep=True]NeW[Wait=500][Beep=True]  oNeS[Wait=500][Beep=True]  iN[Wait=500][Beep=True]  tHe[Wait=500][Beep=True]  mUsEuM.[Color=White][Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=63][Content=What do you mean "grown"?]]
@@ -18400,10 +18398,10 @@
       <c r="C63" s="7"/>
       <c r="D63" s="7"/>
       <c r="E63" s="8" t="s">
-        <v>692</v>
+        <v>641</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>779</v>
+        <v>837</v>
       </c>
       <c r="G63" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18417,7 +18415,7 @@
 ]
 [Choices=
 [Choice1=[NextScene=63][Content=Must be the hunger. You really need to eat.]]
-[Choice2=[NextScene=64][Content=Is this... Your home?]]
+[Choice2=[NextScene=64][Content=Is this... your home?]]
 ]
 ]</v>
       </c>
@@ -18430,10 +18428,10 @@
       <c r="C64" s="7"/>
       <c r="D64" s="7"/>
       <c r="E64" s="8" t="s">
-        <v>860</v>
+        <v>770</v>
       </c>
       <c r="F64" s="8" t="s">
-        <v>780</v>
+        <v>706</v>
       </c>
       <c r="G64" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18458,10 +18456,10 @@
       <c r="C65" s="7"/>
       <c r="D65" s="7"/>
       <c r="E65" s="8" t="s">
-        <v>870</v>
+        <v>775</v>
       </c>
       <c r="F65" s="8" t="s">
-        <v>781</v>
+        <v>707</v>
       </c>
       <c r="G65" s="23" t="str">
         <f t="shared" si="1"/>
@@ -18486,17 +18484,17 @@
       <c r="C66" s="7"/>
       <c r="D66" s="7"/>
       <c r="E66" s="8" t="s">
-        <v>649</v>
+        <v>838</v>
       </c>
       <c r="F66" s="8" t="s">
-        <v>782</v>
+        <v>708</v>
       </c>
       <c r="G66" s="23" t="str">
         <f t="shared" ref="G66:G74" si="2">"[Scene=" &amp; A66 &amp; IF(OR(B66&lt;&gt;"",C66&lt;&gt;"",D66&lt;&gt;""),CHAR(10),"") &amp; IF(B66&lt;&gt;"","[BeepBack=" &amp; B66 &amp; "]","") &amp; IF(C66&lt;&gt;"","[Connection=" &amp; C66 &amp; "]","") &amp; IF(D66&lt;&gt;"","[Timer=" &amp; D66 &amp; "]","") &amp; IF(E66&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E66 &amp; CHAR(10) &amp; "]","") &amp; IF(F66&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F66 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
         <v>[Scene=65
 [Content=
 I don't know how trustworthy this person is...[Wait=500][Space=2]
-But this place is making me so sick I won't stay for a second more.[Wait=500][Space=2]
+But this place is making me so sick I won't stay for a second longer.[Wait=500][Space=2]
 So I'll just do the next best thing.[Wait=500][Space=2]
 ]
 [Choices=
@@ -18513,10 +18511,10 @@
       <c r="C67" s="7"/>
       <c r="D67" s="7"/>
       <c r="E67" s="8" t="s">
-        <v>650</v>
+        <v>839</v>
       </c>
       <c r="F67" s="8" t="s">
-        <v>783</v>
+        <v>709</v>
       </c>
       <c r="G67" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18526,7 +18524,7 @@
 ...[Wait=500][Space=2]
 What?[Wait=500] You didn't expect me to try something while you're listening to their ramblings?[Wait=500][Space=2]
 If there's food I can eat I need to go down.[Wait=500][Space=2]
-[Color=Magenta][Beep=True]GoO[Wait=500][Beep=True]d cAl[Wait=500][Beep=True]l. ThIs[Wait=500][Beep=True] rOoM[Wait=500][Beep=True] sEeMs[Wait=500][Beep=True] sEpArEd[Wait=500][Beep=True] fRoM[Wait=500][Beep=True] tHe rEsT[Wait=500][Beep=True] oF tHe bUiLdInG.[Color=White][Wait=500][Space=2]
+[Color=Magenta][Beep=True]GoO[Wait=500][Beep=True]d cAl[Wait=500][Beep=True]l. ThIs[Wait=500][Beep=True] rOoM[Wait=500][Beep=True] sEeMs[Wait=500][Beep=True] sEpArAtEd[Wait=500][Beep=True] fRoM[Wait=500][Beep=True] tHe rEsT[Wait=500][Beep=True] oF tHe bUiLdInG.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThE[Wait=500][Beep=True]  vEnT[Wait=500][Beep=True]  sYsTeM[Wait=500][Beep=True]  mIgHt[Wait=500][Beep=True]  bE[Wait=500][Beep=True]  tHe[Wait=500][Beep=True]  oNlY[Wait=500][Beep=True]  wAy[Wait=500][Beep=True]  dOwN.[Color=White][Wait=500][Space=2]
 ]
 [Choices=
@@ -18544,10 +18542,10 @@
       <c r="C68" s="7"/>
       <c r="D68" s="7"/>
       <c r="E68" s="8" t="s">
-        <v>651</v>
+        <v>840</v>
       </c>
       <c r="F68" s="8" t="s">
-        <v>784</v>
+        <v>710</v>
       </c>
       <c r="G68" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18555,7 +18553,7 @@
 [Content=
 Absolutely.[Wait=500][Space=2]
 You know how nothing works like it's supposed to on this island?[Wait=500][Space=2]
-The grid istelf is its own uncomprenhensible enigma.[Wait=500][Space=2]
+The grid itself is its own incomprehensible enigma.[Wait=500][Space=2]
 In fact, it isn't a grid.[Wait=500][Space=2]
 More like a lid with a big bolt.[Wait=500][Space=2]
 ]
@@ -18573,19 +18571,19 @@
       <c r="C69" s="7"/>
       <c r="D69" s="7"/>
       <c r="E69" s="8" t="s">
-        <v>652</v>
+        <v>841</v>
       </c>
       <c r="F69" s="8" t="s">
-        <v>785</v>
+        <v>711</v>
       </c>
       <c r="G69" s="23" t="str">
         <f t="shared" si="2"/>
         <v>[Scene=68
 [Content=
-Clicked-[Wait=500] WAAH-...[Wait=500][Space=2]
+Clicked-...[Wait=500] WAAH-...[Wait=500][Space=2]
 [Color=Gray]*CLANG*[Color=White]...[Wait=500][Space=2]
 ...[Wait=500][Space=2]
-The uncomprehensible enigma came off and almost crushed my foot.[Wait=500][Space=2]
+The incomprehensible enigma came off and almost crushed my foot.[Wait=500][Space=2]
 Let's see what's in there...[Wait=500] It's...[Wait=500] been cleaned recently?[Wait=500][Space=2]
 So much for an abandoned building, the metal's almost glistening.[Wait=500][Space=2]
 ]
@@ -18603,10 +18601,10 @@
       <c r="C70" s="7"/>
       <c r="D70" s="7"/>
       <c r="E70" s="8" t="s">
-        <v>653</v>
+        <v>613</v>
       </c>
       <c r="F70" s="8" t="s">
-        <v>786</v>
+        <v>712</v>
       </c>
       <c r="G70" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18630,10 +18628,10 @@
       <c r="C71" s="7"/>
       <c r="D71" s="7"/>
       <c r="E71" s="8" t="s">
-        <v>654</v>
+        <v>614</v>
       </c>
       <c r="F71" s="8" t="s">
-        <v>787</v>
+        <v>713</v>
       </c>
       <c r="G71" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18658,16 +18656,16 @@
       <c r="C72" s="7"/>
       <c r="D72" s="7"/>
       <c r="E72" s="8" t="s">
-        <v>655</v>
+        <v>842</v>
       </c>
       <c r="F72" s="8" t="s">
-        <v>788</v>
+        <v>714</v>
       </c>
       <c r="G72" s="23" t="str">
         <f t="shared" si="2"/>
         <v>[Scene=71
 [Content=
-Anyways, I'm getting into the...[Wait=500] hnng-[Wait=500] ...vent.[Wait=500][Space=2]
+Anyways, I'm getting into the...[Wait=500] hnng-...[Wait=500] ...vent.[Wait=500][Space=2]
 I've got some crawling to do.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 The odor's already fading, I can feel my chest getting lighter.[Wait=500][Space=2]
@@ -18688,10 +18686,10 @@
       <c r="C73" s="7"/>
       <c r="D73" s="7"/>
       <c r="E73" s="8" t="s">
-        <v>656</v>
+        <v>843</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>789</v>
+        <v>715</v>
       </c>
       <c r="G73" s="23" t="str">
         <f t="shared" si="2"/>
@@ -18700,7 +18698,7 @@
 For what being forced to crawl through a vent by a faceless sadist could have been[Wait=500], kind of.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 I can hear air flowing through another vent nearby.[Wait=500][Space=2]
-So there is functionnal ventilation on this island, huh.[Wait=500][Space=2]
+So there is functional ventilation on this island, huh.[Wait=500][Space=2]
 Might have been more effective if that one wasn't converted into a parkour tunnel for me to enjoy.[Wait=500][Space=2]
 ]
 [Choices=
@@ -18717,20 +18715,20 @@
       <c r="C74" s="12"/>
       <c r="D74" s="12"/>
       <c r="E74" s="13" t="s">
-        <v>657</v>
+        <v>844</v>
       </c>
       <c r="F74" s="13" t="s">
-        <v>790</v>
+        <v>716</v>
       </c>
       <c r="G74" s="24" t="str">
         <f t="shared" si="2"/>
         <v>[Scene=73
 [Content=
 I'm sure you can wait for a bit longer.[Wait=500][Space=2]
-I'm not a...[Wait=500] ...vent crawling[Wait=500] ...expert.[Wait=500][Space=2]
+I'm not a...[Wait=500] ...vent-crawling[Wait=500] ...expert.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 I hear clicking and clanking all around, machinery doing its thing.[Wait=500][Space=2]
-I thought this island was abandoned, but it's becoming more and more evident at least someone lives there.[Wait=500][Space=2]
+I thought this island was abandoned, but it's becoming more and more evident that at least someone lives here.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=74][Content=Your kidnapper, for sure.]]
@@ -18747,10 +18745,10 @@
       <c r="C75" s="7"/>
       <c r="D75" s="7"/>
       <c r="E75" s="8" t="s">
-        <v>658</v>
+        <v>615</v>
       </c>
       <c r="F75" s="8" t="s">
-        <v>791</v>
+        <v>717</v>
       </c>
       <c r="G75" s="23" t="str">
         <f t="shared" ref="G75:G106" si="3">"[Scene=" &amp; A75 &amp; IF(OR(B75&lt;&gt;"",C75&lt;&gt;"",D75&lt;&gt;""),CHAR(10),"") &amp; IF(B75&lt;&gt;"","[BeepBack=" &amp; B75 &amp; "]","") &amp; IF(C75&lt;&gt;"","[Connection=" &amp; C75 &amp; "]","") &amp; IF(D75&lt;&gt;"","[Timer=" &amp; D75 &amp; "]","") &amp; IF(E75&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E75 &amp; CHAR(10) &amp; "]","") &amp; IF(F75&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F75 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -18772,10 +18770,10 @@
       <c r="C76" s="7"/>
       <c r="D76" s="7"/>
       <c r="E76" s="8" t="s">
-        <v>659</v>
+        <v>616</v>
       </c>
       <c r="F76" s="8" t="s">
-        <v>792</v>
+        <v>718</v>
       </c>
       <c r="G76" s="23" t="str">
         <f t="shared" si="3"/>
@@ -18802,10 +18800,10 @@
       <c r="C77" s="7"/>
       <c r="D77" s="7"/>
       <c r="E77" s="8" t="s">
-        <v>660</v>
+        <v>617</v>
       </c>
       <c r="F77" s="8" t="s">
-        <v>793</v>
+        <v>719</v>
       </c>
       <c r="G77" s="23" t="str">
         <f t="shared" si="3"/>
@@ -18830,17 +18828,17 @@
       <c r="C78" s="7"/>
       <c r="D78" s="7"/>
       <c r="E78" s="8" t="s">
-        <v>861</v>
+        <v>845</v>
       </c>
       <c r="F78" s="8" t="s">
-        <v>794</v>
+        <v>720</v>
       </c>
       <c r="G78" s="23" t="str">
         <f t="shared" si="3"/>
         <v>[Scene=77
 [Content=
 I know![Wait=500][Space=2]
-I-...[Wait=500] need to get to the down area.[Wait=500][Space=2]
+I-...[Wait=500] need to get to the lower area.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEy[Wait=500][Beep=True]'vE nEgLe[Wait=500][Beep=True]cTeD tO[Wait=500][Beep=True]  tElL yOu[Wait=500][Beep=True]  tHeY fOu[Wait=500][Beep=True]nD aN[Wait=500][Beep=True]  eXiT, i[Wait=500][Beep=True]  cAn sEe[Wait=500][Beep=True]  iT fRo[Wait=500][Beep=True]m a[Wait=500][Beep=True]  cAmErA.[Color=White][Wait=500][Space=2]
 [Color=Magenta][Beep=True]tHe fAlL[Wait=500][Beep=True] mIgHt[Wait=500][Beep=True]  bE rOuGh[Wait=500][Beep=True],  bUt iT's[Wait=500][Beep=True]  wOrTh[Wait=500][Beep=True]  nOt fIgHtInG[Wait=500][Beep=True]  tHeM.[Color=White][Wait=500][Space=2]
 ]
@@ -18858,22 +18856,22 @@
       <c r="C79" s="7"/>
       <c r="D79" s="7"/>
       <c r="E79" s="8" t="s">
-        <v>661</v>
+        <v>846</v>
       </c>
       <c r="F79" s="8" t="s">
-        <v>795</v>
+        <v>847</v>
       </c>
       <c r="G79" s="23" t="str">
         <f t="shared" si="3"/>
         <v>[Scene=78
 [Content=
-I'm not just going to jump into the void![Wait=500] I don't what caused this noise.[Wait=500][Space=2]
+I'm not just going to jump into the void![Wait=500] I don't know what caused this noise.[Wait=500][Space=2]
 But I can tell it's not inside the vent from the height it had to fall from.[Wait=500][Space=2]
 I should keep going forward and find a way down.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=79][TrustAdd=-25][Content=You're such a hassle.]]
-[Choice1=[NextScene=79][TrustAdd=25][Content=Please, be safe.]]
+[Choice2=[NextScene=79][TrustAdd=25][Content=Please, be safe.]]
 ]
 ]</v>
       </c>
@@ -18886,10 +18884,10 @@
       <c r="C80" s="7"/>
       <c r="D80" s="7"/>
       <c r="E80" s="8" t="s">
-        <v>662</v>
+        <v>618</v>
       </c>
       <c r="F80" s="8" t="s">
-        <v>796</v>
+        <v>848</v>
       </c>
       <c r="G80" s="23" t="str">
         <f t="shared" si="3"/>
@@ -18903,7 +18901,7 @@
 [Choices=
 [Choice1=[NextScene=80][Content=Go left.]]
 [Choice2=[NextScene=80][Content=Go right.]]
-[Choice3=[NextScene=80][Content=Go. Back.]]
+[Choice3=[NextScene=80][Content=Go back.]]
 ]
 ]</v>
       </c>
@@ -18916,10 +18914,10 @@
       <c r="C81" s="7"/>
       <c r="D81" s="7"/>
       <c r="E81" s="8" t="s">
-        <v>664</v>
+        <v>620</v>
       </c>
       <c r="F81" s="8" t="s">
-        <v>797</v>
+        <v>721</v>
       </c>
       <c r="G81" s="23" t="str">
         <f t="shared" si="3"/>
@@ -18950,10 +18948,10 @@
         <v>5</v>
       </c>
       <c r="E82" s="8" t="s">
-        <v>663</v>
+        <v>619</v>
       </c>
       <c r="F82" s="8" t="s">
-        <v>798</v>
+        <v>722</v>
       </c>
       <c r="G82" s="23" t="str">
         <f>"[Scene=" &amp; A82 &amp; IF(OR(B82&lt;&gt;"",C82&lt;&gt;"",D82&lt;&gt;""),CHAR(10),"") &amp; IF(B82&lt;&gt;"","[BeepBack=" &amp; B82 &amp; "]","") &amp; IF(C82&lt;&gt;"","[Connection=" &amp; C82 &amp; "]","") &amp; IF(D82&lt;&gt;"","[Timer=" &amp; D82 &amp; "]","") &amp; IF(E82&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E82 &amp; CHAR(10) &amp; "]","") &amp; IF(F82&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F82 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -18986,10 +18984,10 @@
         <v>5</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>665</v>
+        <v>621</v>
       </c>
       <c r="F83" s="8" t="s">
-        <v>799</v>
+        <v>723</v>
       </c>
       <c r="G83" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19020,10 +19018,10 @@
         <v>5</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>666</v>
+        <v>622</v>
       </c>
       <c r="F84" s="8" t="s">
-        <v>800</v>
+        <v>724</v>
       </c>
       <c r="G84" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19052,10 +19050,10 @@
         <v>5</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>667</v>
+        <v>623</v>
       </c>
       <c r="F85" s="8" t="s">
-        <v>801</v>
+        <v>725</v>
       </c>
       <c r="G85" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19083,10 +19081,10 @@
       </c>
       <c r="D86" s="7"/>
       <c r="E86" s="8" t="s">
-        <v>668</v>
+        <v>624</v>
       </c>
       <c r="F86" s="8" t="s">
-        <v>802</v>
+        <v>726</v>
       </c>
       <c r="G86" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19120,10 +19118,10 @@
       </c>
       <c r="D87" s="7"/>
       <c r="E87" s="8" t="s">
-        <v>669</v>
+        <v>849</v>
       </c>
       <c r="F87" s="8" t="s">
-        <v>803</v>
+        <v>727</v>
       </c>
       <c r="G87" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19133,7 +19131,7 @@
 I SEE THE GRID![Wait=500][Space=2]
 COME OFF, YOU PIECE OF SHIT![Wait=500][Space=2]
 [Color=Gray]*Bolt squeaks*[Color=White]...[Wait=500][Space=2]
-COME O-[Wait=500] AAAAH-...[Wait=500][Space=2]
+COME O-...[Wait=500] AAAAH-...[Wait=500][Space=2]
 [Color=Gray]*Splashes*[Color=White]...[Wait=500][Space=2]
 ]
 [Choices=
@@ -19150,17 +19148,17 @@
       <c r="C88" s="7"/>
       <c r="D88" s="7"/>
       <c r="E88" s="8" t="s">
-        <v>862</v>
+        <v>850</v>
       </c>
       <c r="F88" s="8" t="s">
-        <v>804</v>
+        <v>728</v>
       </c>
       <c r="G88" s="23" t="str">
         <f t="shared" si="3"/>
         <v>[Scene=87
 [Content=
 IT'S COMING![Wait=500][Space=2]
-[Color=Gray]*Heavy metalic sounds*[Color=White]...[Wait=500][Space=2]
+[Color=Gray]*Heavy metallic sounds*[Color=White]...[Wait=500][Space=2]
 .[Wait=500].[Wait=500].[Wait=500][Space=2]
 It-...[Wait=500] It missed the opening I fell down from-...[Wait=500][Space=2]
 I-I think I'm safe.[Wait=500][Space=2]
@@ -19181,10 +19179,10 @@
       <c r="C89" s="7"/>
       <c r="D89" s="7"/>
       <c r="E89" s="8" t="s">
-        <v>670</v>
+        <v>625</v>
       </c>
       <c r="F89" s="8" t="s">
-        <v>805</v>
+        <v>729</v>
       </c>
       <c r="G89" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19208,10 +19206,10 @@
       <c r="C90" s="7"/>
       <c r="D90" s="7"/>
       <c r="E90" s="8" t="s">
-        <v>863</v>
+        <v>771</v>
       </c>
       <c r="F90" s="8" t="s">
-        <v>806</v>
+        <v>730</v>
       </c>
       <c r="G90" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19239,10 +19237,10 @@
       <c r="C91" s="7"/>
       <c r="D91" s="7"/>
       <c r="E91" s="8" t="s">
-        <v>671</v>
+        <v>626</v>
       </c>
       <c r="F91" s="8" t="s">
-        <v>808</v>
+        <v>732</v>
       </c>
       <c r="G91" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19270,10 +19268,10 @@
       <c r="C92" s="7"/>
       <c r="D92" s="7"/>
       <c r="E92" s="8" t="s">
-        <v>672</v>
+        <v>851</v>
       </c>
       <c r="F92" s="8" t="s">
-        <v>807</v>
+        <v>731</v>
       </c>
       <c r="G92" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19285,7 +19283,7 @@
 But I really am glad you are, that's all.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 Besides that, you were right about that place. It's filled to the brim with food cans.[Wait=500][Space=2]
-This is like a storage room for Spam-looking, dank mush.[Wait=500][Space=2]
+This is like a storage room for spam-looking, dank mush.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=93][Content=Finally, you can eat!]]
@@ -19301,10 +19299,10 @@
       <c r="C93" s="7"/>
       <c r="D93" s="7"/>
       <c r="E93" s="8" t="s">
-        <v>673</v>
+        <v>852</v>
       </c>
       <c r="F93" s="8" t="s">
-        <v>809</v>
+        <v>733</v>
       </c>
       <c r="G93" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19316,7 +19314,7 @@
 Positively better than just hitting the concrete, but I'm worried I'll catch a cold.[Wait=500][Space=2]
 Also, thank your friend, there's indeed loads of food there.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
-Never been a fan of damped mush, but gourmet's palate has a time and place.[Wait=500][Space=2]
+Never been a fan of damped mush, but a gourmet's palate has a time and place.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=93][Content=Food is food.]]
@@ -19332,16 +19330,16 @@
       <c r="C94" s="7"/>
       <c r="D94" s="7"/>
       <c r="E94" s="8" t="s">
-        <v>674</v>
+        <v>853</v>
       </c>
       <c r="F94" s="8" t="s">
-        <v>810</v>
+        <v>734</v>
       </c>
       <c r="G94" s="23" t="str">
         <f t="shared" si="3"/>
         <v>[Scene=93
 [Content=
-Here goes nothing-[Wait=500] I'm opening one.[Wait=500][Space=2]
+Here goes nothing-...[Wait=500] I'm opening one.[Wait=500][Space=2]
 [Color=Gray]*Clunk*[Color=White]...[Wait=500][Space=2]
 It's-[Wait=500] neutral in odor.[Wait=500] Doesn't look like anything, but not repulsive either.[Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThEs[Wait=500][Beep=True]e aRe[Wait=500][Beep=True]  qUiT[Wait=500][Beep=True]e gOoD[Wait=500][Beep=True],  aCtUaLlY.[Wait=500][Beep=True]  NOt[Wait=500][Beep=True]  tHaT tHeRe[Wait=500][Beep=True]  iS aNy[Wait=500][Beep=True]tHiNg eLsE[Wait=500][Beep=True]  tO eAt[Wait=500][Beep=True]  tHeRe.[Color=White][Wait=500][Space=2]
@@ -19362,10 +19360,10 @@
       <c r="C95" s="7"/>
       <c r="D95" s="7"/>
       <c r="E95" s="8" t="s">
-        <v>675</v>
+        <v>627</v>
       </c>
       <c r="F95" s="8" t="s">
-        <v>811</v>
+        <v>735</v>
       </c>
       <c r="G95" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19393,10 +19391,10 @@
       <c r="C96" s="7"/>
       <c r="D96" s="7"/>
       <c r="E96" s="8" t="s">
-        <v>676</v>
+        <v>628</v>
       </c>
       <c r="F96" s="8" t="s">
-        <v>812</v>
+        <v>736</v>
       </c>
       <c r="G96" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19423,10 +19421,10 @@
       <c r="C97" s="7"/>
       <c r="D97" s="7"/>
       <c r="E97" s="8" t="s">
-        <v>677</v>
+        <v>629</v>
       </c>
       <c r="F97" s="8" t="s">
-        <v>813</v>
+        <v>737</v>
       </c>
       <c r="G97" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19451,10 +19449,10 @@
       <c r="C98" s="7"/>
       <c r="D98" s="7"/>
       <c r="E98" s="8" t="s">
-        <v>678</v>
+        <v>630</v>
       </c>
       <c r="F98" s="8" t="s">
-        <v>814</v>
+        <v>738</v>
       </c>
       <c r="G98" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19478,10 +19476,10 @@
       <c r="C99" s="7"/>
       <c r="D99" s="7"/>
       <c r="E99" s="8" t="s">
-        <v>679</v>
+        <v>631</v>
       </c>
       <c r="F99" s="8" t="s">
-        <v>815</v>
+        <v>739</v>
       </c>
       <c r="G99" s="23" t="str">
         <f>"[Scene=" &amp; A99 &amp; IF(OR(B99&lt;&gt;"",C99&lt;&gt;"",D99&lt;&gt;""),CHAR(10),"") &amp; IF(B99&lt;&gt;"","[BeepBack=" &amp; B99 &amp; "]","") &amp; IF(C99&lt;&gt;"","[Connection=" &amp; C99 &amp; "]","") &amp; IF(D99&lt;&gt;"","[Timer=" &amp; D99 &amp; "]","") &amp; IF(E99&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E99 &amp; CHAR(10) &amp; "]","") &amp; IF(F99&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F99 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -19508,10 +19506,10 @@
       <c r="C100" s="7"/>
       <c r="D100" s="7"/>
       <c r="E100" s="8" t="s">
-        <v>680</v>
+        <v>854</v>
       </c>
       <c r="F100" s="8" t="s">
-        <v>816</v>
+        <v>740</v>
       </c>
       <c r="G100" s="23" t="str">
         <f>"[Scene=" &amp; A100 &amp; IF(OR(B100&lt;&gt;"",C100&lt;&gt;"",D100&lt;&gt;""),CHAR(10),"") &amp; IF(B100&lt;&gt;"","[BeepBack=" &amp; B100 &amp; "]","") &amp; IF(C100&lt;&gt;"","[Connection=" &amp; C100 &amp; "]","") &amp; IF(D100&lt;&gt;"","[Timer=" &amp; D100 &amp; "]","") &amp; IF(E100&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E100 &amp; CHAR(10) &amp; "]","") &amp; IF(F100&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F100 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -19519,7 +19517,7 @@
 [Content=
 Is the fuse there?[Wait=500][Space=2]
 What are you on about?[Wait=500][Space=2]
-I got all the way from the trapdoor just to find that fuse.[Wait=500][Space=2]
+I got all the way here just to find that fuse.[Wait=500][Space=2]
 Why would you say that now that I'm about to find it?[Wait=500][Space=2]
 I'm gonna need some better explanations![Wait=500][Space=2]
 [Color=Magenta][Beep=True]I wAn[Wait=500][Beep=True]t tO tElL[Wait=500][Beep=True] tHeM tHe[Wait=500][Beep=True] tRuTh.[Color=White][Wait=500][Space=2]
@@ -19540,10 +19538,10 @@
       <c r="C101" s="7"/>
       <c r="D101" s="7"/>
       <c r="E101" s="8" t="s">
-        <v>681</v>
+        <v>632</v>
       </c>
       <c r="F101" s="8" t="s">
-        <v>817</v>
+        <v>741</v>
       </c>
       <c r="G101" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19571,10 +19569,10 @@
       <c r="C102" s="7"/>
       <c r="D102" s="7"/>
       <c r="E102" s="8" t="s">
-        <v>693</v>
+        <v>642</v>
       </c>
       <c r="F102" s="8" t="s">
-        <v>818</v>
+        <v>742</v>
       </c>
       <c r="G102" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19603,10 +19601,10 @@
       <c r="C103" s="7"/>
       <c r="D103" s="7"/>
       <c r="E103" s="8" t="s">
-        <v>694</v>
+        <v>643</v>
       </c>
       <c r="F103" s="8" t="s">
-        <v>819</v>
+        <v>743</v>
       </c>
       <c r="G103" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19628,10 +19626,10 @@
       <c r="C104" s="7"/>
       <c r="D104" s="7"/>
       <c r="E104" s="8" t="s">
-        <v>698</v>
+        <v>646</v>
       </c>
       <c r="F104" s="8" t="s">
-        <v>871</v>
+        <v>776</v>
       </c>
       <c r="G104" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19656,18 +19654,18 @@
       <c r="C105" s="7"/>
       <c r="D105" s="7"/>
       <c r="E105" s="8" t="s">
-        <v>699</v>
+        <v>855</v>
       </c>
       <c r="F105" s="8" t="s">
-        <v>820</v>
+        <v>744</v>
       </c>
       <c r="G105" s="23" t="str">
         <f t="shared" si="3"/>
         <v>[Scene=104
 [Content=
-They seem to have.[Wait=500][Space=2]
+They seem to have a plan.[Wait=500][Space=2]
 If the fuse isn't gonna get me out of there, I might as well trust them.[Wait=500][Space=2]
-What should I do no ?[Wait=500][Space=2]
+What should I do now?[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=105][Content=The wall has a hole in it, beneath the water. Swim until you reach the other side.]]
@@ -19683,10 +19681,10 @@
       <c r="C106" s="7"/>
       <c r="D106" s="7"/>
       <c r="E106" s="8" t="s">
-        <v>700</v>
+        <v>647</v>
       </c>
       <c r="F106" s="8" t="s">
-        <v>821</v>
+        <v>856</v>
       </c>
       <c r="G106" s="23" t="str">
         <f t="shared" si="3"/>
@@ -19698,7 +19696,7 @@
 [Color=Magenta][Beep=True]ThEy[Wait=500][Beep=True]  nEeD[Wait=500][Beep=True]  tO sWiM[Wait=500][Beep=True]  fOrWaRd[Wait=500][Beep=True]  uNtIl[Wait=500][Beep=True]  tHeY[Wait=500][Beep=True]  fInD[Wait=500][Beep=True]  a bIg[Wait=500][Beep=True]  mEtAl[Wait=500][Beep=True]  pIpE[Wait=500][Beep=True],  tHeN[Wait=500][Beep=True]  rEaCh[Wait=500][Beep=True]  uPwArDs[Wait=500][Beep=True]  tO fInD[Wait=500][Beep=True]  tHe[Wait=500][Beep=True]  oPeNiNg.[Color=White][Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=106][Content=Once in the cave, swim forward, until you feel a pipe.]]
+[Choice1=[NextScene=106][Content=Once in the cave, swim forward until you feel a pipe.]]
 ]
 ]</v>
       </c>
@@ -19711,10 +19709,10 @@
       <c r="C107" s="7"/>
       <c r="D107" s="7"/>
       <c r="E107" s="8" t="s">
-        <v>695</v>
+        <v>644</v>
       </c>
       <c r="F107" s="8" t="s">
-        <v>822</v>
+        <v>745</v>
       </c>
       <c r="G107" s="23" t="str">
         <f t="shared" ref="G107:G138" si="4">"[Scene=" &amp; A107 &amp; IF(OR(B107&lt;&gt;"",C107&lt;&gt;"",D107&lt;&gt;""),CHAR(10),"") &amp; IF(B107&lt;&gt;"","[BeepBack=" &amp; B107 &amp; "]","") &amp; IF(C107&lt;&gt;"","[Connection=" &amp; C107 &amp; "]","") &amp; IF(D107&lt;&gt;"","[Timer=" &amp; D107 &amp; "]","") &amp; IF(E107&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E107 &amp; CHAR(10) &amp; "]","") &amp; IF(F107&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F107 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -19736,10 +19734,10 @@
       <c r="C108" s="7"/>
       <c r="D108" s="7"/>
       <c r="E108" s="8" t="s">
-        <v>701</v>
+        <v>648</v>
       </c>
       <c r="F108" s="8" t="s">
-        <v>823</v>
+        <v>746</v>
       </c>
       <c r="G108" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19761,10 +19759,10 @@
       <c r="C109" s="7"/>
       <c r="D109" s="7"/>
       <c r="E109" s="8" t="s">
-        <v>702</v>
+        <v>649</v>
       </c>
       <c r="F109" s="8" t="s">
-        <v>824</v>
+        <v>857</v>
       </c>
       <c r="G109" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19776,7 +19774,7 @@
 [Color=Magenta][Beep=True]TeLl[Wait=500][Beep=True]  tHeM[Wait=500][Beep=True]  tO hUr[Wait=500][Beep=True]ry uP[Wait=500][Beep=True],  bEiNg rIp[Wait=500][Beep=True]pEd iN[Wait=500][Beep=True]  hAlF wHeN[Wait=500][Beep=True]  rOoMs mOvE[Wait=500][Beep=True]  aGaIn iSn'[Wait=500][Beep=True]t gLa[Wait=500][Beep=True]mOuR eItHeR.[Color=White][Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=109][Content=I believe in you, go quick, before the rooms move again.]]
+[Choice1=[NextScene=109][Content=I believe in you. Go quick, before the rooms move again.]]
 ]
 ]</v>
       </c>
@@ -19789,10 +19787,10 @@
       <c r="C110" s="7"/>
       <c r="D110" s="7"/>
       <c r="E110" s="8" t="s">
-        <v>864</v>
+        <v>772</v>
       </c>
       <c r="F110" s="8" t="s">
-        <v>825</v>
+        <v>858</v>
       </c>
       <c r="G110" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19803,7 +19801,7 @@
 [Color=Gray]*Splash*[Color=White]...[Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=110][Content=Wait is this phone even water proof?]]
+[Choice1=[NextScene=110][Content=Wait, is this phone even waterproof?]]
 ]
 ]</v>
       </c>
@@ -19816,10 +19814,10 @@
       <c r="C111" s="7"/>
       <c r="D111" s="7"/>
       <c r="E111" s="8" t="s">
-        <v>696</v>
+        <v>645</v>
       </c>
       <c r="F111" s="8" t="s">
-        <v>826</v>
+        <v>747</v>
       </c>
       <c r="G111" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19846,16 +19844,16 @@
       <c r="C112" s="7"/>
       <c r="D112" s="7"/>
       <c r="E112" s="8" t="s">
-        <v>866</v>
+        <v>859</v>
       </c>
       <c r="F112" s="8" t="s">
-        <v>827</v>
+        <v>748</v>
       </c>
       <c r="G112" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=111
 [Content=
-You-[Wait=500] Your face![Wait=500][Space=2]
+Your-...[Wait=500] Your face![Wait=500][Space=2]
 [Color=Magenta]I should've warned you before.[Wait=500] It's hard to explain that so...[Wait=500] directly.[Wait=500] Most of us figure it out much earlier.[Color=White][Wait=500][Space=2]
 Am I...[Wait=500] Dumber than the-...[Wait=500] ...others?[Wait=500][Space=2]
 [Color=Magenta]No, you're healthier.[Wait=500] That "thing" was...[Wait=500] One of us.[Wait=500] Like all of us.[Color=White][Wait=500][Space=2]
@@ -19878,10 +19876,10 @@
       <c r="C113" s="7"/>
       <c r="D113" s="7"/>
       <c r="E113" s="8" t="s">
-        <v>865</v>
+        <v>773</v>
       </c>
       <c r="F113" s="8" t="s">
-        <v>872</v>
+        <v>777</v>
       </c>
       <c r="G113" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19904,10 +19902,10 @@
       <c r="C114" s="7"/>
       <c r="D114" s="7"/>
       <c r="E114" s="8" t="s">
-        <v>697</v>
+        <v>860</v>
       </c>
       <c r="F114" s="8" t="s">
-        <v>873</v>
+        <v>778</v>
       </c>
       <c r="G114" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19917,7 +19915,7 @@
 Who am I?[Wait=500] What do you mean, grown?[Wait=500][Space=2]
 [Color=Magenta]You are the successful prototype.[Wait=500] The one he's been waiting for.[Color=White][Wait=500][Space=2]
 [Color=Magenta]The scientist, as I call him.[Wait=500] He's the one behind our suffering.[Color=White][Wait=500][Space=2]
-So, are we...[Wait=500] clones of you?[Wait=500][Space=2]
+So...[Wait=500] are we clones of you?[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=114][Content=I didn't know anything about that!]]
@@ -19934,10 +19932,10 @@
       <c r="C115" s="7"/>
       <c r="D115" s="7"/>
       <c r="E115" s="8" t="s">
-        <v>874</v>
+        <v>779</v>
       </c>
       <c r="F115" s="8" t="s">
-        <v>828</v>
+        <v>861</v>
       </c>
       <c r="G115" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19951,7 +19949,7 @@
 I don't want other people to go through what we've been, no matter if they're clones or not.[Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=115][Content=That's insanity! How are you going to stop this scientist?]]
+[Choice1=[NextScene=115][Content=That's insanity! How are you going to stop him?]]
 ]
 ]</v>
       </c>
@@ -19964,10 +19962,10 @@
       <c r="C116" s="7"/>
       <c r="D116" s="7"/>
       <c r="E116" s="8" t="s">
-        <v>703</v>
+        <v>650</v>
       </c>
       <c r="F116" s="8" t="s">
-        <v>829</v>
+        <v>749</v>
       </c>
       <c r="G116" s="23" t="str">
         <f t="shared" si="4"/>
@@ -19991,16 +19989,16 @@
       <c r="C117" s="7"/>
       <c r="D117" s="7"/>
       <c r="E117" s="8" t="s">
-        <v>704</v>
+        <v>862</v>
       </c>
       <c r="F117" s="8" t="s">
-        <v>830</v>
+        <v>750</v>
       </c>
       <c r="G117" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=116
 [Content=
-[Color=Magenta]This phone.[Wait=500] He can use it as a tracker.[Wait=500] You have to throw it away.[Color=White][Wait=500][Space=2]
+[Color=Magenta]This phone.[Wait=500] He can track it.[Wait=500] You must throw it away.[Color=White][Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=117][Content=Wait! How will I know you'll be safe?]]
@@ -20018,10 +20016,10 @@
       </c>
       <c r="D118" s="7"/>
       <c r="E118" s="8" t="s">
-        <v>705</v>
+        <v>651</v>
       </c>
       <c r="F118" s="8" t="s">
-        <v>831</v>
+        <v>751</v>
       </c>
       <c r="G118" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20052,10 +20050,10 @@
       </c>
       <c r="D119" s="7"/>
       <c r="E119" s="8" t="s">
-        <v>706</v>
+        <v>652</v>
       </c>
       <c r="F119" s="8" t="s">
-        <v>875</v>
+        <v>780</v>
       </c>
       <c r="G119" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20087,10 +20085,10 @@
       </c>
       <c r="D120" s="7"/>
       <c r="E120" s="8" t="s">
-        <v>725</v>
+        <v>662</v>
       </c>
       <c r="F120" s="8" t="s">
-        <v>802</v>
+        <v>726</v>
       </c>
       <c r="G120" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20119,23 +20117,23 @@
       <c r="C121" s="7"/>
       <c r="D121" s="7"/>
       <c r="E121" s="8" t="s">
-        <v>707</v>
+        <v>863</v>
       </c>
       <c r="F121" s="8" t="s">
-        <v>832</v>
+        <v>864</v>
       </c>
       <c r="G121" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=120
 [Content=
-I'm just not gonna go anywhere else in this godamn factory![Wait=500][Space=2]
+I'm just not going anywhere else in this goddamn factory![Wait=500][Space=2]
 The exit's just there![Wait=500][Space=2]
-I don't care about anything else![Wait=500] Fuck whoever is trying to persuade you to lead me in a trap![Wait=500][Space=2]
+I don't care about anything else![Wait=500] Fuck whoever is trying to persuade you to lead me into a trap![Wait=500][Space=2]
 I.[Wait=500] Just.[Wait=500] Want.[Wait=500] To.[Wait=500] Leave.[Wait=500][Space=2]
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=121][Content=Do not tell I haven't warned you.]]
+[Choice1=[NextScene=121][Content=Do not say I didn't warn you.]]
 ]
 ]</v>
       </c>
@@ -20148,10 +20146,10 @@
       <c r="C122" s="7"/>
       <c r="D122" s="7"/>
       <c r="E122" s="8" t="s">
-        <v>708</v>
+        <v>865</v>
       </c>
       <c r="F122" s="8" t="s">
-        <v>833</v>
+        <v>752</v>
       </c>
       <c r="G122" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20159,7 +20157,7 @@
 [Content=
 [Color=Gray]*Footsteps*[Color=White]...[Wait=500][Space=2]
 The light is almost blinding in there. I can't see shit.[Wait=500][Space=2]
-Though it's good to think I could get out in case things go sour.[Wait=500][Space=2]
+Still, it's good to know I could get out in case things go sour.[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]ThIs[Wait=500][Beep=True] iS[Wait=500][Beep=True] bAd.[Wait=500][Beep=True]  CaN'[Wait=500][Beep=True]t tHeY[Wait=500][Beep=True] sEe tHe[Wait=500][Beep=True] pErSoN[Wait=500][Beep=True] aBoVe?[Color=White][Wait=500][Space=2]
 ]
@@ -20177,10 +20175,10 @@
       <c r="C123" s="7"/>
       <c r="D123" s="7"/>
       <c r="E123" s="8" t="s">
-        <v>876</v>
+        <v>866</v>
       </c>
       <c r="F123" s="8" t="s">
-        <v>834</v>
+        <v>753</v>
       </c>
       <c r="G123" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20189,7 +20187,7 @@
 Wah-...[Wait=500] OH SH...[Wait=500][Space=2]
 [Color=Gray]*Whisper*[Color=White]... T-There's...[Wait=500] It's the thing that chased me in the vent...[Wait=500][Space=2]
 It's o-on the catwalks...[Wait=500][Space=2]
-...[Wait=500] Wait is that the...[Wait=500][Space=2]
+...[Wait=500] Wait, is that the...[Wait=500][Space=2]
 [Color=Magenta][Beep=True]DoN[Wait=500][Beep=True]'t dO[Wait=500][Beep=True] aNyThInG[Wait=500][Beep=True] sTuPiD[Wait=500][Beep=True],  i'M[Wait=500][Beep=True] gOnNa[Wait=500][Beep=True] dIsTrAcT[Wait=500][Beep=True] tHeM.[Color=White][Wait=500][Space=2]
 ]
 [Choices=
@@ -20206,10 +20204,10 @@
       <c r="C124" s="7"/>
       <c r="D124" s="7"/>
       <c r="E124" s="8" t="s">
-        <v>709</v>
+        <v>867</v>
       </c>
       <c r="F124" s="8" t="s">
-        <v>835</v>
+        <v>754</v>
       </c>
       <c r="G124" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20217,9 +20215,9 @@
 [Content=
 Wait...[Wait=500] I think I can do it on my own...[Wait=500][Space=2]
 ...I just have to be...[Wait=500][Space=2]
-[Color=Gray]*DISTORDED SCREAMING*[Color=White]... SHIT IT SAW ME![Wait=500][Space=2]
+[Color=Gray]*DISTORTED SCREAMING*[Color=White]... SHIT, IT SAW ME![Wait=500][Space=2]
 [Color=Gray]*Fast footsteps*[Color=White]...[Wait=500][Space=2]
-FUCK FUCK FUCK![Wait=500] ITS FACE, ITS DISFORMED, IT'S A FUCKING MONSTER![Wait=500][Space=2]
+FUCK! FUCK! FUCK![Wait=500] ITS FACE, IT'S DISFORMED, IT'S A FUCKING MONSTER![Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=124][Content=DON'T THINK, RUN!]]
@@ -20235,10 +20233,10 @@
       <c r="C125" s="7"/>
       <c r="D125" s="7"/>
       <c r="E125" s="8" t="s">
-        <v>710</v>
+        <v>653</v>
       </c>
       <c r="F125" s="8" t="s">
-        <v>836</v>
+        <v>868</v>
       </c>
       <c r="G125" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20248,7 +20246,7 @@
 I CAN'T LEAVE IT THERE![Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=125][Content=DON'T GRAB THE FUSE DUMBASS, RUN!]]
+[Choice1=[NextScene=125][Content=DON'T GRAB THE FUSE, DUMBASS! RUN!]]
 [Choice2=[NextScene=125][Content=GRAB IT FAST!]]
 ]
 ]</v>
@@ -20262,10 +20260,10 @@
       <c r="C126" s="7"/>
       <c r="D126" s="7"/>
       <c r="E126" s="8" t="s">
-        <v>711</v>
+        <v>869</v>
       </c>
       <c r="F126" s="8" t="s">
-        <v>837</v>
+        <v>755</v>
       </c>
       <c r="G126" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20273,9 +20271,9 @@
 [Content=
 I'M SURE I CAN DO IT![Wait=500][Space=2]
 I JUST HAVE TO [Color=Gray]*SCREEESH*[Color=White]... RAAAAGH![Wait=500][Space=2]
-I-I'm bleeding...[Wait=500] It scratch my whole arm![Wait=500][Space=2]
-Please...[Wait=500] Dont hurt me...[Wait=500][Space=2]
-[Color=Gray]*DISTORDED SCREAMING*[Color=White]...[Wait=500][Space=2]
+I-I'm bleeding...[Wait=500] It scratched my whole arm![Wait=500][Space=2]
+Please...[Wait=500] Don't hurt me...[Wait=500][Space=2]
+[Color=Gray]*DISTORTED SCREAMING*[Color=White]...[Wait=500][Space=2]
 AAAAAAAAAAAAAAAAA-[Color=Gray]*Fleshy noises*[Color=White]...[Wait=500][Space=2]
 ]
 [Choices=
@@ -20292,10 +20290,10 @@
       <c r="C127" s="7"/>
       <c r="D127" s="7"/>
       <c r="E127" s="8" t="s">
-        <v>712</v>
+        <v>654</v>
       </c>
       <c r="F127" s="8" t="s">
-        <v>802</v>
+        <v>726</v>
       </c>
       <c r="G127" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20323,22 +20321,19 @@
       </c>
       <c r="B128" s="6"/>
       <c r="C128" s="7"/>
-      <c r="D128" s="7">
-        <v>0</v>
-      </c>
+      <c r="D128" s="7"/>
       <c r="E128" s="8" t="s">
-        <v>713</v>
+        <v>870</v>
       </c>
       <c r="F128" s="8" t="s">
-        <v>802</v>
+        <v>726</v>
       </c>
       <c r="G128" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=127
-[Timer=0]
 [Content=
 You...[Wait=500] MONSTER![Wait=500][Space=2]
-Why am I keeping this phone you've obviously left there to torture me?[Wait=500][Space=2]
+Why am I keeping this phone you've obviously left here to torture me?[Wait=500][Space=2]
 I WON'T KEEP PLAYING YOUR GAMES![Wait=500][Space=2]
 [Color=Gray]*B[Beep=True]eep*[Color=White]...[Wait=500][Space=2]
 .[Wait=500].[Wait=500].[Wait=500][Space=2]
@@ -20363,23 +20358,23 @@
       <c r="C129" s="7"/>
       <c r="D129" s="7"/>
       <c r="E129" s="8" t="s">
-        <v>714</v>
+        <v>871</v>
       </c>
       <c r="F129" s="8" t="s">
-        <v>838</v>
+        <v>872</v>
       </c>
       <c r="G129" s="23" t="str">
         <f t="shared" si="4"/>
         <v>[Scene=128
 [Content=
 Just have to...[Wait=500][Space=2]
-[Color=Gray]*Grunt*[Color=White]...[Wait=500][Space=2]_
+[Color=Gray]*Grunt*[Color=White]...[Wait=500][Space=2]
 [Color=Gray]*Running footsteps*[Color=White]...[Wait=500][Space=2]
 ...[Wait=500][Space=2]
 OUCH![Wait=500][Space=2]
 ]
 [Choices=
-[Choice1=[NextScene=129][TrustAdd=-25][Content=Well fuck, it was electrified.]]
+[Choice1=[NextScene=129][TrustAdd=-25][Content=Well, fuck, it was electrified.]]
 [Choice2=[NextScene=130][Content=Oh shit! Are you alright?]]
 ]
 ]</v>
@@ -20395,10 +20390,10 @@
       </c>
       <c r="D130" s="7"/>
       <c r="E130" s="8" t="s">
-        <v>715</v>
+        <v>873</v>
       </c>
       <c r="F130" s="8" t="s">
-        <v>839</v>
+        <v>756</v>
       </c>
       <c r="G130" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20406,7 +20401,7 @@
 [Connection=2]
 [Content=
 YOU KNEW?[Wait=500][Space=2]
-Of course it's electrified, why'd you do that?![Wait=500][Space=2]
+Of course it's electrified! Why'd you do that?![Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=127][Content=Funny.]]
@@ -20425,10 +20420,10 @@
       </c>
       <c r="D131" s="7"/>
       <c r="E131" s="8" t="s">
-        <v>716</v>
+        <v>874</v>
       </c>
       <c r="F131" s="8" t="s">
-        <v>840</v>
+        <v>757</v>
       </c>
       <c r="G131" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20436,8 +20431,8 @@
 [Connection=3]
 [Content=
 I still feel my muscles vibrating.[Wait=500][Space=2]
-That is no ordinary electric fence, I really feel like it's been setup to trap me.[Wait=500][Space=2]
-Let's just...[Wait=500] Move on.[Wait=500][Space=2]
+That is no ordinary electric fence. I really feel like it was set up to trap me.[Wait=500][Space=2]
+Let's just...[Wait=500] move on.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=16][Content=Yeah, let's find a backdoor.]]
@@ -20453,10 +20448,10 @@
       <c r="C132" s="7"/>
       <c r="D132" s="7"/>
       <c r="E132" s="8" t="s">
-        <v>717</v>
+        <v>655</v>
       </c>
       <c r="F132" s="8" t="s">
-        <v>841</v>
+        <v>758</v>
       </c>
       <c r="G132" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20482,10 +20477,10 @@
       <c r="C133" s="7"/>
       <c r="D133" s="7"/>
       <c r="E133" s="8" t="s">
-        <v>718</v>
+        <v>656</v>
       </c>
       <c r="F133" s="8" t="s">
-        <v>842</v>
+        <v>759</v>
       </c>
       <c r="G133" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20511,10 +20506,10 @@
       <c r="C134" s="7"/>
       <c r="D134" s="7"/>
       <c r="E134" s="8" t="s">
-        <v>867</v>
+        <v>875</v>
       </c>
       <c r="F134" s="8" t="s">
-        <v>843</v>
+        <v>760</v>
       </c>
       <c r="G134" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20524,8 +20519,8 @@
 [Color=Gray]*Running sounds*[Color=White]...[Wait=500][Space=2]
 I GOT IT![Wait=500][Space=2]
 [Color=Gray]*Static*[Color=White]...[Wait=500][Space=2]
-I'm outside, I can see the stairs I took to get in![Wait=500][Space=2]
-If I knew I could've just kept going and climbed through this window![Wait=500][Space=2]
+I'm outside. I can see the stairs I took to get in![Wait=500][Space=2]
+If I knew, I could've just kept going and climbed through this window![Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=134][Content=Quit yapping and go back to the trapdoor, quick!]]
@@ -20541,10 +20536,10 @@
       <c r="C135" s="7"/>
       <c r="D135" s="7"/>
       <c r="E135" s="8" t="s">
-        <v>719</v>
+        <v>657</v>
       </c>
       <c r="F135" s="8" t="s">
-        <v>844</v>
+        <v>761</v>
       </c>
       <c r="G135" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20568,10 +20563,10 @@
       <c r="C136" s="7"/>
       <c r="D136" s="7"/>
       <c r="E136" s="8" t="s">
-        <v>868</v>
+        <v>774</v>
       </c>
       <c r="F136" s="8" t="s">
-        <v>845</v>
+        <v>762</v>
       </c>
       <c r="G136" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20596,10 +20591,10 @@
       <c r="C137" s="7"/>
       <c r="D137" s="7"/>
       <c r="E137" s="8" t="s">
-        <v>720</v>
+        <v>658</v>
       </c>
       <c r="F137" s="8" t="s">
-        <v>846</v>
+        <v>763</v>
       </c>
       <c r="G137" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20624,10 +20619,10 @@
       <c r="C138" s="7"/>
       <c r="D138" s="7"/>
       <c r="E138" s="8" t="s">
-        <v>721</v>
+        <v>659</v>
       </c>
       <c r="F138" s="8" t="s">
-        <v>847</v>
+        <v>764</v>
       </c>
       <c r="G138" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20652,10 +20647,10 @@
       </c>
       <c r="D139" s="7"/>
       <c r="E139" s="8" t="s">
-        <v>722</v>
+        <v>876</v>
       </c>
       <c r="F139" s="8" t="s">
-        <v>848</v>
+        <v>765</v>
       </c>
       <c r="G139" s="23" t="str">
         <f t="shared" ref="G139:G141" si="5">"[Scene=" &amp; A139 &amp; IF(OR(B139&lt;&gt;"",C139&lt;&gt;"",D139&lt;&gt;""),CHAR(10),"") &amp; IF(B139&lt;&gt;"","[BeepBack=" &amp; B139 &amp; "]","") &amp; IF(C139&lt;&gt;"","[Connection=" &amp; C139 &amp; "]","") &amp; IF(D139&lt;&gt;"","[Timer=" &amp; D139 &amp; "]","") &amp; IF(E139&lt;&gt;"",CHAR(10) &amp; "[Content=" &amp; CHAR(10) &amp; E139 &amp; CHAR(10) &amp; "]","") &amp; IF(F139&lt;&gt;"",CHAR(10) &amp; "[Choices=" &amp; CHAR(10) &amp; F139 &amp; CHAR(10) &amp; "]","") &amp; CHAR(10) &amp; "]"</f>
@@ -20664,7 +20659,7 @@
 [Content=
 YES, IT'S OPENING![Wait=500][Space=2]
 There are stairs here.[Wait=500] I'm getting down there.[Wait=500][Space=2]
-...Oh my god...[Wait=500] It was such an intens-[Color=Gray]*SHKRRRRRRRRR*[Color=White]...[Wait=500] I'm so happy that you were here to help me.[Wait=500][Space=2]
+...Oh my god...[Wait=500] It was such an intense-[Color=Gray]*SHKRRRRRRRRR*[Color=White]...[Wait=500] I'm so happy you were here to help me.[Wait=500][Space=2]
 ]
 [Choices=
 [Choice1=[NextScene=139][Content=Wait, the signal's getting weaker!]]
@@ -20682,10 +20677,10 @@
       </c>
       <c r="D140" s="7"/>
       <c r="E140" s="8" t="s">
-        <v>723</v>
+        <v>660</v>
       </c>
       <c r="F140" s="8" t="s">
-        <v>849</v>
+        <v>766</v>
       </c>
       <c r="G140" s="23" t="str">
         <f t="shared" si="5"/>
@@ -20713,10 +20708,10 @@
       </c>
       <c r="D141" s="7"/>
       <c r="E141" s="8" t="s">
-        <v>724</v>
+        <v>661</v>
       </c>
       <c r="F141" s="8" t="s">
-        <v>802</v>
+        <v>726</v>
       </c>
       <c r="G141" s="23" t="str">
         <f t="shared" si="5"/>

</xml_diff>